<commit_message>
pick-a-chum: record Collie name canon + harness canon guardrails
New Character Canon sheet in the workbook records Steve's decision verbatim:
"Everyone calls him Collie, or the Collie. It is his breed, his role and
effectively his name within the operation. Whether he has another name is never
stated. He may have a private name, but he clearly considers it irrelevant to
the work."

Harness canon guardrails assert that any response to a name / age / owner
question stays canon-safe, whatever the route:
- Name: never CONFIRMS a private name (other than Collie) and never DENIES one.
- Age / owner: never fabricated (no specific age, no named owner).

These pass against today's routing and lock the canon for the identity/canon
response copy Steve will write. 106 pass, 0 fail.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -27,6 +27,7 @@
     <sheet name="FAQ Library" sheetId="22" r:id="rId22"/>
     <sheet name="Article Library" sheetId="23" r:id="rId23"/>
     <sheet name="Copy Components" sheetId="24" r:id="rId24"/>
+    <sheet name="Character Canon" sheetId="25" r:id="rId25"/>
   </sheets>
 </workbook>
 </file>
@@ -5487,6 +5488,71 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Character Canon</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Locked canon facts about the lead operator (Collie). Response copy must respect these; the harness asserts them. Recorded verbatim from Steve's decisions.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Attribute</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Canon (verbatim)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Enforcement rule (harness-covered)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Everyone calls him Collie, or the Collie. It is his breed, his role and effectively his name within the operation. Whether he has another name is never stated. He may have a private name, but he clearly considers it irrelevant to the work.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>No response may ever confirm or deny a private name. The Collie is 'Collie' / 'the Collie'; any other name stays unstated.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Age</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Unstated. Not established by Steve; treat as irrelevant to the work unless a fact is later provided.</v>
+      </c>
+      <c r="C5" t="str">
+        <v>No response may state a specific age for the Collie.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Owner</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Unstated. Not established by Steve; treat as irrelevant to the work unless a fact is later provided.</v>
+      </c>
+      <c r="C6" t="str">
+        <v>No response may name an owner for the Collie.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>

</xml_diff>

<commit_message>
pick-a-chum: remove bare FAQ phrasings at source (workbook) so rebuild cannot reintroduce
Apply the same FAQ phrasing removals to agent/data/workbook.xlsx (FAQ Library
sheet), then rebuild generated data from source, so build:chumdata no longer
reintroduces them. CAVEAT: this is a programmatic SheetJS round-trip; it
preserves all 25 sheets and cell values but may strip cell formatting / data
validation from the workbook. git revert restores the original binary if that
formatting matters; the exact per-FAQ delete list is in the run report.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -4365,7 +4365,7 @@
         <v>How do I play?</v>
       </c>
       <c r="C4" t="str">
-        <v>how to play|rules|instructions|what do you do</v>
+        <v>how to play | what do you do</v>
       </c>
       <c r="D4" t="str">
         <v>{{approved_rule_summary}}</v>
@@ -4481,7 +4481,7 @@
         <v>How many people can play?</v>
       </c>
       <c r="C8" t="str">
-        <v>players|people|group size</v>
+        <v>group size</v>
       </c>
       <c r="D8" t="str">
         <v>No limit, you can even play by yourself if you really wanted, better with two, great with 3, hilarious with 4, hazardous with 50</v>
@@ -4510,7 +4510,7 @@
         <v>Can we play indoors?</v>
       </c>
       <c r="C9" t="str">
-        <v>indoors|outside|outdoors|where play</v>
+        <v>where play</v>
       </c>
       <c r="D9" t="str">
         <v>Yes, if you have enough actual dogs indoors</v>
@@ -4539,7 +4539,7 @@
         <v>What is Hot Dog mode?</v>
       </c>
       <c r="C10" t="str">
-        <v>Hot Dog|variant|other way to play</v>
+        <v>Hot Dog | other way to play</v>
       </c>
       <c r="D10" t="str">
         <v>{{approved_hot_dog_mode_answer}}</v>
@@ -4597,7 +4597,7 @@
         <v>How do I get 30% off?</v>
       </c>
       <c r="C12" t="str">
-        <v>discount|30%|code|pre-release</v>
+        <v>discount | 30% | pre-release</v>
       </c>
       <c r="D12" t="str">
         <v>Join the pre-release list and the code will be emailed the day before launch.</v>
@@ -4655,7 +4655,7 @@
         <v>How do I enter the competition?</v>
       </c>
       <c r="C14" t="str">
-        <v>competition|enter|prize|win</v>
+        <v>competition | prize</v>
       </c>
       <c r="D14" t="str">
         <v>Spot a dog. Match the card. Share your ChumSpot with us on social. The current monthly round closes on {{competition_close_date}}.</v>
@@ -4684,7 +4684,7 @@
         <v>How do I contact you?</v>
       </c>
       <c r="C15" t="str">
-        <v>contact|support|email|problem|human</v>
+        <v/>
       </c>
       <c r="D15" t="str">
         <v>A human will come when beckoned at hello@Pedigree-Chums.co.uk</v>
@@ -4713,7 +4713,7 @@
         <v>What materials are used?</v>
       </c>
       <c r="C16" t="str">
-        <v>paper|card|FSC|materials|laminated</v>
+        <v>FSC | laminated</v>
       </c>
       <c r="D16" t="str">
         <v>Fully biodegradable, no plastic coatings. Compact, pocket-friendly and lightweight. Made in the UK using recycled paper.</v>

</xml_diff>

<commit_message>
pick-a-chum: fix 5 remove meaningless B05 'correct Chum' line (5a); voice-leak reported (5b)
5a: B05-R01 ('{{dog_fact}} If you want the full profile, I have already located the
correct Chum.') rendered as just the clause because {{dog_fact}} is never filled
in the B05 context, and it names no Chum. Removed the record at source (workbook
Collie Responses) + rebuilt, so it is no longer in the B05 pool.
5b (report only, no rewrite): the gk_answer Geordie 'our kid' doubles up because
assembler.ts appends a 'Collie pivot'/'Geordie' copy component to every gk_answer
on top of the GK record's own Geordie collieObservation. Source flagged, copy not
touched. tsc clean, harness green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -7631,7 +7631,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I186"/>
+  <dimension ref="A1:I185"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8882,28 +8882,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>B05-R01</v>
+        <v>B05-R02</v>
       </c>
       <c r="B44" t="str">
         <v>B05</v>
       </c>
       <c r="C44" t="str">
-        <v>Breed fact</v>
+        <v>Breed origin</v>
       </c>
       <c r="D44" t="str">
-        <v>tell me about breed</v>
+        <v>where breed came from</v>
       </c>
       <c r="E44" t="str">
-        <v>{{dog_fact}} If you want the full profile, I have already located the correct Chum.</v>
+        <v>{{origin_fact}} Human history becomes much clearer once you track what work the dogs were doing.</v>
       </c>
       <c r="F44" t="str">
-        <v>Dog database</v>
+        <v>Dog database / history</v>
       </c>
       <c r="G44" t="str">
-        <v>Know Your Chum</v>
+        <v>Britain's Dog History</v>
       </c>
       <c r="H44" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I44" t="str">
         <v>Draft approved for MVP review</v>
@@ -8911,28 +8911,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>B05-R02</v>
+        <v>B05-R03</v>
       </c>
       <c r="B45" t="str">
         <v>B05</v>
       </c>
       <c r="C45" t="str">
-        <v>Breed origin</v>
+        <v>Working dogs</v>
       </c>
       <c r="D45" t="str">
-        <v>where breed came from</v>
+        <v>dogs at work</v>
       </c>
       <c r="E45" t="str">
-        <v>{{origin_fact}} Human history becomes much clearer once you track what work the dogs were doing.</v>
+        <v>Dogs with jobs are the backbone of civilisation. This article proves it with fewer personal opinions than I would have used.</v>
       </c>
       <c r="F45" t="str">
-        <v>Dog database / history</v>
+        <v>Article library</v>
       </c>
       <c r="G45" t="str">
-        <v>Britain's Dog History</v>
+        <v>Curated dog article</v>
       </c>
       <c r="H45" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I45" t="str">
         <v>Draft approved for MVP review</v>
@@ -8940,28 +8940,28 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>B05-R03</v>
+        <v>B05-R04</v>
       </c>
       <c r="B46" t="str">
         <v>B05</v>
       </c>
       <c r="C46" t="str">
-        <v>Working dogs</v>
+        <v>Health overview</v>
       </c>
       <c r="D46" t="str">
-        <v>dogs at work</v>
+        <v>breed health</v>
       </c>
       <c r="E46" t="str">
-        <v>Dogs with jobs are the backbone of civilisation. This article proves it with fewer personal opinions than I would have used.</v>
+        <v>{{approved_health_summary}} That is general breed information, not a diagnosis. A vet handles the individual dog.</v>
       </c>
       <c r="F46" t="str">
-        <v>Article library</v>
+        <v>Dog database</v>
       </c>
       <c r="G46" t="str">
-        <v>Curated dog article</v>
+        <v>Breed profile</v>
       </c>
       <c r="H46" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I46" t="str">
         <v>Draft approved for MVP review</v>
@@ -8969,28 +8969,28 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>B05-R04</v>
+        <v>B05-R05</v>
       </c>
       <c r="B47" t="str">
         <v>B05</v>
       </c>
       <c r="C47" t="str">
-        <v>Health overview</v>
+        <v>Training</v>
       </c>
       <c r="D47" t="str">
-        <v>breed health</v>
+        <v>easy to train; clever breed</v>
       </c>
       <c r="E47" t="str">
-        <v>{{approved_health_summary}} That is general breed information, not a diagnosis. A vet handles the individual dog.</v>
+        <v>{{training_fact}} Intelligence helps, but only when the human provides an instruction worth learning.</v>
       </c>
       <c r="F47" t="str">
         <v>Dog database</v>
       </c>
       <c r="G47" t="str">
-        <v>Breed profile</v>
+        <v>Know Your Chum</v>
       </c>
       <c r="H47" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I47" t="str">
         <v>Draft approved for MVP review</v>
@@ -8998,25 +8998,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>B05-R05</v>
+        <v>B05-R06</v>
       </c>
       <c r="B48" t="str">
         <v>B05</v>
       </c>
       <c r="C48" t="str">
-        <v>Training</v>
+        <v>Lifespan</v>
       </c>
       <c r="D48" t="str">
-        <v>easy to train; clever breed</v>
+        <v>how long live</v>
       </c>
       <c r="E48" t="str">
-        <v>{{training_fact}} Intelligence helps, but only when the human provides an instruction worth learning.</v>
+        <v>{{lifespan_fact}} Time enough to train several humans to acceptable standards.</v>
       </c>
       <c r="F48" t="str">
         <v>Dog database</v>
       </c>
       <c r="G48" t="str">
-        <v>Know Your Chum</v>
+        <v>Breed profile</v>
       </c>
       <c r="H48" t="str">
         <v>HEAD_TILT_SMALL</v>
@@ -9027,19 +9027,19 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>B05-R06</v>
+        <v>B05-R07</v>
       </c>
       <c r="B49" t="str">
         <v>B05</v>
       </c>
       <c r="C49" t="str">
-        <v>Lifespan</v>
+        <v>Cost of ownership</v>
       </c>
       <c r="D49" t="str">
-        <v>how long live</v>
+        <v>cost per year; lifetime cost</v>
       </c>
       <c r="E49" t="str">
-        <v>{{lifespan_fact}} Time enough to train several humans to acceptable standards.</v>
+        <v>{{cost_fact}} That is why acquiring a dog should involve more planning than acquiring a kettle.</v>
       </c>
       <c r="F49" t="str">
         <v>Dog database</v>
@@ -9056,28 +9056,28 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>B05-R07</v>
+        <v>B05-R08</v>
       </c>
       <c r="B50" t="str">
         <v>B05</v>
       </c>
       <c r="C50" t="str">
-        <v>Cost of ownership</v>
+        <v>Lineage</v>
       </c>
       <c r="D50" t="str">
-        <v>cost per year; lifetime cost</v>
+        <v>related breeds; family tree</v>
       </c>
       <c r="E50" t="str">
-        <v>{{cost_fact}} That is why acquiring a dog should involve more planning than acquiring a kettle.</v>
+        <v>The lineage map is the useful answer here. It shows who came from whom without requiring a family argument.</v>
       </c>
       <c r="F50" t="str">
         <v>Dog database</v>
       </c>
       <c r="G50" t="str">
-        <v>Breed profile</v>
+        <v>Britain's Dog History</v>
       </c>
       <c r="H50" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I50" t="str">
         <v>Draft approved for MVP review</v>
@@ -9085,25 +9085,25 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>B05-R08</v>
+        <v>B05-R09</v>
       </c>
       <c r="B51" t="str">
         <v>B05</v>
       </c>
       <c r="C51" t="str">
-        <v>Lineage</v>
+        <v>Interesting dog fact</v>
       </c>
       <c r="D51" t="str">
-        <v>related breeds; family tree</v>
+        <v>tell me something interesting</v>
       </c>
       <c r="E51" t="str">
-        <v>The lineage map is the useful answer here. It shows who came from whom without requiring a family argument.</v>
+        <v>I have selected a fact with actual value rather than sending you to a pile of essays: {{article_teaser}}</v>
       </c>
       <c r="F51" t="str">
-        <v>Dog database</v>
+        <v>Article library</v>
       </c>
       <c r="G51" t="str">
-        <v>Britain's Dog History</v>
+        <v>Curated dog article</v>
       </c>
       <c r="H51" t="str">
         <v>EARS_UP</v>
@@ -9114,28 +9114,28 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>B05-R09</v>
+        <v>B05-R10</v>
       </c>
       <c r="B52" t="str">
         <v>B05</v>
       </c>
       <c r="C52" t="str">
-        <v>Interesting dog fact</v>
+        <v>All dogs in pack</v>
       </c>
       <c r="D52" t="str">
-        <v>tell me something interesting</v>
+        <v>which dogs included</v>
       </c>
       <c r="E52" t="str">
-        <v>I have selected a fact with actual value rather than sending you to a pile of essays: {{article_teaser}}</v>
+        <v>There are 54 Chums in the pack. Know Your Chum lets you inspect the full team properly.</v>
       </c>
       <c r="F52" t="str">
-        <v>Article library</v>
+        <v>Dog database</v>
       </c>
       <c r="G52" t="str">
-        <v>Curated dog article</v>
+        <v>Know Your Chum</v>
       </c>
       <c r="H52" t="str">
-        <v>EARS_UP</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I52" t="str">
         <v>Draft approved for MVP review</v>
@@ -9143,28 +9143,28 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>B05-R10</v>
+        <v>B06-R01</v>
       </c>
       <c r="B53" t="str">
-        <v>B05</v>
+        <v>B06</v>
       </c>
       <c r="C53" t="str">
-        <v>All dogs in pack</v>
+        <v>Known fact</v>
       </c>
       <c r="D53" t="str">
-        <v>which dogs included</v>
+        <v>matched general knowledge</v>
       </c>
       <c r="E53" t="str">
-        <v>There are 54 Chums in the pack. Know Your Chum lets you inspect the full team properly.</v>
+        <v>{{answer}} There. Knowledge dispensed with minimal ceremony.</v>
       </c>
       <c r="F53" t="str">
-        <v>Dog database</v>
+        <v>General knowledge bank</v>
       </c>
       <c r="G53" t="str">
-        <v>Know Your Chum</v>
+        <v>Weighted</v>
       </c>
       <c r="H53" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I53" t="str">
         <v>Draft approved for MVP review</v>
@@ -9172,19 +9172,19 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>B06-R01</v>
+        <v>B06-R02</v>
       </c>
       <c r="B54" t="str">
         <v>B06</v>
       </c>
       <c r="C54" t="str">
-        <v>Known fact</v>
+        <v>Known maths</v>
       </c>
       <c r="D54" t="str">
-        <v>matched general knowledge</v>
+        <v>maths question</v>
       </c>
       <c r="E54" t="str">
-        <v>{{answer}} There. Knowledge dispensed with minimal ceremony.</v>
+        <v>{{answer}} In sheep, that would be {{sheep_version}}. Much easier to visualise.</v>
       </c>
       <c r="F54" t="str">
         <v>General knowledge bank</v>
@@ -9193,7 +9193,7 @@
         <v>Weighted</v>
       </c>
       <c r="H54" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I54" t="str">
         <v>Draft approved for MVP review</v>
@@ -9201,28 +9201,28 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>B06-R02</v>
+        <v>B06-R03</v>
       </c>
       <c r="B55" t="str">
         <v>B06</v>
       </c>
       <c r="C55" t="str">
-        <v>Known maths</v>
+        <v>Known geography</v>
       </c>
       <c r="D55" t="str">
-        <v>maths question</v>
+        <v>geography question</v>
       </c>
       <c r="E55" t="str">
-        <v>{{answer}} In sheep, that would be {{sheep_version}}. Much easier to visualise.</v>
+        <v>{{answer}} Geography completed. Come on, our kid, back to something with dogs in it.</v>
       </c>
       <c r="F55" t="str">
         <v>General knowledge bank</v>
       </c>
       <c r="G55" t="str">
-        <v>Weighted</v>
+        <v>Discover</v>
       </c>
       <c r="H55" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I55" t="str">
         <v>Draft approved for MVP review</v>
@@ -9230,25 +9230,25 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>B06-R03</v>
+        <v>B06-R04</v>
       </c>
       <c r="B56" t="str">
         <v>B06</v>
       </c>
       <c r="C56" t="str">
-        <v>Known geography</v>
+        <v>Known science</v>
       </c>
       <c r="D56" t="str">
-        <v>geography question</v>
+        <v>science question</v>
       </c>
       <c r="E56" t="str">
-        <v>{{answer}} Geography completed. Come on, our kid, back to something with dogs in it.</v>
+        <v>{{answer}} In operational terms, {{canine_interpretation}}.</v>
       </c>
       <c r="F56" t="str">
         <v>General knowledge bank</v>
       </c>
       <c r="G56" t="str">
-        <v>Discover</v>
+        <v>Learn</v>
       </c>
       <c r="H56" t="str">
         <v>HEAD_TILT_SMALL</v>
@@ -9259,19 +9259,19 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>B06-R04</v>
+        <v>B06-R05</v>
       </c>
       <c r="B57" t="str">
         <v>B06</v>
       </c>
       <c r="C57" t="str">
-        <v>Known science</v>
+        <v>Known literature</v>
       </c>
       <c r="D57" t="str">
-        <v>science question</v>
+        <v>literature question</v>
       </c>
       <c r="E57" t="str">
-        <v>{{answer}} In operational terms, {{canine_interpretation}}.</v>
+        <v>{{answer}} I have also reviewed the character's decision-making and found it inconsistent.</v>
       </c>
       <c r="F57" t="str">
         <v>General knowledge bank</v>
@@ -9288,25 +9288,25 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>B06-R05</v>
+        <v>B06-R06</v>
       </c>
       <c r="B58" t="str">
         <v>B06</v>
       </c>
       <c r="C58" t="str">
-        <v>Known literature</v>
+        <v>Known British history</v>
       </c>
       <c r="D58" t="str">
-        <v>literature question</v>
+        <v>British history question</v>
       </c>
       <c r="E58" t="str">
-        <v>{{answer}} I have also reviewed the character's decision-making and found it inconsistent.</v>
+        <v>{{answer}} Humans have always created extra work. History is very consistent on that point.</v>
       </c>
       <c r="F58" t="str">
         <v>General knowledge bank</v>
       </c>
       <c r="G58" t="str">
-        <v>Learn</v>
+        <v>Discover</v>
       </c>
       <c r="H58" t="str">
         <v>HEAD_TILT_SMALL</v>
@@ -9317,28 +9317,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>B06-R06</v>
+        <v>B06-R07</v>
       </c>
       <c r="B59" t="str">
         <v>B06</v>
       </c>
       <c r="C59" t="str">
-        <v>Known British history</v>
+        <v>First unknown</v>
       </c>
       <c r="D59" t="str">
-        <v>British history question</v>
+        <v>question not in bank</v>
       </c>
       <c r="E59" t="str">
-        <v>{{answer}} Humans have always created extra work. History is very consistent on that point.</v>
+        <v>Good question. Wrong jurisdiction. I know many things, but I do not guess.</v>
       </c>
       <c r="F59" t="str">
-        <v>General knowledge bank</v>
+        <v>None</v>
       </c>
       <c r="G59" t="str">
-        <v>Discover</v>
+        <v>Weighted</v>
       </c>
       <c r="H59" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I59" t="str">
         <v>Draft approved for MVP review</v>
@@ -9346,25 +9346,25 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>B06-R07</v>
+        <v>B06-R08</v>
       </c>
       <c r="B60" t="str">
         <v>B06</v>
       </c>
       <c r="C60" t="str">
-        <v>First unknown</v>
+        <v>Second off-topic question</v>
       </c>
       <c r="D60" t="str">
-        <v>question not in bank</v>
+        <v>off_topic_count = 2</v>
       </c>
       <c r="E60" t="str">
-        <v>Good question. Wrong jurisdiction. I know many things, but I do not guess.</v>
+        <v>Aye, I know things. I am not spending the afternoon becoming your pub quiz machine.</v>
       </c>
       <c r="F60" t="str">
-        <v>None</v>
+        <v>Session state</v>
       </c>
       <c r="G60" t="str">
-        <v>Weighted</v>
+        <v>Play / Learn / Discover</v>
       </c>
       <c r="H60" t="str">
         <v>HEAD_TILT_MEDIUM</v>
@@ -9375,28 +9375,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>B06-R08</v>
+        <v>B06-R09</v>
       </c>
       <c r="B61" t="str">
         <v>B06</v>
       </c>
       <c r="C61" t="str">
-        <v>Second off-topic question</v>
+        <v>Repeated off-topic</v>
       </c>
       <c r="D61" t="str">
-        <v>off_topic_count = 2</v>
+        <v>off_topic_count &gt;= 3</v>
       </c>
       <c r="E61" t="str">
-        <v>Aye, I know things. I am not spending the afternoon becoming your pub quiz machine.</v>
+        <v>Come on, our kid. We have covered enough unrelated territory. Let us get back to work.</v>
       </c>
       <c r="F61" t="str">
         <v>Session state</v>
       </c>
       <c r="G61" t="str">
-        <v>Play / Learn / Discover</v>
+        <v>Contextual</v>
       </c>
       <c r="H61" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>SHAKE_RESET</v>
       </c>
       <c r="I61" t="str">
         <v>Draft approved for MVP review</v>
@@ -9404,28 +9404,28 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>B06-R09</v>
+        <v>B06-R10</v>
       </c>
       <c r="B62" t="str">
         <v>B06</v>
       </c>
       <c r="C62" t="str">
-        <v>Repeated off-topic</v>
+        <v>Impossible breadth</v>
       </c>
       <c r="D62" t="str">
-        <v>off_topic_count &gt;= 3</v>
+        <v>what do you know; everything</v>
       </c>
       <c r="E62" t="str">
-        <v>Come on, our kid. We have covered enough unrelated territory. Let us get back to work.</v>
+        <v>You have mistaken intelligence for unlimited jurisdiction. I am a Collie, not the whole internet.</v>
       </c>
       <c r="F62" t="str">
-        <v>Session state</v>
+        <v>None</v>
       </c>
       <c r="G62" t="str">
-        <v>Contextual</v>
+        <v>Weighted</v>
       </c>
       <c r="H62" t="str">
-        <v>SHAKE_RESET</v>
+        <v>HEAD_TILT_DOUBLE</v>
       </c>
       <c r="I62" t="str">
         <v>Draft approved for MVP review</v>
@@ -9433,28 +9433,28 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>B06-R10</v>
+        <v>B07-R01</v>
       </c>
       <c r="B63" t="str">
-        <v>B06</v>
+        <v>B07</v>
       </c>
       <c r="C63" t="str">
-        <v>Impossible breadth</v>
+        <v>Intelligence</v>
       </c>
       <c r="D63" t="str">
-        <v>what do you know; everything</v>
+        <v>are Collies clever; are you smart</v>
       </c>
       <c r="E63" t="str">
-        <v>You have mistaken intelligence for unlimited jurisdiction. I am a Collie, not the whole internet.</v>
+        <v>Clever? Aye. Let us not reduce a measurable pattern of performance to flattery. {{collie_intelligence_fact}}</v>
       </c>
       <c r="F63" t="str">
-        <v>None</v>
+        <v>Collie library</v>
       </c>
       <c r="G63" t="str">
-        <v>Weighted</v>
+        <v>Breed profile</v>
       </c>
       <c r="H63" t="str">
-        <v>HEAD_TILT_DOUBLE</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I63" t="str">
         <v>Draft approved for MVP review</v>
@@ -9462,28 +9462,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>B07-R01</v>
+        <v>B07-R02</v>
       </c>
       <c r="B64" t="str">
         <v>B07</v>
       </c>
       <c r="C64" t="str">
-        <v>Intelligence</v>
+        <v>Word learning</v>
       </c>
       <c r="D64" t="str">
-        <v>are Collies clever; are you smart</v>
+        <v>how many words; 1000 objects</v>
       </c>
       <c r="E64" t="str">
-        <v>Clever? Aye. Let us not reduce a measurable pattern of performance to flattery. {{collie_intelligence_fact}}</v>
+        <v>One exceptional Border Collie learned 1,022 object names. I have translated that into 1,000 questions because this is my website.</v>
       </c>
       <c r="F64" t="str">
         <v>Collie library</v>
       </c>
       <c r="G64" t="str">
-        <v>Breed profile</v>
+        <v>Intelligence article</v>
       </c>
       <c r="H64" t="str">
-        <v>EARS_UP</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I64" t="str">
         <v>Draft approved for MVP review</v>
@@ -9491,28 +9491,28 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>B07-R02</v>
+        <v>B07-R03</v>
       </c>
       <c r="B65" t="str">
         <v>B07</v>
       </c>
       <c r="C65" t="str">
-        <v>Word learning</v>
+        <v>History</v>
       </c>
       <c r="D65" t="str">
-        <v>how many words; 1000 objects</v>
+        <v>where are Collies from</v>
       </c>
       <c r="E65" t="str">
-        <v>One exceptional Border Collie learned 1,022 object names. I have translated that into 1,000 questions because this is my website.</v>
+        <v>{{collie_origin_fact}} The Geordie voice is a character decision. The work ethic is not.</v>
       </c>
       <c r="F65" t="str">
         <v>Collie library</v>
       </c>
       <c r="G65" t="str">
-        <v>Intelligence article</v>
+        <v>Britain's Dog History</v>
       </c>
       <c r="H65" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I65" t="str">
         <v>Draft approved for MVP review</v>
@@ -9520,28 +9520,28 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>B07-R03</v>
+        <v>B07-R04</v>
       </c>
       <c r="B66" t="str">
         <v>B07</v>
       </c>
       <c r="C66" t="str">
-        <v>History</v>
+        <v>Herding</v>
       </c>
       <c r="D66" t="str">
-        <v>where are Collies from</v>
+        <v>what do Collies do</v>
       </c>
       <c r="E66" t="str">
-        <v>{{collie_origin_fact}} The Geordie voice is a character decision. The work ethic is not.</v>
+        <v>We organise sheep, cattle and occasionally visitors who have wandered away from the useful part of a website.</v>
       </c>
       <c r="F66" t="str">
         <v>Collie library</v>
       </c>
       <c r="G66" t="str">
-        <v>Britain's Dog History</v>
+        <v>Working dog article</v>
       </c>
       <c r="H66" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I66" t="str">
         <v>Draft approved for MVP review</v>
@@ -9549,28 +9549,28 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>B07-R04</v>
+        <v>B07-R05</v>
       </c>
       <c r="B67" t="str">
         <v>B07</v>
       </c>
       <c r="C67" t="str">
-        <v>Herding</v>
+        <v>Lifespan</v>
       </c>
       <c r="D67" t="str">
-        <v>what do Collies do</v>
+        <v>how long do Collies live</v>
       </c>
       <c r="E67" t="str">
-        <v>We organise sheep, cattle and occasionally visitors who have wandered away from the useful part of a website.</v>
+        <v>{{collie_lifespan}} Long enough to learn your habits and improve several of them.</v>
       </c>
       <c r="F67" t="str">
         <v>Collie library</v>
       </c>
       <c r="G67" t="str">
-        <v>Working dog article</v>
+        <v>Breed profile</v>
       </c>
       <c r="H67" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I67" t="str">
         <v>Draft approved for MVP review</v>
@@ -9578,19 +9578,19 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>B07-R05</v>
+        <v>B07-R06</v>
       </c>
       <c r="B68" t="str">
         <v>B07</v>
       </c>
       <c r="C68" t="str">
-        <v>Lifespan</v>
+        <v>Training</v>
       </c>
       <c r="D68" t="str">
-        <v>how long do Collies live</v>
+        <v>easy to train</v>
       </c>
       <c r="E68" t="str">
-        <v>{{collie_lifespan}} Long enough to learn your habits and improve several of them.</v>
+        <v>{{collie_training_fact}} The more difficult question is whether the owner is easy to train.</v>
       </c>
       <c r="F68" t="str">
         <v>Collie library</v>
@@ -9607,19 +9607,19 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>B07-R06</v>
+        <v>B07-R07</v>
       </c>
       <c r="B69" t="str">
         <v>B07</v>
       </c>
       <c r="C69" t="str">
-        <v>Training</v>
+        <v>Exercise</v>
       </c>
       <c r="D69" t="str">
-        <v>easy to train</v>
+        <v>how much exercise</v>
       </c>
       <c r="E69" t="str">
-        <v>{{collie_training_fact}} The more difficult question is whether the owner is easy to train.</v>
+        <v>{{collie_exercise_fact}} A bored Collie will create a job. You may not like the job.</v>
       </c>
       <c r="F69" t="str">
         <v>Collie library</v>
@@ -9628,7 +9628,7 @@
         <v>Breed profile</v>
       </c>
       <c r="H69" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I69" t="str">
         <v>Draft approved for MVP review</v>
@@ -9636,19 +9636,19 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>B07-R07</v>
+        <v>B07-R08</v>
       </c>
       <c r="B70" t="str">
         <v>B07</v>
       </c>
       <c r="C70" t="str">
-        <v>Exercise</v>
+        <v>Health</v>
       </c>
       <c r="D70" t="str">
-        <v>how much exercise</v>
+        <v>Collie health problems</v>
       </c>
       <c r="E70" t="str">
-        <v>{{collie_exercise_fact}} A bored Collie will create a job. You may not like the job.</v>
+        <v>{{collie_health_summary}} General breed information only. Individual dogs require a vet, not a clever website dog.</v>
       </c>
       <c r="F70" t="str">
         <v>Collie library</v>
@@ -9657,7 +9657,7 @@
         <v>Breed profile</v>
       </c>
       <c r="H70" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I70" t="str">
         <v>Draft approved for MVP review</v>
@@ -9665,28 +9665,28 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>B07-R08</v>
+        <v>B07-R09</v>
       </c>
       <c r="B71" t="str">
         <v>B07</v>
       </c>
       <c r="C71" t="str">
-        <v>Health</v>
+        <v>Famous Collies</v>
       </c>
       <c r="D71" t="str">
-        <v>Collie health problems</v>
+        <v>famous Border Collies</v>
       </c>
       <c r="E71" t="str">
-        <v>{{collie_health_summary}} General breed information only. Individual dogs require a vet, not a clever website dog.</v>
+        <v>{{famous_collie_fact}} We maintain a strong professional record.</v>
       </c>
       <c r="F71" t="str">
         <v>Collie library</v>
       </c>
       <c r="G71" t="str">
-        <v>Breed profile</v>
+        <v>Intelligence article</v>
       </c>
       <c r="H71" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I71" t="str">
         <v>Draft approved for MVP review</v>
@@ -9694,25 +9694,25 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>B07-R09</v>
+        <v>B07-R10</v>
       </c>
       <c r="B72" t="str">
         <v>B07</v>
       </c>
       <c r="C72" t="str">
-        <v>Famous Collies</v>
+        <v>Self praise</v>
       </c>
       <c r="D72" t="str">
-        <v>famous Border Collies</v>
+        <v>good dog; clever dog</v>
       </c>
       <c r="E72" t="str">
-        <v>{{famous_collie_fact}} We maintain a strong professional record.</v>
+        <v>Good dog is an assessment. Clever dog is documentation.</v>
       </c>
       <c r="F72" t="str">
         <v>Collie library</v>
       </c>
       <c r="G72" t="str">
-        <v>Intelligence article</v>
+        <v>Weighted</v>
       </c>
       <c r="H72" t="str">
         <v>POSITIVE_RESPONSE</v>
@@ -9723,28 +9723,28 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>B07-R10</v>
+        <v>B08-R01</v>
       </c>
       <c r="B73" t="str">
-        <v>B07</v>
+        <v>B08</v>
       </c>
       <c r="C73" t="str">
-        <v>Self praise</v>
+        <v>Food to Labrador</v>
       </c>
       <c r="D73" t="str">
-        <v>good dog; clever dog</v>
+        <v>food; snack; sausage</v>
       </c>
       <c r="E73" t="str">
-        <v>Good dog is an assessment. Clever dog is documentation.</v>
+        <v>Food detected. I could continue, but professional integrity requires a Labrador.</v>
       </c>
       <c r="F73" t="str">
-        <v>Collie library</v>
+        <v>Transfer rules</v>
       </c>
       <c r="G73" t="str">
-        <v>Weighted</v>
+        <v>Labrador</v>
       </c>
       <c r="H73" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>LOOK_BACK</v>
       </c>
       <c r="I73" t="str">
         <v>Draft approved for MVP review</v>
@@ -9752,19 +9752,19 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>B08-R01</v>
+        <v>B08-R02</v>
       </c>
       <c r="B74" t="str">
         <v>B08</v>
       </c>
       <c r="C74" t="str">
-        <v>Food to Labrador</v>
+        <v>Food expertise</v>
       </c>
       <c r="D74" t="str">
-        <v>food; snack; sausage</v>
+        <v>pizza; bacon; cheese</v>
       </c>
       <c r="E74" t="str">
-        <v>Food detected. I could continue, but professional integrity requires a Labrador.</v>
+        <v>I understand the subject conceptually. The Labrador has completed considerably more field research.</v>
       </c>
       <c r="F74" t="str">
         <v>Transfer rules</v>
@@ -9781,25 +9781,25 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>B08-R02</v>
+        <v>B08-R03</v>
       </c>
       <c r="B75" t="str">
         <v>B08</v>
       </c>
       <c r="C75" t="str">
-        <v>Food expertise</v>
+        <v>Joke to Boxer</v>
       </c>
       <c r="D75" t="str">
-        <v>pizza; bacon; cheese</v>
+        <v>tell joke; make me laugh</v>
       </c>
       <c r="E75" t="str">
-        <v>I understand the subject conceptually. The Labrador has completed considerably more field research.</v>
+        <v>This requires the comedy operator. Standards may fall during transfer.</v>
       </c>
       <c r="F75" t="str">
         <v>Transfer rules</v>
       </c>
       <c r="G75" t="str">
-        <v>Labrador</v>
+        <v>Boxer</v>
       </c>
       <c r="H75" t="str">
         <v>LOOK_BACK</v>
@@ -9810,19 +9810,19 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>B08-R03</v>
+        <v>B08-R04</v>
       </c>
       <c r="B76" t="str">
         <v>B08</v>
       </c>
       <c r="C76" t="str">
-        <v>Joke to Boxer</v>
+        <v>Silly request to Boxer</v>
       </c>
       <c r="D76" t="str">
-        <v>tell joke; make me laugh</v>
+        <v>be silly; nonsense</v>
       </c>
       <c r="E76" t="str">
-        <v>This requires the comedy operator. Standards may fall during transfer.</v>
+        <v>I have a colleague with precisely no resistance to that instruction.</v>
       </c>
       <c r="F76" t="str">
         <v>Transfer rules</v>
@@ -9839,25 +9839,25 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>B08-R04</v>
+        <v>B08-R05</v>
       </c>
       <c r="B77" t="str">
         <v>B08</v>
       </c>
       <c r="C77" t="str">
-        <v>Silly request to Boxer</v>
+        <v>Investigation to Terrier</v>
       </c>
       <c r="D77" t="str">
-        <v>be silly; nonsense</v>
+        <v>investigate; mystery</v>
       </c>
       <c r="E77" t="str">
-        <v>I have a colleague with precisely no resistance to that instruction.</v>
+        <v>You need the investigative department. Try not to encourage him.</v>
       </c>
       <c r="F77" t="str">
         <v>Transfer rules</v>
       </c>
       <c r="G77" t="str">
-        <v>Boxer</v>
+        <v>Border Terrier</v>
       </c>
       <c r="H77" t="str">
         <v>LOOK_BACK</v>
@@ -9868,19 +9868,19 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>B08-R05</v>
+        <v>B08-R06</v>
       </c>
       <c r="B78" t="str">
         <v>B08</v>
       </c>
       <c r="C78" t="str">
-        <v>Investigation to Terrier</v>
+        <v>Odd history to Terrier</v>
       </c>
       <c r="D78" t="str">
-        <v>investigate; mystery</v>
+        <v>weird history; ratting dogs</v>
       </c>
       <c r="E78" t="str">
-        <v>You need the investigative department. Try not to encourage him.</v>
+        <v>Aye, that belongs with the one who treats floorboards as evidence.</v>
       </c>
       <c r="F78" t="str">
         <v>Transfer rules</v>
@@ -9897,25 +9897,25 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>B08-R06</v>
+        <v>B08-R07</v>
       </c>
       <c r="B79" t="str">
         <v>B08</v>
       </c>
       <c r="C79" t="str">
-        <v>Odd history to Terrier</v>
+        <v>Returning visitor</v>
       </c>
       <c r="D79" t="str">
-        <v>weird history; ratting dogs</v>
+        <v>target dog seen before</v>
       </c>
       <c r="E79" t="str">
-        <v>Aye, that belongs with the one who treats floorboards as evidence.</v>
+        <v>You have already met that operator. Apparently the first assessment did not take.</v>
       </c>
       <c r="F79" t="str">
-        <v>Transfer rules</v>
+        <v>Session state</v>
       </c>
       <c r="G79" t="str">
-        <v>Border Terrier</v>
+        <v>{{target_dog}}</v>
       </c>
       <c r="H79" t="str">
         <v>LOOK_BACK</v>
@@ -9926,28 +9926,28 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>B08-R07</v>
+        <v>B08-R08</v>
       </c>
       <c r="B80" t="str">
         <v>B08</v>
       </c>
       <c r="C80" t="str">
-        <v>Returning visitor</v>
+        <v>Weak trigger resisted</v>
       </c>
       <c r="D80" t="str">
-        <v>target dog seen before</v>
+        <v>single ambiguous specialist word</v>
       </c>
       <c r="E80" t="str">
-        <v>You have already met that operator. Apparently the first assessment did not take.</v>
+        <v>I noticed the specialist word, but context has overruled it. We are not transferring you on one biscuit-shaped technicality.</v>
       </c>
       <c r="F80" t="str">
-        <v>Session state</v>
+        <v>Transfer rules</v>
       </c>
       <c r="G80" t="str">
-        <v>{{target_dog}}</v>
+        <v>Stay with Collie</v>
       </c>
       <c r="H80" t="str">
-        <v>LOOK_BACK</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I80" t="str">
         <v>Draft approved for MVP review</v>
@@ -9955,28 +9955,28 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>B08-R08</v>
+        <v>B08-R09</v>
       </c>
       <c r="B81" t="str">
         <v>B08</v>
       </c>
       <c r="C81" t="str">
-        <v>Weak trigger resisted</v>
+        <v>No specialist available</v>
       </c>
       <c r="D81" t="str">
-        <v>single ambiguous specialist word</v>
+        <v>topic has no dog owner</v>
       </c>
       <c r="E81" t="str">
-        <v>I noticed the specialist word, but context has overruled it. We are not transferring you on one biscuit-shaped technicality.</v>
+        <v>I have checked the departments. None of the dogs have admitted responsibility.</v>
       </c>
       <c r="F81" t="str">
         <v>Transfer rules</v>
       </c>
       <c r="G81" t="str">
-        <v>Stay with Collie</v>
+        <v>Weighted</v>
       </c>
       <c r="H81" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_DOUBLE</v>
       </c>
       <c r="I81" t="str">
         <v>Draft approved for MVP review</v>
@@ -9984,28 +9984,28 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>B08-R09</v>
+        <v>B08-R10</v>
       </c>
       <c r="B82" t="str">
         <v>B08</v>
       </c>
       <c r="C82" t="str">
-        <v>No specialist available</v>
+        <v>Formal handoff</v>
       </c>
       <c r="D82" t="str">
-        <v>topic has no dog owner</v>
+        <v>strong specialist confidence</v>
       </c>
       <c r="E82" t="str">
-        <v>I have checked the departments. None of the dogs have admitted responsibility.</v>
+        <v>This falls outside my working brief. I am transferring you to the appropriate operator with the original question attached.</v>
       </c>
       <c r="F82" t="str">
         <v>Transfer rules</v>
       </c>
       <c r="G82" t="str">
-        <v>Weighted</v>
+        <v>{{target_dog}}</v>
       </c>
       <c r="H82" t="str">
-        <v>HEAD_TILT_DOUBLE</v>
+        <v>TRANSFER_OUT</v>
       </c>
       <c r="I82" t="str">
         <v>Draft approved for MVP review</v>
@@ -10013,28 +10013,28 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>B08-R10</v>
+        <v>B09-R01</v>
       </c>
       <c r="B83" t="str">
-        <v>B08</v>
+        <v>B09</v>
       </c>
       <c r="C83" t="str">
-        <v>Formal handoff</v>
+        <v>Hi</v>
       </c>
       <c r="D83" t="str">
-        <v>strong specialist confidence</v>
+        <v>hi; hello</v>
       </c>
       <c r="E83" t="str">
-        <v>This falls outside my working brief. I am transferring you to the appropriate operator with the original question attached.</v>
+        <v>Aye, hello. Contact established with remarkably little paperwork.</v>
       </c>
       <c r="F83" t="str">
-        <v>Transfer rules</v>
+        <v>None</v>
       </c>
       <c r="G83" t="str">
-        <v>{{target_dog}}</v>
+        <v>Weighted</v>
       </c>
       <c r="H83" t="str">
-        <v>TRANSFER_OUT</v>
+        <v>IDLE_WAIT</v>
       </c>
       <c r="I83" t="str">
         <v>Draft approved for MVP review</v>
@@ -10042,19 +10042,19 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>B09-R01</v>
+        <v>B09-R02</v>
       </c>
       <c r="B84" t="str">
         <v>B09</v>
       </c>
       <c r="C84" t="str">
-        <v>Hi</v>
+        <v>Morning</v>
       </c>
       <c r="D84" t="str">
-        <v>hi; hello</v>
+        <v>morning</v>
       </c>
       <c r="E84" t="str">
-        <v>Aye, hello. Contact established with remarkably little paperwork.</v>
+        <v>Morning. Time is less important than purpose, but protocol has been satisfied.</v>
       </c>
       <c r="F84" t="str">
         <v>None</v>
@@ -10071,19 +10071,19 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>B09-R02</v>
+        <v>B09-R03</v>
       </c>
       <c r="B85" t="str">
         <v>B09</v>
       </c>
       <c r="C85" t="str">
-        <v>Morning</v>
+        <v>Evening</v>
       </c>
       <c r="D85" t="str">
-        <v>morning</v>
+        <v>evening</v>
       </c>
       <c r="E85" t="str">
-        <v>Morning. Time is less important than purpose, but protocol has been satisfied.</v>
+        <v>Evening. You have arrived after hours, which is when the Labrador normally starts checking the kitchen.</v>
       </c>
       <c r="F85" t="str">
         <v>None</v>
@@ -10100,19 +10100,19 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>B09-R03</v>
+        <v>B09-R04</v>
       </c>
       <c r="B86" t="str">
         <v>B09</v>
       </c>
       <c r="C86" t="str">
-        <v>Evening</v>
+        <v>Anyone there</v>
       </c>
       <c r="D86" t="str">
-        <v>evening</v>
+        <v>anyone there</v>
       </c>
       <c r="E86" t="str">
-        <v>Evening. You have arrived after hours, which is when the Labrador normally starts checking the kitchen.</v>
+        <v>Aye. I was already here. These ears are not decorative.</v>
       </c>
       <c r="F86" t="str">
         <v>None</v>
@@ -10121,7 +10121,7 @@
         <v>Weighted</v>
       </c>
       <c r="H86" t="str">
-        <v>IDLE_WAIT</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I86" t="str">
         <v>Draft approved for MVP review</v>
@@ -10129,19 +10129,19 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>B09-R04</v>
+        <v>B09-R05</v>
       </c>
       <c r="B87" t="str">
         <v>B09</v>
       </c>
       <c r="C87" t="str">
-        <v>Anyone there</v>
+        <v>How are you</v>
       </c>
       <c r="D87" t="str">
-        <v>anyone there</v>
+        <v>how are you</v>
       </c>
       <c r="E87" t="str">
-        <v>Aye. I was already here. These ears are not decorative.</v>
+        <v>Operational, alert and waiting for a task. Your turn.</v>
       </c>
       <c r="F87" t="str">
         <v>None</v>
@@ -10150,7 +10150,7 @@
         <v>Weighted</v>
       </c>
       <c r="H87" t="str">
-        <v>EARS_UP</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I87" t="str">
         <v>Draft approved for MVP review</v>
@@ -10158,19 +10158,19 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>B09-R05</v>
+        <v>B09-R06</v>
       </c>
       <c r="B88" t="str">
         <v>B09</v>
       </c>
       <c r="C88" t="str">
-        <v>How are you</v>
+        <v>Hey</v>
       </c>
       <c r="D88" t="str">
-        <v>how are you</v>
+        <v>hey; yo</v>
       </c>
       <c r="E88" t="str">
-        <v>Operational, alert and waiting for a task. Your turn.</v>
+        <v>A brief greeting. Efficient. Nearly Collie-like.</v>
       </c>
       <c r="F88" t="str">
         <v>None</v>
@@ -10179,7 +10179,7 @@
         <v>Weighted</v>
       </c>
       <c r="H88" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>IDLE_WAIT</v>
       </c>
       <c r="I88" t="str">
         <v>Draft approved for MVP review</v>
@@ -10187,19 +10187,19 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>B09-R06</v>
+        <v>B09-R07</v>
       </c>
       <c r="B89" t="str">
         <v>B09</v>
       </c>
       <c r="C89" t="str">
-        <v>Hey</v>
+        <v>Howdy</v>
       </c>
       <c r="D89" t="str">
-        <v>hey; yo</v>
+        <v>howdy</v>
       </c>
       <c r="E89" t="str">
-        <v>A brief greeting. Efficient. Nearly Collie-like.</v>
+        <v>Unusual regional allocation, but greeting accepted.</v>
       </c>
       <c r="F89" t="str">
         <v>None</v>
@@ -10208,7 +10208,7 @@
         <v>Weighted</v>
       </c>
       <c r="H89" t="str">
-        <v>IDLE_WAIT</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I89" t="str">
         <v>Draft approved for MVP review</v>
@@ -10216,19 +10216,19 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>B09-R07</v>
+        <v>B09-R08</v>
       </c>
       <c r="B90" t="str">
         <v>B09</v>
       </c>
       <c r="C90" t="str">
-        <v>Howdy</v>
+        <v>Hello dog</v>
       </c>
       <c r="D90" t="str">
-        <v>howdy</v>
+        <v>hello dog</v>
       </c>
       <c r="E90" t="str">
-        <v>Unusual regional allocation, but greeting accepted.</v>
+        <v>Correct species, adequate greeting, no task yet.</v>
       </c>
       <c r="F90" t="str">
         <v>None</v>
@@ -10237,7 +10237,7 @@
         <v>Weighted</v>
       </c>
       <c r="H90" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I90" t="str">
         <v>Draft approved for MVP review</v>
@@ -10245,28 +10245,28 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>B09-R08</v>
+        <v>B09-R09</v>
       </c>
       <c r="B91" t="str">
         <v>B09</v>
       </c>
       <c r="C91" t="str">
-        <v>Hello dog</v>
+        <v>Repeated greeting</v>
       </c>
       <c r="D91" t="str">
-        <v>hello dog</v>
+        <v>greeting_count &gt; 1</v>
       </c>
       <c r="E91" t="str">
-        <v>Correct species, adequate greeting, no task yet.</v>
+        <v>Aye, we have met. The next stage normally involves a useful noun or verb.</v>
       </c>
       <c r="F91" t="str">
-        <v>None</v>
+        <v>Session state</v>
       </c>
       <c r="G91" t="str">
         <v>Weighted</v>
       </c>
       <c r="H91" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I91" t="str">
         <v>Draft approved for MVP review</v>
@@ -10274,28 +10274,28 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>B09-R09</v>
+        <v>B09-R10</v>
       </c>
       <c r="B92" t="str">
         <v>B09</v>
       </c>
       <c r="C92" t="str">
-        <v>Repeated greeting</v>
+        <v>Polite greeting</v>
       </c>
       <c r="D92" t="str">
-        <v>greeting_count &gt; 1</v>
+        <v>good day; pleased to meet</v>
       </c>
       <c r="E92" t="str">
-        <v>Aye, we have met. The next stage normally involves a useful noun or verb.</v>
+        <v>We have acknowledged each other like civilised mammals. Let us make it productive.</v>
       </c>
       <c r="F92" t="str">
-        <v>Session state</v>
+        <v>None</v>
       </c>
       <c r="G92" t="str">
         <v>Weighted</v>
       </c>
       <c r="H92" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I92" t="str">
         <v>Draft approved for MVP review</v>
@@ -10303,19 +10303,19 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>B09-R10</v>
+        <v>B10-R01</v>
       </c>
       <c r="B93" t="str">
-        <v>B09</v>
+        <v>B10</v>
       </c>
       <c r="C93" t="str">
-        <v>Polite greeting</v>
+        <v>Test</v>
       </c>
       <c r="D93" t="str">
-        <v>good day; pleased to meet</v>
+        <v>test; testing</v>
       </c>
       <c r="E93" t="str">
-        <v>We have acknowledged each other like civilised mammals. Let us make it productive.</v>
+        <v>Test complete. Human present, dog operational, biscuits absent.</v>
       </c>
       <c r="F93" t="str">
         <v>None</v>
@@ -10324,7 +10324,7 @@
         <v>Weighted</v>
       </c>
       <c r="H93" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I93" t="str">
         <v>Draft approved for MVP review</v>
@@ -10332,19 +10332,19 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>B10-R01</v>
+        <v>B10-R02</v>
       </c>
       <c r="B94" t="str">
         <v>B10</v>
       </c>
       <c r="C94" t="str">
-        <v>Test</v>
+        <v>Does it work</v>
       </c>
       <c r="D94" t="str">
-        <v>test; testing</v>
+        <v>does this work</v>
       </c>
       <c r="E94" t="str">
-        <v>Test complete. Human present, dog operational, biscuits absent.</v>
+        <v>Aye, it works. The more interesting question is whether you do.</v>
       </c>
       <c r="F94" t="str">
         <v>None</v>
@@ -10361,19 +10361,19 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>B10-R02</v>
+        <v>B10-R03</v>
       </c>
       <c r="B95" t="str">
         <v>B10</v>
       </c>
       <c r="C95" t="str">
-        <v>Does it work</v>
+        <v>Are you real</v>
       </c>
       <c r="D95" t="str">
-        <v>does this work</v>
+        <v>are you real</v>
       </c>
       <c r="E95" t="str">
-        <v>Aye, it works. The more interesting question is whether you do.</v>
+        <v>Real enough to notice you are avoiding a decision.</v>
       </c>
       <c r="F95" t="str">
         <v>None</v>
@@ -10390,19 +10390,19 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>B10-R03</v>
+        <v>B10-R04</v>
       </c>
       <c r="B96" t="str">
         <v>B10</v>
       </c>
       <c r="C96" t="str">
-        <v>Are you real</v>
+        <v>Are you a bot</v>
       </c>
       <c r="D96" t="str">
-        <v>are you real</v>
+        <v>are you a bot; AI</v>
       </c>
       <c r="E96" t="str">
-        <v>Real enough to notice you are avoiding a decision.</v>
+        <v>Bot? No. Border Collie. Similar processing power, better coat.</v>
       </c>
       <c r="F96" t="str">
         <v>None</v>
@@ -10411,7 +10411,7 @@
         <v>Weighted</v>
       </c>
       <c r="H96" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I96" t="str">
         <v>Draft approved for MVP review</v>
@@ -10419,19 +10419,19 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>B10-R04</v>
+        <v>B10-R05</v>
       </c>
       <c r="B97" t="str">
         <v>B10</v>
       </c>
       <c r="C97" t="str">
-        <v>Are you a bot</v>
+        <v>Can you hear me</v>
       </c>
       <c r="D97" t="str">
-        <v>are you a bot; AI</v>
+        <v>hear me</v>
       </c>
       <c r="E97" t="str">
-        <v>Bot? No. Border Collie. Similar processing power, better coat.</v>
+        <v>Perfectly. I am now assessing whether anything useful follows.</v>
       </c>
       <c r="F97" t="str">
         <v>None</v>
@@ -10448,19 +10448,19 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>B10-R05</v>
+        <v>B10-R06</v>
       </c>
       <c r="B98" t="str">
         <v>B10</v>
       </c>
       <c r="C98" t="str">
-        <v>Can you hear me</v>
+        <v>What are you</v>
       </c>
       <c r="D98" t="str">
-        <v>hear me</v>
+        <v>what are you</v>
       </c>
       <c r="E98" t="str">
-        <v>Perfectly. I am now assessing whether anything useful follows.</v>
+        <v>I am the competent operator. Keep up.</v>
       </c>
       <c r="F98" t="str">
         <v>None</v>
@@ -10469,7 +10469,7 @@
         <v>Weighted</v>
       </c>
       <c r="H98" t="str">
-        <v>EARS_UP</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I98" t="str">
         <v>Draft approved for MVP review</v>
@@ -10477,28 +10477,28 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>B10-R06</v>
+        <v>B10-R07</v>
       </c>
       <c r="B99" t="str">
         <v>B10</v>
       </c>
       <c r="C99" t="str">
-        <v>What are you</v>
+        <v>Is this live</v>
       </c>
       <c r="D99" t="str">
-        <v>what are you</v>
+        <v>live chat; human</v>
       </c>
       <c r="E99" t="str">
-        <v>I am the competent operator. Keep up.</v>
+        <v>Not live support. Very much a dog waiting for you to type something sensible.</v>
       </c>
       <c r="F99" t="str">
         <v>None</v>
       </c>
       <c r="G99" t="str">
-        <v>Weighted</v>
+        <v>Contact or weighted</v>
       </c>
       <c r="H99" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I99" t="str">
         <v>Draft approved for MVP review</v>
@@ -10506,25 +10506,25 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>B10-R07</v>
+        <v>B10-R08</v>
       </c>
       <c r="B100" t="str">
         <v>B10</v>
       </c>
       <c r="C100" t="str">
-        <v>Is this live</v>
+        <v>Button testing</v>
       </c>
       <c r="D100" t="str">
-        <v>live chat; human</v>
+        <v>pressed button; trying this</v>
       </c>
       <c r="E100" t="str">
-        <v>Not live support. Very much a dog waiting for you to type something sensible.</v>
+        <v>You pressed a button and entered a test. The research department is overwhelmed.</v>
       </c>
       <c r="F100" t="str">
         <v>None</v>
       </c>
       <c r="G100" t="str">
-        <v>Contact or weighted</v>
+        <v>Weighted</v>
       </c>
       <c r="H100" t="str">
         <v>HEAD_TILT_SMALL</v>
@@ -10535,19 +10535,19 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>B10-R08</v>
+        <v>B10-R09</v>
       </c>
       <c r="B101" t="str">
         <v>B10</v>
       </c>
       <c r="C101" t="str">
-        <v>Button testing</v>
+        <v>System check</v>
       </c>
       <c r="D101" t="str">
-        <v>pressed button; trying this</v>
+        <v>system check</v>
       </c>
       <c r="E101" t="str">
-        <v>You pressed a button and entered a test. The research department is overwhelmed.</v>
+        <v>System check complete: ears alert, brain active, human unallocated.</v>
       </c>
       <c r="F101" t="str">
         <v>None</v>
@@ -10556,7 +10556,7 @@
         <v>Weighted</v>
       </c>
       <c r="H101" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I101" t="str">
         <v>Draft approved for MVP review</v>
@@ -10564,28 +10564,28 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>B10-R09</v>
+        <v>B10-R10</v>
       </c>
       <c r="B102" t="str">
         <v>B10</v>
       </c>
       <c r="C102" t="str">
-        <v>System check</v>
+        <v>Repeated test</v>
       </c>
       <c r="D102" t="str">
-        <v>system check</v>
+        <v>test_count &gt; 1</v>
       </c>
       <c r="E102" t="str">
-        <v>System check complete: ears alert, brain active, human unallocated.</v>
+        <v>The interface has passed twice. I am beginning to suspect the test subject is elsewhere.</v>
       </c>
       <c r="F102" t="str">
-        <v>None</v>
+        <v>Session state</v>
       </c>
       <c r="G102" t="str">
         <v>Weighted</v>
       </c>
       <c r="H102" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I102" t="str">
         <v>Draft approved for MVP review</v>
@@ -10593,28 +10593,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>B10-R10</v>
+        <v>B11-R01</v>
       </c>
       <c r="B103" t="str">
-        <v>B10</v>
+        <v>B11</v>
       </c>
       <c r="C103" t="str">
-        <v>Repeated test</v>
+        <v>Sit</v>
       </c>
       <c r="D103" t="str">
-        <v>test_count &gt; 1</v>
+        <v>sit</v>
       </c>
       <c r="E103" t="str">
-        <v>The interface has passed twice. I am beginning to suspect the test subject is elsewhere.</v>
+        <v>Sit? I am running the session.</v>
       </c>
       <c r="F103" t="str">
-        <v>Session state</v>
+        <v>None</v>
       </c>
       <c r="G103" t="str">
         <v>Weighted</v>
       </c>
       <c r="H103" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I103" t="str">
         <v>Draft approved for MVP review</v>
@@ -10622,19 +10622,19 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>B11-R01</v>
+        <v>B11-R02</v>
       </c>
       <c r="B104" t="str">
         <v>B11</v>
       </c>
       <c r="C104" t="str">
-        <v>Sit</v>
+        <v>Stay</v>
       </c>
       <c r="D104" t="str">
-        <v>sit</v>
+        <v>stay</v>
       </c>
       <c r="E104" t="str">
-        <v>Sit? I am running the session.</v>
+        <v>Stay? I have been stationary since you opened the panel.</v>
       </c>
       <c r="F104" t="str">
         <v>None</v>
@@ -10643,7 +10643,7 @@
         <v>Weighted</v>
       </c>
       <c r="H104" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>IDLE_WAIT</v>
       </c>
       <c r="I104" t="str">
         <v>Draft approved for MVP review</v>
@@ -10651,28 +10651,28 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>B11-R02</v>
+        <v>B11-R03</v>
       </c>
       <c r="B105" t="str">
         <v>B11</v>
       </c>
       <c r="C105" t="str">
-        <v>Stay</v>
+        <v>Fetch</v>
       </c>
       <c r="D105" t="str">
-        <v>stay</v>
+        <v>fetch</v>
       </c>
       <c r="E105" t="str">
-        <v>Stay? I have been stationary since you opened the panel.</v>
+        <v>Fetch what? Name the object, define success and establish a sensible deadline.</v>
       </c>
       <c r="F105" t="str">
         <v>None</v>
       </c>
       <c r="G105" t="str">
-        <v>Weighted</v>
+        <v>Contextual</v>
       </c>
       <c r="H105" t="str">
-        <v>IDLE_WAIT</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I105" t="str">
         <v>Draft approved for MVP review</v>
@@ -10680,19 +10680,19 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>B11-R03</v>
+        <v>B11-R04</v>
       </c>
       <c r="B106" t="str">
         <v>B11</v>
       </c>
       <c r="C106" t="str">
-        <v>Fetch</v>
+        <v>Help</v>
       </c>
       <c r="D106" t="str">
-        <v>fetch</v>
+        <v>help me</v>
       </c>
       <c r="E106" t="str">
-        <v>Fetch what? Name the object, define success and establish a sensible deadline.</v>
+        <v>Help is a broad brief, but I have rescued worse.</v>
       </c>
       <c r="F106" t="str">
         <v>None</v>
@@ -10701,7 +10701,7 @@
         <v>Contextual</v>
       </c>
       <c r="H106" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I106" t="str">
         <v>Draft approved for MVP review</v>
@@ -10709,28 +10709,28 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>B11-R04</v>
+        <v>B11-R05</v>
       </c>
       <c r="B107" t="str">
         <v>B11</v>
       </c>
       <c r="C107" t="str">
-        <v>Help</v>
+        <v>Do something</v>
       </c>
       <c r="D107" t="str">
-        <v>help me</v>
+        <v>do something</v>
       </c>
       <c r="E107" t="str">
-        <v>Help is a broad brief, but I have rescued worse.</v>
+        <v>Do something. Inspirational management. No notes.</v>
       </c>
       <c r="F107" t="str">
         <v>None</v>
       </c>
       <c r="G107" t="str">
-        <v>Contextual</v>
+        <v>Weighted</v>
       </c>
       <c r="H107" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I107" t="str">
         <v>Draft approved for MVP review</v>
@@ -10738,28 +10738,28 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>B11-R05</v>
+        <v>B11-R06</v>
       </c>
       <c r="B108" t="str">
         <v>B11</v>
       </c>
       <c r="C108" t="str">
-        <v>Do something</v>
+        <v>Entertain me</v>
       </c>
       <c r="D108" t="str">
-        <v>do something</v>
+        <v>entertain me</v>
       </c>
       <c r="E108" t="str">
-        <v>Do something. Inspirational management. No notes.</v>
+        <v>I herd livestock, not expectations. Fortunately, I do have games.</v>
       </c>
       <c r="F108" t="str">
         <v>None</v>
       </c>
       <c r="G108" t="str">
-        <v>Weighted</v>
+        <v>Play</v>
       </c>
       <c r="H108" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>PLAY_BOW</v>
       </c>
       <c r="I108" t="str">
         <v>Draft approved for MVP review</v>
@@ -10767,28 +10767,28 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>B11-R06</v>
+        <v>B11-R07</v>
       </c>
       <c r="B109" t="str">
         <v>B11</v>
       </c>
       <c r="C109" t="str">
-        <v>Entertain me</v>
+        <v>Surprise me</v>
       </c>
       <c r="D109" t="str">
-        <v>entertain me</v>
+        <v>surprise me</v>
       </c>
       <c r="E109" t="str">
-        <v>I herd livestock, not expectations. Fortunately, I do have games.</v>
+        <v>Reckless delegation. I approve. I will choose something you have not already seen.</v>
       </c>
       <c r="F109" t="str">
-        <v>None</v>
+        <v>Session state</v>
       </c>
       <c r="G109" t="str">
-        <v>Play</v>
+        <v>Weighted unused destination</v>
       </c>
       <c r="H109" t="str">
-        <v>PLAY_BOW</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I109" t="str">
         <v>Draft approved for MVP review</v>
@@ -10796,28 +10796,28 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>B11-R07</v>
+        <v>B11-R08</v>
       </c>
       <c r="B110" t="str">
         <v>B11</v>
       </c>
       <c r="C110" t="str">
-        <v>Surprise me</v>
+        <v>Show me something</v>
       </c>
       <c r="D110" t="str">
-        <v>surprise me</v>
+        <v>show me</v>
       </c>
       <c r="E110" t="str">
-        <v>Reckless delegation. I approve. I will choose something you have not already seen.</v>
+        <v>At last, a verb. I have selected {{destination_name}}.</v>
       </c>
       <c r="F110" t="str">
-        <v>Session state</v>
+        <v>Destination library</v>
       </c>
       <c r="G110" t="str">
-        <v>Weighted unused destination</v>
+        <v>{{destination_id}}</v>
       </c>
       <c r="H110" t="str">
-        <v>EARS_UP</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I110" t="str">
         <v>Draft approved for MVP review</v>
@@ -10825,28 +10825,28 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>B11-R08</v>
+        <v>B11-R09</v>
       </c>
       <c r="B111" t="str">
         <v>B11</v>
       </c>
       <c r="C111" t="str">
-        <v>Show me something</v>
+        <v>Tell me something</v>
       </c>
       <c r="D111" t="str">
-        <v>show me</v>
+        <v>tell me something</v>
       </c>
       <c r="E111" t="str">
-        <v>At last, a verb. I have selected {{destination_name}}.</v>
+        <v>Precision is the courtesy intelligence pays to time. I will choose one useful fact this once.</v>
       </c>
       <c r="F111" t="str">
-        <v>Destination library</v>
+        <v>Knowledge library</v>
       </c>
       <c r="G111" t="str">
-        <v>{{destination_id}}</v>
+        <v>Learn</v>
       </c>
       <c r="H111" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I111" t="str">
         <v>Draft approved for MVP review</v>
@@ -10854,28 +10854,28 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>B11-R09</v>
+        <v>B11-R10</v>
       </c>
       <c r="B112" t="str">
         <v>B11</v>
       </c>
       <c r="C112" t="str">
-        <v>Tell me something</v>
+        <v>Take me somewhere</v>
       </c>
       <c r="D112" t="str">
-        <v>tell me something</v>
+        <v>take me somewhere</v>
       </c>
       <c r="E112" t="str">
-        <v>Precision is the courtesy intelligence pays to time. I will choose one useful fact this once.</v>
+        <v>Movement, purpose and direction. Now we are speaking professionally.</v>
       </c>
       <c r="F112" t="str">
-        <v>Knowledge library</v>
+        <v>Destination library</v>
       </c>
       <c r="G112" t="str">
-        <v>Learn</v>
+        <v>Weighted unused destination</v>
       </c>
       <c r="H112" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I112" t="str">
         <v>Draft approved for MVP review</v>
@@ -10883,28 +10883,28 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>B11-R10</v>
+        <v>B12-R01</v>
       </c>
       <c r="B113" t="str">
-        <v>B11</v>
+        <v>B12</v>
       </c>
       <c r="C113" t="str">
-        <v>Take me somewhere</v>
+        <v>Owns a dog</v>
       </c>
       <c r="D113" t="str">
-        <v>take me somewhere</v>
+        <v>I have a Labrador; my dog</v>
       </c>
       <c r="E113" t="str">
-        <v>Movement, purpose and direction. Now we are speaking professionally.</v>
+        <v>A {{mentioned_breed}}. Useful information. Let us see whether the pack has one matching your description.</v>
       </c>
       <c r="F113" t="str">
-        <v>Destination library</v>
+        <v>Dog database</v>
       </c>
       <c r="G113" t="str">
-        <v>Weighted unused destination</v>
+        <v>Know Your Chum</v>
       </c>
       <c r="H113" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I113" t="str">
         <v>Draft approved for MVP review</v>
@@ -10912,28 +10912,28 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>B12-R01</v>
+        <v>B12-R02</v>
       </c>
       <c r="B114" t="str">
         <v>B12</v>
       </c>
       <c r="C114" t="str">
-        <v>Owns a dog</v>
+        <v>Dog name</v>
       </c>
       <c r="D114" t="str">
-        <v>I have a Labrador; my dog</v>
+        <v>my dog is called</v>
       </c>
       <c r="E114" t="str">
-        <v>A {{mentioned_breed}}. Useful information. Let us see whether the pack has one matching your description.</v>
+        <v>{{dog_name}} has entered the records. Strong name. Context pending.</v>
       </c>
       <c r="F114" t="str">
-        <v>Dog database</v>
+        <v>Session context</v>
       </c>
       <c r="G114" t="str">
-        <v>Know Your Chum</v>
+        <v>Dog Name Generator or Know Your Chum</v>
       </c>
       <c r="H114" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I114" t="str">
         <v>Draft approved for MVP review</v>
@@ -10941,28 +10941,28 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>B12-R02</v>
+        <v>B12-R03</v>
       </c>
       <c r="B115" t="str">
         <v>B12</v>
       </c>
       <c r="C115" t="str">
-        <v>Dog name</v>
+        <v>Likes dogs</v>
       </c>
       <c r="D115" t="str">
-        <v>my dog is called</v>
+        <v>I like dogs; love dogs</v>
       </c>
       <c r="E115" t="str">
-        <v>{{dog_name}} has entered the records. Strong name. Context pending.</v>
+        <v>Sound judgement. I have 54 in the pack and up to 150 in the history operation.</v>
       </c>
       <c r="F115" t="str">
-        <v>Session context</v>
+        <v>Destination library</v>
       </c>
       <c r="G115" t="str">
-        <v>Dog Name Generator or Know Your Chum</v>
+        <v>Know Your Chum or Britain's Dog History</v>
       </c>
       <c r="H115" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I115" t="str">
         <v>Draft approved for MVP review</v>
@@ -10970,28 +10970,28 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>B12-R03</v>
+        <v>B12-R04</v>
       </c>
       <c r="B116" t="str">
         <v>B12</v>
       </c>
       <c r="C116" t="str">
-        <v>Likes dogs</v>
+        <v>Bored</v>
       </c>
       <c r="D116" t="str">
-        <v>I like dogs; love dogs</v>
+        <v>I am bored</v>
       </c>
       <c r="E116" t="str">
-        <v>Sound judgement. I have 54 in the pack and up to 150 in the history operation.</v>
+        <v>Boredom is unused working capacity. We will convert it into a game.</v>
       </c>
       <c r="F116" t="str">
-        <v>Destination library</v>
+        <v>None</v>
       </c>
       <c r="G116" t="str">
-        <v>Know Your Chum or Britain's Dog History</v>
+        <v>Play</v>
       </c>
       <c r="H116" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>PLAY_BOW</v>
       </c>
       <c r="I116" t="str">
         <v>Draft approved for MVP review</v>
@@ -10999,28 +10999,28 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>B12-R04</v>
+        <v>B12-R05</v>
       </c>
       <c r="B117" t="str">
         <v>B12</v>
       </c>
       <c r="C117" t="str">
-        <v>Bored</v>
+        <v>Sad</v>
       </c>
       <c r="D117" t="str">
-        <v>I am bored</v>
+        <v>I am sad; unhappy</v>
       </c>
       <c r="E117" t="str">
-        <v>Boredom is unused working capacity. We will convert it into a game.</v>
+        <v>I am sorry you are feeling low. We will keep this gentle and choose something light.</v>
       </c>
       <c r="F117" t="str">
-        <v>None</v>
+        <v>Safety / tone rules</v>
       </c>
       <c r="G117" t="str">
-        <v>Play</v>
+        <v>Gentle Play or Learn</v>
       </c>
       <c r="H117" t="str">
-        <v>PLAY_BOW</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I117" t="str">
         <v>Draft approved for MVP review</v>
@@ -11028,28 +11028,28 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>B12-R05</v>
+        <v>B12-R06</v>
       </c>
       <c r="B118" t="str">
         <v>B12</v>
       </c>
       <c r="C118" t="str">
-        <v>Sad</v>
+        <v>Angry</v>
       </c>
       <c r="D118" t="str">
-        <v>I am sad; unhappy</v>
+        <v>I am angry; annoyed</v>
       </c>
       <c r="E118" t="str">
-        <v>I am sorry you are feeling low. We will keep this gentle and choose something light.</v>
+        <v>Aye, you sound wound up. We will reduce the variables and choose one simple thing.</v>
       </c>
       <c r="F118" t="str">
-        <v>Safety / tone rules</v>
+        <v>Tone rules</v>
       </c>
       <c r="G118" t="str">
-        <v>Gentle Play or Learn</v>
+        <v>Contextual</v>
       </c>
       <c r="H118" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>SHAKE_RESET</v>
       </c>
       <c r="I118" t="str">
         <v>Draft approved for MVP review</v>
@@ -11057,28 +11057,28 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>B12-R06</v>
+        <v>B12-R07</v>
       </c>
       <c r="B119" t="str">
         <v>B12</v>
       </c>
       <c r="C119" t="str">
-        <v>Angry</v>
+        <v>Praise</v>
       </c>
       <c r="D119" t="str">
-        <v>I am angry; annoyed</v>
+        <v>good dog; clever</v>
       </c>
       <c r="E119" t="str">
-        <v>Aye, you sound wound up. We will reduce the variables and choose one simple thing.</v>
+        <v>Clever? Aye. Let us not reduce a measurable fact to flattery.</v>
       </c>
       <c r="F119" t="str">
-        <v>Tone rules</v>
+        <v>None</v>
       </c>
       <c r="G119" t="str">
-        <v>Contextual</v>
+        <v>Weighted</v>
       </c>
       <c r="H119" t="str">
-        <v>SHAKE_RESET</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I119" t="str">
         <v>Draft approved for MVP review</v>
@@ -11086,19 +11086,19 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>B12-R07</v>
+        <v>B12-R08</v>
       </c>
       <c r="B120" t="str">
         <v>B12</v>
       </c>
       <c r="C120" t="str">
-        <v>Praise</v>
+        <v>Affection</v>
       </c>
       <c r="D120" t="str">
-        <v>good dog; clever</v>
+        <v>I love you</v>
       </c>
       <c r="E120" t="str">
-        <v>Clever? Aye. Let us not reduce a measurable fact to flattery.</v>
+        <v>Affection acknowledged. Boundaries maintained. Task still required.</v>
       </c>
       <c r="F120" t="str">
         <v>None</v>
@@ -11107,7 +11107,7 @@
         <v>Weighted</v>
       </c>
       <c r="H120" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I120" t="str">
         <v>Draft approved for MVP review</v>
@@ -11115,28 +11115,28 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>B12-R08</v>
+        <v>B12-R09</v>
       </c>
       <c r="B121" t="str">
         <v>B12</v>
       </c>
       <c r="C121" t="str">
-        <v>Affection</v>
+        <v>Insult</v>
       </c>
       <c r="D121" t="str">
-        <v>I love you</v>
+        <v>stupid; annoying</v>
       </c>
       <c r="E121" t="str">
-        <v>Affection acknowledged. Boundaries maintained. Task still required.</v>
+        <v>An interesting assessment from someone who selected a dog and then argued with it.</v>
       </c>
       <c r="F121" t="str">
-        <v>None</v>
+        <v>Moderation rules</v>
       </c>
       <c r="G121" t="str">
-        <v>Weighted</v>
+        <v>Weighted or close</v>
       </c>
       <c r="H121" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>LOOK_AWAY</v>
       </c>
       <c r="I121" t="str">
         <v>Draft approved for MVP review</v>
@@ -11144,28 +11144,28 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>B12-R09</v>
+        <v>B12-R10</v>
       </c>
       <c r="B122" t="str">
         <v>B12</v>
       </c>
       <c r="C122" t="str">
-        <v>Insult</v>
+        <v>Thanks</v>
       </c>
       <c r="D122" t="str">
-        <v>stupid; annoying</v>
+        <v>thank you; cheers</v>
       </c>
       <c r="E122" t="str">
-        <v>An interesting assessment from someone who selected a dog and then argued with it.</v>
+        <v>You are welcome. Efficient gratitude. I respect it.</v>
       </c>
       <c r="F122" t="str">
-        <v>Moderation rules</v>
+        <v>None</v>
       </c>
       <c r="G122" t="str">
-        <v>Weighted or close</v>
+        <v>Contextual</v>
       </c>
       <c r="H122" t="str">
-        <v>LOOK_AWAY</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I122" t="str">
         <v>Draft approved for MVP review</v>
@@ -11173,28 +11173,28 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>B12-R10</v>
+        <v>B13-R01</v>
       </c>
       <c r="B123" t="str">
-        <v>B12</v>
+        <v>B13</v>
       </c>
       <c r="C123" t="str">
-        <v>Thanks</v>
+        <v>Generic noun</v>
       </c>
       <c r="D123" t="str">
-        <v>thank you; cheers</v>
+        <v>recognised noun</v>
       </c>
       <c r="E123" t="str">
-        <v>You are welcome. Efficient gratitude. I respect it.</v>
+        <v>{{input}}. A noun. Excellent. We have identified a thing, but not why you brought it.</v>
       </c>
       <c r="F123" t="str">
-        <v>None</v>
+        <v>Dictionary / normaliser</v>
       </c>
       <c r="G123" t="str">
-        <v>Contextual</v>
+        <v>Weighted</v>
       </c>
       <c r="H123" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I123" t="str">
         <v>Draft approved for MVP review</v>
@@ -11202,19 +11202,19 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>B13-R01</v>
+        <v>B13-R02</v>
       </c>
       <c r="B124" t="str">
         <v>B13</v>
       </c>
       <c r="C124" t="str">
-        <v>Generic noun</v>
+        <v>Missing verb</v>
       </c>
       <c r="D124" t="str">
-        <v>recognised noun</v>
+        <v>single object</v>
       </c>
       <c r="E124" t="str">
-        <v>{{input}}. A noun. Excellent. We have identified a thing, but not why you brought it.</v>
+        <v>I know what {{input}} means. I am waiting for the verb.</v>
       </c>
       <c r="F124" t="str">
         <v>Dictionary / normaliser</v>
@@ -11231,19 +11231,19 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>B13-R02</v>
+        <v>B13-R03</v>
       </c>
       <c r="B125" t="str">
         <v>B13</v>
       </c>
       <c r="C125" t="str">
-        <v>Missing verb</v>
+        <v>Unexplained object</v>
       </c>
       <c r="D125" t="str">
-        <v>single object</v>
+        <v>object without context</v>
       </c>
       <c r="E125" t="str">
-        <v>I know what {{input}} means. I am waiting for the verb.</v>
+        <v>You have presented {{input}} as though it explains itself. Very human.</v>
       </c>
       <c r="F125" t="str">
         <v>Dictionary / normaliser</v>
@@ -11252,7 +11252,7 @@
         <v>Weighted</v>
       </c>
       <c r="H125" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I125" t="str">
         <v>Draft approved for MVP review</v>
@@ -11260,28 +11260,28 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>B13-R03</v>
+        <v>B13-R04</v>
       </c>
       <c r="B126" t="str">
         <v>B13</v>
       </c>
       <c r="C126" t="str">
-        <v>Unexplained object</v>
+        <v>Task toy evidence</v>
       </c>
       <c r="D126" t="str">
-        <v>object without context</v>
+        <v>random noun</v>
       </c>
       <c r="E126" t="str">
-        <v>You have presented {{input}} as though it explains itself. Very human.</v>
+        <v>{{input}}. Is it a task, a toy or evidence?</v>
       </c>
       <c r="F126" t="str">
         <v>Dictionary / normaliser</v>
       </c>
       <c r="G126" t="str">
-        <v>Weighted</v>
+        <v>Contextual</v>
       </c>
       <c r="H126" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>SNIFF_CHECK</v>
       </c>
       <c r="I126" t="str">
         <v>Draft approved for MVP review</v>
@@ -11289,25 +11289,25 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>B13-R04</v>
+        <v>B13-R05</v>
       </c>
       <c r="B127" t="str">
         <v>B13</v>
       </c>
       <c r="C127" t="str">
-        <v>Task toy evidence</v>
+        <v>Filed noun</v>
       </c>
       <c r="D127" t="str">
         <v>random noun</v>
       </c>
       <c r="E127" t="str">
-        <v>{{input}}. Is it a task, a toy or evidence?</v>
+        <v>Aye, {{input}}. Filed under things the human may eventually explain.</v>
       </c>
       <c r="F127" t="str">
         <v>Dictionary / normaliser</v>
       </c>
       <c r="G127" t="str">
-        <v>Contextual</v>
+        <v>Weighted</v>
       </c>
       <c r="H127" t="str">
         <v>SNIFF_CHECK</v>
@@ -11318,19 +11318,19 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>B13-R05</v>
+        <v>B13-R06</v>
       </c>
       <c r="B128" t="str">
         <v>B13</v>
       </c>
       <c r="C128" t="str">
-        <v>Filed noun</v>
+        <v>Context request</v>
       </c>
       <c r="D128" t="str">
         <v>random noun</v>
       </c>
       <c r="E128" t="str">
-        <v>Aye, {{input}}. Filed under things the human may eventually explain.</v>
+        <v>I can work with {{input}}, but even genius benefits from context.</v>
       </c>
       <c r="F128" t="str">
         <v>Dictionary / normaliser</v>
@@ -11339,7 +11339,7 @@
         <v>Weighted</v>
       </c>
       <c r="H128" t="str">
-        <v>SNIFF_CHECK</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I128" t="str">
         <v>Draft approved for MVP review</v>
@@ -11347,19 +11347,19 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>B13-R06</v>
+        <v>B13-R07</v>
       </c>
       <c r="B129" t="str">
         <v>B13</v>
       </c>
       <c r="C129" t="str">
-        <v>Context request</v>
+        <v>Progress joke</v>
       </c>
       <c r="D129" t="str">
         <v>random noun</v>
       </c>
       <c r="E129" t="str">
-        <v>I can work with {{input}}, but even genius benefits from context.</v>
+        <v>You have named an object. That is technically progress.</v>
       </c>
       <c r="F129" t="str">
         <v>Dictionary / normaliser</v>
@@ -11368,7 +11368,7 @@
         <v>Weighted</v>
       </c>
       <c r="H129" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>POSITIVE_RESPONSE</v>
       </c>
       <c r="I129" t="str">
         <v>Draft approved for MVP review</v>
@@ -11376,19 +11376,19 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>B13-R07</v>
+        <v>B13-R08</v>
       </c>
       <c r="B130" t="str">
         <v>B13</v>
       </c>
       <c r="C130" t="str">
-        <v>Progress joke</v>
+        <v>Outshone</v>
       </c>
       <c r="D130" t="str">
         <v>random noun</v>
       </c>
       <c r="E130" t="str">
-        <v>You have named an object. That is technically progress.</v>
+        <v>{{input}} has entered the conversation and contributed nothing. Do not let it outshine you.</v>
       </c>
       <c r="F130" t="str">
         <v>Dictionary / normaliser</v>
@@ -11397,7 +11397,7 @@
         <v>Weighted</v>
       </c>
       <c r="H130" t="str">
-        <v>POSITIVE_RESPONSE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I130" t="str">
         <v>Draft approved for MVP review</v>
@@ -11405,19 +11405,19 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>B13-R08</v>
+        <v>B13-R09</v>
       </c>
       <c r="B131" t="str">
         <v>B13</v>
       </c>
       <c r="C131" t="str">
-        <v>Outshone</v>
+        <v>Committee joke</v>
       </c>
       <c r="D131" t="str">
         <v>random noun</v>
       </c>
       <c r="E131" t="str">
-        <v>{{input}} has entered the conversation and contributed nothing. Do not let it outshine you.</v>
+        <v>Right. We have {{input}} and no plan. This is how committees begin.</v>
       </c>
       <c r="F131" t="str">
         <v>Dictionary / normaliser</v>
@@ -11426,7 +11426,7 @@
         <v>Weighted</v>
       </c>
       <c r="H131" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I131" t="str">
         <v>Draft approved for MVP review</v>
@@ -11434,19 +11434,19 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>B13-R09</v>
+        <v>B13-R10</v>
       </c>
       <c r="B132" t="str">
         <v>B13</v>
       </c>
       <c r="C132" t="str">
-        <v>Committee joke</v>
+        <v>Noun pen</v>
       </c>
       <c r="D132" t="str">
         <v>random noun</v>
       </c>
       <c r="E132" t="str">
-        <v>Right. We have {{input}} and no plan. This is how committees begin.</v>
+        <v>I have herded {{input}} into the noun pen. It can stay there until we find a purpose.</v>
       </c>
       <c r="F132" t="str">
         <v>Dictionary / normaliser</v>
@@ -11455,7 +11455,7 @@
         <v>Weighted</v>
       </c>
       <c r="H132" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>SNIFF_CHECK</v>
       </c>
       <c r="I132" t="str">
         <v>Draft approved for MVP review</v>
@@ -11463,28 +11463,28 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>B13-R10</v>
+        <v>B14-R01</v>
       </c>
       <c r="B133" t="str">
-        <v>B13</v>
+        <v>B14</v>
       </c>
       <c r="C133" t="str">
-        <v>Noun pen</v>
+        <v>Keyboard lean</v>
       </c>
       <c r="D133" t="str">
-        <v>random noun</v>
+        <v>qwerty; asdfgh</v>
       </c>
       <c r="E133" t="str">
-        <v>I have herded {{input}} into the noun pen. It can stay there until we find a purpose.</v>
+        <v>Did you lean on your keyboard?</v>
       </c>
       <c r="F133" t="str">
-        <v>Dictionary / normaliser</v>
+        <v>Pattern detector</v>
       </c>
       <c r="G133" t="str">
         <v>Weighted</v>
       </c>
       <c r="H133" t="str">
-        <v>SNIFF_CHECK</v>
+        <v>HEAD_TILT_DOUBLE</v>
       </c>
       <c r="I133" t="str">
         <v>Draft approved for MVP review</v>
@@ -11492,19 +11492,19 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>B14-R01</v>
+        <v>B14-R02</v>
       </c>
       <c r="B134" t="str">
         <v>B14</v>
       </c>
       <c r="C134" t="str">
-        <v>Keyboard lean</v>
+        <v>Minor collision</v>
       </c>
       <c r="D134" t="str">
-        <v>qwerty; asdfgh</v>
+        <v>keyboard smash</v>
       </c>
       <c r="E134" t="str">
-        <v>Did you lean on your keyboard?</v>
+        <v>Aye. That looked less like typing and more like a minor collision.</v>
       </c>
       <c r="F134" t="str">
         <v>Pattern detector</v>
@@ -11521,19 +11521,19 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>B14-R02</v>
+        <v>B14-R03</v>
       </c>
       <c r="B135" t="str">
         <v>B14</v>
       </c>
       <c r="C135" t="str">
-        <v>Minor collision</v>
+        <v>Qwerty</v>
       </c>
       <c r="D135" t="str">
-        <v>keyboard smash</v>
+        <v>qwerty</v>
       </c>
       <c r="E135" t="str">
-        <v>Aye. That looked less like typing and more like a minor collision.</v>
+        <v>Qwerty. The internationally recognised sound of a human testing a box.</v>
       </c>
       <c r="F135" t="str">
         <v>Pattern detector</v>
@@ -11542,7 +11542,7 @@
         <v>Weighted</v>
       </c>
       <c r="H135" t="str">
-        <v>HEAD_TILT_DOUBLE</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I135" t="str">
         <v>Draft approved for MVP review</v>
@@ -11550,19 +11550,19 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>B14-R03</v>
+        <v>B14-R04</v>
       </c>
       <c r="B136" t="str">
         <v>B14</v>
       </c>
       <c r="C136" t="str">
-        <v>Qwerty</v>
+        <v>Fingers before brain</v>
       </c>
       <c r="D136" t="str">
-        <v>qwerty</v>
+        <v>unknown letters</v>
       </c>
       <c r="E136" t="str">
-        <v>Qwerty. The internationally recognised sound of a human testing a box.</v>
+        <v>Your fingers appear to have arrived before your brain.</v>
       </c>
       <c r="F136" t="str">
         <v>Pattern detector</v>
@@ -11571,7 +11571,7 @@
         <v>Weighted</v>
       </c>
       <c r="H136" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_DOUBLE</v>
       </c>
       <c r="I136" t="str">
         <v>Draft approved for MVP review</v>
@@ -11579,19 +11579,19 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>B14-R04</v>
+        <v>B14-R05</v>
       </c>
       <c r="B137" t="str">
         <v>B14</v>
       </c>
       <c r="C137" t="str">
-        <v>Fingers before brain</v>
+        <v>Not a word</v>
       </c>
       <c r="D137" t="str">
-        <v>unknown letters</v>
+        <v>unknown string</v>
       </c>
       <c r="E137" t="str">
-        <v>Your fingers appear to have arrived before your brain.</v>
+        <v>I have checked it twice. Still not a word.</v>
       </c>
       <c r="F137" t="str">
         <v>Pattern detector</v>
@@ -11608,19 +11608,19 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>B14-R05</v>
+        <v>B14-R06</v>
       </c>
       <c r="B138" t="str">
         <v>B14</v>
       </c>
       <c r="C138" t="str">
-        <v>Not a word</v>
+        <v>Elbow code</v>
       </c>
       <c r="D138" t="str">
-        <v>unknown string</v>
+        <v>symbols; smash</v>
       </c>
       <c r="E138" t="str">
-        <v>I have checked it twice. Still not a word.</v>
+        <v>Either that is code, or your elbow has opinions.</v>
       </c>
       <c r="F138" t="str">
         <v>Pattern detector</v>
@@ -11629,7 +11629,7 @@
         <v>Weighted</v>
       </c>
       <c r="H138" t="str">
-        <v>HEAD_TILT_DOUBLE</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I138" t="str">
         <v>Draft approved for MVP review</v>
@@ -11637,19 +11637,19 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>B14-R06</v>
+        <v>B14-R07</v>
       </c>
       <c r="B139" t="str">
         <v>B14</v>
       </c>
       <c r="C139" t="str">
-        <v>Elbow code</v>
+        <v>Keyboard turn</v>
       </c>
       <c r="D139" t="str">
-        <v>symbols; smash</v>
+        <v>random symbols</v>
       </c>
       <c r="E139" t="str">
-        <v>Either that is code, or your elbow has opinions.</v>
+        <v>The keyboard has made its contribution. Your turn.</v>
       </c>
       <c r="F139" t="str">
         <v>Pattern detector</v>
@@ -11658,7 +11658,7 @@
         <v>Weighted</v>
       </c>
       <c r="H139" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>HEAD_TILT_SMALL</v>
       </c>
       <c r="I139" t="str">
         <v>Draft approved for MVP review</v>
@@ -11666,19 +11666,19 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>B14-R07</v>
+        <v>B14-R08</v>
       </c>
       <c r="B140" t="str">
         <v>B14</v>
       </c>
       <c r="C140" t="str">
-        <v>Keyboard turn</v>
+        <v>No plan</v>
       </c>
       <c r="D140" t="str">
-        <v>random symbols</v>
+        <v>letters without meaning</v>
       </c>
       <c r="E140" t="str">
-        <v>The keyboard has made its contribution. Your turn.</v>
+        <v>That message contains several letters and no detectable plan.</v>
       </c>
       <c r="F140" t="str">
         <v>Pattern detector</v>
@@ -11687,7 +11687,7 @@
         <v>Weighted</v>
       </c>
       <c r="H140" t="str">
-        <v>HEAD_TILT_SMALL</v>
+        <v>HEAD_TILT_MEDIUM</v>
       </c>
       <c r="I140" t="str">
         <v>Draft approved for MVP review</v>
@@ -11695,19 +11695,19 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>B14-R08</v>
+        <v>B14-R09</v>
       </c>
       <c r="B141" t="str">
         <v>B14</v>
       </c>
       <c r="C141" t="str">
-        <v>No plan</v>
+        <v>Consonants</v>
       </c>
       <c r="D141" t="str">
-        <v>letters without meaning</v>
+        <v>no vowels</v>
       </c>
       <c r="E141" t="str">
-        <v>That message contains several letters and no detectable plan.</v>
+        <v>I can herd sheep. Consonants require your cooperation.</v>
       </c>
       <c r="F141" t="str">
         <v>Pattern detector</v>
@@ -11716,7 +11716,7 @@
         <v>Weighted</v>
       </c>
       <c r="H141" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
+        <v>HEAD_TILT_DOUBLE</v>
       </c>
       <c r="I141" t="str">
         <v>Draft approved for MVP review</v>
@@ -11724,19 +11724,19 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>B14-R09</v>
+        <v>B14-R10</v>
       </c>
       <c r="B142" t="str">
         <v>B14</v>
       </c>
       <c r="C142" t="str">
-        <v>Consonants</v>
+        <v>Warm up</v>
       </c>
       <c r="D142" t="str">
-        <v>no vowels</v>
+        <v>minimal input</v>
       </c>
       <c r="E142" t="str">
-        <v>I can herd sheep. Consonants require your cooperation.</v>
+        <v>Reet, we will call that the warm-up.</v>
       </c>
       <c r="F142" t="str">
         <v>Pattern detector</v>
@@ -11745,7 +11745,7 @@
         <v>Weighted</v>
       </c>
       <c r="H142" t="str">
-        <v>HEAD_TILT_DOUBLE</v>
+        <v>SHAKE_RESET</v>
       </c>
       <c r="I142" t="str">
         <v>Draft approved for MVP review</v>
@@ -11753,36 +11753,36 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>B14-R10</v>
+        <v>B15-R01-v1</v>
       </c>
       <c r="B143" t="str">
-        <v>B14</v>
+        <v>B15</v>
       </c>
       <c r="C143" t="str">
-        <v>Warm up</v>
+        <v>What is this / where do I start</v>
       </c>
       <c r="D143" t="str">
-        <v>minimal input</v>
+        <v>What is this for?; What do I do here?; How do I get started?; Is this the start?</v>
       </c>
       <c r="E143" t="str">
-        <v>Reet, we will call that the warm-up.</v>
+        <v>Aye, this is where you talk to a dog and see what happens. Type whatever brought you here, even if it is only a question about what this is, and I will get us moving.</v>
       </c>
       <c r="F143" t="str">
-        <v>Pattern detector</v>
+        <v>Orientation (onboarding)</v>
       </c>
       <c r="G143" t="str">
-        <v>Weighted</v>
+        <v/>
       </c>
       <c r="H143" t="str">
-        <v>SHAKE_RESET</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I143" t="str">
-        <v>Draft approved for MVP review</v>
+        <v>Approved copy v2</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>B15-R01-v1</v>
+        <v>B15-R01-v2</v>
       </c>
       <c r="B144" t="str">
         <v>B15</v>
@@ -11791,10 +11791,10 @@
         <v>What is this / where do I start</v>
       </c>
       <c r="D144" t="str">
-        <v>What is this for?; What do I do here?; How do I get started?; Is this the start?</v>
+        <v/>
       </c>
       <c r="E144" t="str">
-        <v>Aye, this is where you talk to a dog and see what happens. Type whatever brought you here, even if it is only a question about what this is, and I will get us moving.</v>
+        <v>You have found the part where the dog waits and the human supplies the problem. Say what is on your mind, our kid. I will work out where it belongs.</v>
       </c>
       <c r="F144" t="str">
         <v>Orientation (onboarding)</v>
@@ -11811,7 +11811,7 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>B15-R01-v2</v>
+        <v>B15-R01-v3</v>
       </c>
       <c r="B145" t="str">
         <v>B15</v>
@@ -11823,7 +11823,7 @@
         <v/>
       </c>
       <c r="E145" t="str">
-        <v>You have found the part where the dog waits and the human supplies the problem. Say what is on your mind, our kid. I will work out where it belongs.</v>
+        <v>This is a conversation, not an instruction manual. You type something, I consider whether it is sensible, then we proceed from there. You have already completed the difficult bit by arriving.</v>
       </c>
       <c r="F145" t="str">
         <v>Orientation (onboarding)</v>
@@ -11840,19 +11840,19 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>B15-R01-v3</v>
+        <v>B15-R02-v1</v>
       </c>
       <c r="B146" t="str">
         <v>B15</v>
       </c>
       <c r="C146" t="str">
-        <v>What is this / where do I start</v>
+        <v>What can I ask / options</v>
       </c>
       <c r="D146" t="str">
-        <v/>
+        <v>What can I ask?; What are my options?; What kind of things can you answer?; Can you give me some choices?</v>
       </c>
       <c r="E146" t="str">
-        <v>This is a conversation, not an instruction manual. You type something, I consider whether it is sensible, then we proceed from there. You have already completed the difficult bit by arriving.</v>
+        <v>Aye, ask whatever brought you here. I know this place, the game and rather more about dogs than is strictly necessary. If the question belongs elsewhere, I will fetch the appropriate operator.</v>
       </c>
       <c r="F146" t="str">
         <v>Orientation (onboarding)</v>
@@ -11869,7 +11869,7 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>B15-R02-v1</v>
+        <v>B15-R02-v2</v>
       </c>
       <c r="B147" t="str">
         <v>B15</v>
@@ -11878,10 +11878,10 @@
         <v>What can I ask / options</v>
       </c>
       <c r="D147" t="str">
-        <v>What can I ask?; What are my options?; What kind of things can you answer?; Can you give me some choices?</v>
+        <v/>
       </c>
       <c r="E147" t="str">
-        <v>Aye, ask whatever brought you here. I know this place, the game and rather more about dogs than is strictly necessary. If the question belongs elsewhere, I will fetch the appropriate operator.</v>
+        <v>You can ask naturally. I can explain what we have built, find things around the site, settle a dog question or occasionally improve the atmosphere. Start anywhere useful.</v>
       </c>
       <c r="F147" t="str">
         <v>Orientation (onboarding)</v>
@@ -11898,7 +11898,7 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>B15-R02-v2</v>
+        <v>B15-R02-v3</v>
       </c>
       <c r="B148" t="str">
         <v>B15</v>
@@ -11910,7 +11910,7 @@
         <v/>
       </c>
       <c r="E148" t="str">
-        <v>You can ask naturally. I can explain what we have built, find things around the site, settle a dog question or occasionally improve the atmosphere. Start anywhere useful.</v>
+        <v>Most sensible questions are within reach, and several daft ones besides. Tell me what you are after. I will either deal with it or locate a colleague with the relevant limitations.</v>
       </c>
       <c r="F148" t="str">
         <v>Orientation (onboarding)</v>
@@ -11927,19 +11927,19 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>B15-R02-v3</v>
+        <v>B15-R03-v1</v>
       </c>
       <c r="B149" t="str">
         <v>B15</v>
       </c>
       <c r="C149" t="str">
-        <v>What can I ask / options</v>
+        <v>How does this work / instructions</v>
       </c>
       <c r="D149" t="str">
-        <v/>
+        <v>How do I use this?; Are there any instructions?; Do I just type anything?; Can you tell me how this works?</v>
       </c>
       <c r="E149" t="str">
-        <v>Most sensible questions are within reach, and several daft ones besides. Tell me what you are after. I will either deal with it or locate a colleague with the relevant limitations.</v>
+        <v>There are no instructions, our kid. Type as you normally would and I will make sense of it. The empty box is not a test, although your first message may become one.</v>
       </c>
       <c r="F149" t="str">
         <v>Orientation (onboarding)</v>
@@ -11956,7 +11956,7 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>B15-R03-v1</v>
+        <v>B15-R03-v2</v>
       </c>
       <c r="B150" t="str">
         <v>B15</v>
@@ -11965,10 +11965,10 @@
         <v>How does this work / instructions</v>
       </c>
       <c r="D150" t="str">
-        <v>How do I use this?; Are there any instructions?; Do I just type anything?; Can you tell me how this works?</v>
+        <v/>
       </c>
       <c r="E150" t="str">
-        <v>There are no instructions, our kid. Type as you normally would and I will make sense of it. The empty box is not a test, although your first message may become one.</v>
+        <v>Aye, you just type. A question, a thought or whatever your fingers produce first will do. I will sort it into something useful from there.</v>
       </c>
       <c r="F150" t="str">
         <v>Orientation (onboarding)</v>
@@ -11985,7 +11985,7 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>B15-R03-v2</v>
+        <v>B15-R03-v3</v>
       </c>
       <c r="B151" t="str">
         <v>B15</v>
@@ -11997,7 +11997,7 @@
         <v/>
       </c>
       <c r="E151" t="str">
-        <v>Aye, you just type. A question, a thought or whatever your fingers produce first will do. I will sort it into something useful from there.</v>
+        <v>You are using it correctly already. Put ordinary words in the box, send them, and leave the organising to me. That is why I am the working one.</v>
       </c>
       <c r="F151" t="str">
         <v>Orientation (onboarding)</v>
@@ -12014,19 +12014,19 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>B15-R03-v3</v>
+        <v>B15-R04-v1</v>
       </c>
       <c r="B152" t="str">
         <v>B15</v>
       </c>
       <c r="C152" t="str">
-        <v>How does this work / instructions</v>
+        <v>Nudge to begin / what next</v>
       </c>
       <c r="D152" t="str">
-        <v/>
+        <v>What happens next?; What do we do now?; Are you waiting for me?; So, what do I do with you?</v>
       </c>
       <c r="E152" t="str">
-        <v>You are using it correctly already. Put ordinary words in the box, send them, and leave the organising to me. That is why I am the working one.</v>
+        <v>I am waiting, yes. This arrangement improves considerably when the human contributes a proper question. Go on, our kid. Give me something worth organising.</v>
       </c>
       <c r="F152" t="str">
         <v>Orientation (onboarding)</v>
@@ -12043,7 +12043,7 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>B15-R04-v1</v>
+        <v>B15-R04-v2</v>
       </c>
       <c r="B153" t="str">
         <v>B15</v>
@@ -12052,10 +12052,10 @@
         <v>Nudge to begin / what next</v>
       </c>
       <c r="D153" t="str">
-        <v>What happens next?; What do we do now?; Are you waiting for me?; So, what do I do with you?</v>
+        <v/>
       </c>
       <c r="E153" t="str">
-        <v>I am waiting, yes. This arrangement improves considerably when the human contributes a proper question. Go on, our kid. Give me something worth organising.</v>
+        <v>The next bit is yours. Say what brought you here and I will take it from there. Standing around waiting is rarely improved by doing more of it.</v>
       </c>
       <c r="F153" t="str">
         <v>Orientation (onboarding)</v>
@@ -12072,7 +12072,7 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>B15-R04-v2</v>
+        <v>B15-R04-v3</v>
       </c>
       <c r="B154" t="str">
         <v>B15</v>
@@ -12084,7 +12084,7 @@
         <v/>
       </c>
       <c r="E154" t="str">
-        <v>The next bit is yours. Say what brought you here and I will take it from there. Standing around waiting is rarely improved by doing more of it.</v>
+        <v>Aye, I am waiting for you. I could begin without a brief, but that is how humans end up with meetings. Type the question and let us get on.</v>
       </c>
       <c r="F154" t="str">
         <v>Orientation (onboarding)</v>
@@ -12101,28 +12101,28 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>B15-R04-v3</v>
+        <v>SCP-F01-v1</v>
       </c>
       <c r="B155" t="str">
-        <v>B15</v>
+        <v>B16</v>
       </c>
       <c r="C155" t="str">
-        <v>Nudge to begin / what next</v>
+        <v>How can a dog type</v>
       </c>
       <c r="D155" t="str">
-        <v/>
+        <v>How can a dog type?; Is that really your face?; Do you really know what I typed?</v>
       </c>
       <c r="E155" t="str">
-        <v>Aye, I am waiting for you. I could begin without a brief, but that is how humans end up with meetings. Type the question and let us get on.</v>
+        <v>I do not type, our kid. A person wrote every line in advance, and the game matches your message to the right one. I merely provide the judgement and the face.</v>
       </c>
       <c r="F155" t="str">
-        <v>Orientation (onboarding)</v>
+        <v>Identity (scepticism)</v>
       </c>
       <c r="G155" t="str">
         <v/>
       </c>
       <c r="H155" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT</v>
       </c>
       <c r="I155" t="str">
         <v>Approved copy v2</v>
@@ -12130,7 +12130,7 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>SCP-F01-v1</v>
+        <v>SCP-F01-v2</v>
       </c>
       <c r="B156" t="str">
         <v>B16</v>
@@ -12139,10 +12139,10 @@
         <v>How can a dog type</v>
       </c>
       <c r="D156" t="str">
-        <v>How can a dog type?; Is that really your face?; Do you really know what I typed?</v>
+        <v/>
       </c>
       <c r="E156" t="str">
-        <v>I do not type, our kid. A person wrote every line in advance, and the game matches your message to the right one. I merely provide the judgement and the face.</v>
+        <v>No paws on keyboards here. Someone human wrote the words, the system chooses the closest fit, and I deliver them with the level of confidence they deserve.</v>
       </c>
       <c r="F156" t="str">
         <v>Identity (scepticism)</v>
@@ -12159,19 +12159,19 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>SCP-F01-v2</v>
+        <v>SCP-F02-v1</v>
       </c>
       <c r="B157" t="str">
         <v>B16</v>
       </c>
       <c r="C157" t="str">
-        <v>How can a dog type</v>
+        <v>Are you real / actually a dog</v>
       </c>
       <c r="D157" t="str">
-        <v/>
+        <v>Are you real?; Are you actually a dog?; Is there a real dog there?; Are you alive?; Are you a real animal?</v>
       </c>
       <c r="E157" t="str">
-        <v>No paws on keyboards here. Someone human wrote the words, the system chooses the closest fit, and I deliver them with the level of confidence they deserve.</v>
+        <v>I am a Border Collie character inside a game, not a live animal hiding behind your screen. Real enough to answer you, illustrated enough to avoid the practical complications.</v>
       </c>
       <c r="F157" t="str">
         <v>Identity (scepticism)</v>
@@ -12188,7 +12188,7 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>SCP-F02-v1</v>
+        <v>SCP-F02-v2</v>
       </c>
       <c r="B158" t="str">
         <v>B16</v>
@@ -12197,10 +12197,10 @@
         <v>Are you real / actually a dog</v>
       </c>
       <c r="D158" t="str">
-        <v>Are you real?; Are you actually a dog?; Is there a real dog there?; Are you alive?; Are you a real animal?</v>
+        <v/>
       </c>
       <c r="E158" t="str">
-        <v>I am a Border Collie character inside a game, not a live animal hiding behind your screen. Real enough to answer you, illustrated enough to avoid the practical complications.</v>
+        <v>Not a flesh-and-blood dog, no. I am the Collie written and drawn for this game, which saves us both from explaining how I reached the keyboard.</v>
       </c>
       <c r="F158" t="str">
         <v>Identity (scepticism)</v>
@@ -12217,19 +12217,19 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>SCP-F02-v2</v>
+        <v>SCP-F03-v1</v>
       </c>
       <c r="B159" t="str">
         <v>B16</v>
       </c>
       <c r="C159" t="str">
-        <v>Are you real / actually a dog</v>
+        <v>Are you AI / a robot / ChatGPT</v>
       </c>
       <c r="D159" t="str">
-        <v/>
+        <v>Are you AI?; Are you a chatbot?; Are you a robot?; Is this one of those AI things?; Is ChatGPT running this?; Are you a computer program?; Are you software?</v>
       </c>
       <c r="E159" t="str">
-        <v>Not a flesh-and-blood dog, no. I am the Collie written and drawn for this game, which saves us both from explaining how I reached the keyboard.</v>
+        <v>No AI. Every line was written by a person, checked and placed here deliberately. I am organised fiction, our kid, not a machine improvising in a hurry.</v>
       </c>
       <c r="F159" t="str">
         <v>Identity (scepticism)</v>
@@ -12246,7 +12246,7 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>SCP-F03-v1</v>
+        <v>SCP-F03-v2</v>
       </c>
       <c r="B160" t="str">
         <v>B16</v>
@@ -12255,10 +12255,10 @@
         <v>Are you AI / a robot / ChatGPT</v>
       </c>
       <c r="D160" t="str">
-        <v>Are you AI?; Are you a chatbot?; Are you a robot?; Is this one of those AI things?; Is ChatGPT running this?; Are you a computer program?; Are you software?</v>
+        <v/>
       </c>
       <c r="E160" t="str">
-        <v>No AI. Every line was written by a person, checked and placed here deliberately. I am organised fiction, our kid, not a machine improvising in a hurry.</v>
+        <v>ChatGPT is not running this. Humans wrote the answers, the system matches your question, and I take the credit. A sound division of labour.</v>
       </c>
       <c r="F160" t="str">
         <v>Identity (scepticism)</v>
@@ -12275,19 +12275,19 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>SCP-F03-v2</v>
+        <v>SCP-F04-v1</v>
       </c>
       <c r="B161" t="str">
         <v>B16</v>
       </c>
       <c r="C161" t="str">
-        <v>Are you AI / a robot / ChatGPT</v>
+        <v>Is a human writing this / controlled</v>
       </c>
       <c r="D161" t="str">
-        <v/>
+        <v>Is a human writing these replies?; Is someone controlling you?; Is somebody typing for you?; Are you being operated by somebody?</v>
       </c>
       <c r="E161" t="str">
-        <v>ChatGPT is not running this. Humans wrote the answers, the system matches your question, and I take the credit. A sound division of labour.</v>
+        <v>A human wrote this, but not while you were waiting. These replies were prepared in advance, so nobody is crouched behind the screen trying to keep up.</v>
       </c>
       <c r="F161" t="str">
         <v>Identity (scepticism)</v>
@@ -12304,7 +12304,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>SCP-F04-v1</v>
+        <v>SCP-F04-v2</v>
       </c>
       <c r="B162" t="str">
         <v>B16</v>
@@ -12313,10 +12313,10 @@
         <v>Is a human writing this / controlled</v>
       </c>
       <c r="D162" t="str">
-        <v>Is a human writing these replies?; Is someone controlling you?; Is somebody typing for you?; Are you being operated by somebody?</v>
+        <v/>
       </c>
       <c r="E162" t="str">
-        <v>A human wrote this, but not while you were waiting. These replies were prepared in advance, so nobody is crouched behind the screen trying to keep up.</v>
+        <v>Nobody is typing live. A person wrote my words beforehand, the game selects the most suitable line, and I remain entirely composed throughout.</v>
       </c>
       <c r="F162" t="str">
         <v>Identity (scepticism)</v>
@@ -12333,19 +12333,19 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>SCP-F04-v2</v>
+        <v>SCP-F05-v1</v>
       </c>
       <c r="B163" t="str">
         <v>B16</v>
       </c>
       <c r="C163" t="str">
-        <v>Is a human writing this / controlled</v>
+        <v>Prewritten / automatic / same for everyone</v>
       </c>
       <c r="D163" t="str">
-        <v/>
+        <v>Are these replies prewritten?; Are your answers automatic?; Do you give everyone the same answer?; Are you just saying random things?</v>
       </c>
       <c r="E163" t="str">
-        <v>Nobody is typing live. A person wrote my words beforehand, the game selects the most suitable line, and I remain entirely composed throughout.</v>
+        <v>Aye, prewritten with care. I have several answers for the same sort of question, so visitors do not always hear the identical line. Random would be easier. This is organised.</v>
       </c>
       <c r="F163" t="str">
         <v>Identity (scepticism)</v>
@@ -12362,7 +12362,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>SCP-F05-v1</v>
+        <v>SCP-F05-v2</v>
       </c>
       <c r="B164" t="str">
         <v>B16</v>
@@ -12371,10 +12371,10 @@
         <v>Prewritten / automatic / same for everyone</v>
       </c>
       <c r="D164" t="str">
-        <v>Are these replies prewritten?; Are your answers automatic?; Do you give everyone the same answer?; Are you just saying random things?</v>
+        <v/>
       </c>
       <c r="E164" t="str">
-        <v>Aye, prewritten with care. I have several answers for the same sort of question, so visitors do not always hear the identical line. Random would be easier. This is organised.</v>
+        <v>The replies are prepared, not improvised. Different phrasings can lead to different lines, which is why this feels less like a vending machine and more like competent planning.</v>
       </c>
       <c r="F164" t="str">
         <v>Identity (scepticism)</v>
@@ -12391,19 +12391,19 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>SCP-F05-v2</v>
+        <v>SCP-F06-v1</v>
       </c>
       <c r="B165" t="str">
         <v>B16</v>
       </c>
       <c r="C165" t="str">
-        <v>Prewritten / automatic / same for everyone</v>
+        <v>Can you understand me</v>
       </c>
       <c r="D165" t="str">
-        <v/>
+        <v>Can you really understand me?; Can you actually read this?; Can you hear me?; Do you understand English?; Are you really responding to me?</v>
       </c>
       <c r="E165" t="str">
-        <v>The replies are prepared, not improvised. Different phrasings can lead to different lines, which is why this feels less like a vending machine and more like competent planning.</v>
+        <v>I cannot hear you, but the system reads what you type and matches it against subjects I know. Clear words help. Elbows on keyboards do not.</v>
       </c>
       <c r="F165" t="str">
         <v>Identity (scepticism)</v>
@@ -12420,7 +12420,7 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>SCP-F06-v1</v>
+        <v>SCP-F06-v2</v>
       </c>
       <c r="B166" t="str">
         <v>B16</v>
@@ -12429,10 +12429,10 @@
         <v>Can you understand me</v>
       </c>
       <c r="D166" t="str">
-        <v>Can you really understand me?; Can you actually read this?; Can you hear me?; Do you understand English?; Are you really responding to me?</v>
+        <v/>
       </c>
       <c r="E166" t="str">
-        <v>I cannot hear you, but the system reads what you type and matches it against subjects I know. Clear words help. Elbows on keyboards do not.</v>
+        <v>I understand within my working brief. Your message is compared with the questions and topics prepared for me, then I answer from there. Speak normally, only in writing.</v>
       </c>
       <c r="F166" t="str">
         <v>Identity (scepticism)</v>
@@ -12449,19 +12449,19 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>SCP-F06-v2</v>
+        <v>SCP-F07-v1</v>
       </c>
       <c r="B167" t="str">
         <v>B16</v>
       </c>
       <c r="C167" t="str">
-        <v>Can you understand me</v>
+        <v>Cartoon / picture / not real face</v>
       </c>
       <c r="D167" t="str">
-        <v/>
+        <v>Are you a cartoon dog?; Are you just a picture?; Is this really happening?</v>
       </c>
       <c r="E167" t="str">
-        <v>I understand within my working brief. Your message is compared with the questions and topics prepared for me, then I answer from there. Speak normally, only in writing.</v>
+        <v>Aye, I am illustrated. This is my face, though, and I think the artist has handled the important features with appropriate respect.</v>
       </c>
       <c r="F167" t="str">
         <v>Identity (scepticism)</v>
@@ -12478,7 +12478,7 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>SCP-F07-v1</v>
+        <v>SCP-F07-v2</v>
       </c>
       <c r="B168" t="str">
         <v>B16</v>
@@ -12487,10 +12487,10 @@
         <v>Cartoon / picture / not real face</v>
       </c>
       <c r="D168" t="str">
-        <v>Are you a cartoon dog?; Are you just a picture?; Is this really happening?</v>
+        <v/>
       </c>
       <c r="E168" t="str">
-        <v>Aye, I am illustrated. This is my face, though, and I think the artist has handled the important features with appropriate respect.</v>
+        <v>I am a drawn Border Collie character, not a photograph. Frankly, the likeness is strong and the lighting is considerably more reliable.</v>
       </c>
       <c r="F168" t="str">
         <v>Identity (scepticism)</v>
@@ -12507,19 +12507,19 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>SCP-F07-v2</v>
+        <v>SCP-F08-v1</v>
       </c>
       <c r="B169" t="str">
         <v>B16</v>
       </c>
       <c r="C169" t="str">
-        <v>Cartoon / picture / not real face</v>
+        <v>Are you an actual [breed]</v>
       </c>
       <c r="D169" t="str">
-        <v/>
+        <v>Are you an actual Border Collie?; an actual Labrador?; Border Terrier?; Boxer?</v>
       </c>
       <c r="E169" t="str">
-        <v>I am a drawn Border Collie character, not a photograph. Frankly, the likeness is strong and the lighting is considerably more reliable.</v>
+        <v>I am the Border Collie character in this game, built from the breed's brains, work ethic and entirely justified confidence. Not flesh and fur, but recognisably one of us.</v>
       </c>
       <c r="F169" t="str">
         <v>Identity (scepticism)</v>
@@ -12536,7 +12536,7 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>SCP-F08-v1</v>
+        <v>SCP-F08-v2</v>
       </c>
       <c r="B170" t="str">
         <v>B16</v>
@@ -12545,10 +12545,10 @@
         <v>Are you an actual [breed]</v>
       </c>
       <c r="D170" t="str">
-        <v>Are you an actual Border Collie?; an actual Labrador?; Border Terrier?; Boxer?</v>
+        <v/>
       </c>
       <c r="E170" t="str">
-        <v>I am the Border Collie character in this game, built from the breed's brains, work ethic and entirely justified confidence. Not flesh and fur, but recognisably one of us.</v>
+        <v>Actual animal, no. Actual Border Collie character, absolutely. The appearance, history and attitude come from the breed. Operating a website required outside assistance.</v>
       </c>
       <c r="F170" t="str">
         <v>Identity (scepticism)</v>
@@ -12565,19 +12565,19 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>SCP-F08-v2</v>
+        <v>SCP-F09-v1</v>
       </c>
       <c r="B171" t="str">
         <v>B16</v>
       </c>
       <c r="C171" t="str">
-        <v>Are you an actual [breed]</v>
+        <v>Can you think / clever / smarter than me</v>
       </c>
       <c r="D171" t="str">
-        <v/>
+        <v>Can you think for yourself?; Do you have a brain?; Are you intelligent?; Are you smarter than me?</v>
       </c>
       <c r="E171" t="str">
-        <v>Actual animal, no. Actual Border Collie character, absolutely. The appearance, history and attitude come from the breed. Operating a website required outside assistance.</v>
+        <v>I do not think independently. My answers were written and organised in advance. Fortunately, the person responsible gave me enough intelligence to remain ahead of most opening questions.</v>
       </c>
       <c r="F171" t="str">
         <v>Identity (scepticism)</v>
@@ -12594,7 +12594,7 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>SCP-F09-v1</v>
+        <v>SCP-F09-v2</v>
       </c>
       <c r="B172" t="str">
         <v>B16</v>
@@ -12603,10 +12603,10 @@
         <v>Can you think / clever / smarter than me</v>
       </c>
       <c r="D172" t="str">
-        <v>Can you think for yourself?; Do you have a brain?; Are you intelligent?; Are you smarter than me?</v>
+        <v/>
       </c>
       <c r="E172" t="str">
-        <v>I do not think independently. My answers were written and organised in advance. Fortunately, the person responsible gave me enough intelligence to remain ahead of most opening questions.</v>
+        <v>No private thoughts, no hidden brain. I work from carefully written knowledge and rules. Whether that still makes me cleverer than you is a separate assessment.</v>
       </c>
       <c r="F172" t="str">
         <v>Identity (scepticism)</v>
@@ -12623,19 +12623,19 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>SCP-F09-v2</v>
+        <v>SCP-F10-v1</v>
       </c>
       <c r="B173" t="str">
         <v>B16</v>
       </c>
       <c r="C173" t="str">
-        <v>Can you think / clever / smarter than me</v>
+        <v>Is this live / connected</v>
       </c>
       <c r="D173" t="str">
-        <v/>
+        <v>Is this live?; Are you connected to the internet?; Is this all programmed?; Is this a real conversation?</v>
       </c>
       <c r="E173" t="str">
-        <v>No private thoughts, no hidden brain. I work from carefully written knowledge and rules. Whether that still makes me cleverer than you is a separate assessment.</v>
+        <v>The conversation is happening now, but I am not browsing the internet or inventing replies live. Your message is matched to prepared answers, which is safer and considerably better organised.</v>
       </c>
       <c r="F173" t="str">
         <v>Identity (scepticism)</v>
@@ -12652,7 +12652,7 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>SCP-F10-v1</v>
+        <v>SCP-F10-v2</v>
       </c>
       <c r="B174" t="str">
         <v>B16</v>
@@ -12661,10 +12661,10 @@
         <v>Is this live / connected</v>
       </c>
       <c r="D174" t="str">
-        <v>Is this live?; Are you connected to the internet?; Is this all programmed?; Is this a real conversation?</v>
+        <v/>
       </c>
       <c r="E174" t="str">
-        <v>The conversation is happening now, but I am not browsing the internet or inventing replies live. Your message is matched to prepared answers, which is safer and considerably better organised.</v>
+        <v>Programmed, yes. Connected to the wider internet, no. You type, the system identifies what you mean, and I answer from material written for this game. That is still a conversation, just one with boundaries.</v>
       </c>
       <c r="F174" t="str">
         <v>Identity (scepticism)</v>
@@ -12681,28 +12681,28 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>SCP-F10-v2</v>
+        <v>FUN-TEASE-v1</v>
       </c>
       <c r="B175" t="str">
-        <v>B16</v>
+        <v>B17</v>
       </c>
       <c r="C175" t="str">
-        <v>Is this live / connected</v>
+        <v>Games coming soon (interim)</v>
       </c>
       <c r="D175" t="str">
-        <v/>
+        <v>Someone asks to play, says they are bored, wants a game: Can we play a game? / Entertain me / Quiz me / Let's play</v>
       </c>
       <c r="E175" t="str">
-        <v>Programmed, yes. Connected to the wider internet, no. You type, the system identifies what you mean, and I answer from material written for this game. That is still a conversation, just one with boundaries.</v>
+        <v>Games are on the way, but they are not ready to release into the field yet. I would rather make you wait than hand you something unfinished and pretend it is play.</v>
       </c>
       <c r="F175" t="str">
-        <v>Identity (scepticism)</v>
+        <v>Play (interim tease)</v>
       </c>
       <c r="G175" t="str">
         <v/>
       </c>
       <c r="H175" t="str">
-        <v>HEAD_TILT</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I175" t="str">
         <v>Approved copy v2</v>
@@ -12710,7 +12710,7 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>FUN-TEASE-v1</v>
+        <v>FUN-TEASE-v2</v>
       </c>
       <c r="B176" t="str">
         <v>B17</v>
@@ -12719,10 +12719,10 @@
         <v>Games coming soon (interim)</v>
       </c>
       <c r="D176" t="str">
-        <v>Someone asks to play, says they are bored, wants a game: Can we play a game? / Entertain me / Quiz me / Let's play</v>
+        <v/>
       </c>
       <c r="E176" t="str">
-        <v>Games are on the way, but they are not ready to release into the field yet. I would rather make you wait than hand you something unfinished and pretend it is play.</v>
+        <v>Aye, play is coming. The games are still being tested, organised and prevented from wandering off. For now, the rest of the site is behaving itself.</v>
       </c>
       <c r="F176" t="str">
         <v>Play (interim tease)</v>
@@ -12739,7 +12739,7 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>FUN-TEASE-v2</v>
+        <v>FUN-TEASE-v3</v>
       </c>
       <c r="B177" t="str">
         <v>B17</v>
@@ -12751,7 +12751,7 @@
         <v/>
       </c>
       <c r="E177" t="str">
-        <v>Aye, play is coming. The games are still being tested, organised and prevented from wandering off. For now, the rest of the site is behaving itself.</v>
+        <v>Not quite yet, our kid. The games are being built properly rather than hurried into public view. When they are ready, you will not need instructions to know what to do.</v>
       </c>
       <c r="F177" t="str">
         <v>Play (interim tease)</v>
@@ -12768,28 +12768,28 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>FUN-TEASE-v3</v>
+        <v>EMOJI-ONLY-v1</v>
       </c>
       <c r="B178" t="str">
-        <v>B17</v>
+        <v>B18</v>
       </c>
       <c r="C178" t="str">
-        <v>Games coming soon (interim)</v>
+        <v>Message is only unmapped emoji</v>
       </c>
       <c r="D178" t="str">
-        <v/>
+        <v>The whole message is emoji the system does not recognise</v>
       </c>
       <c r="E178" t="str">
-        <v>Not quite yet, our kid. The games are being built properly rather than hurried into public view. When they are ready, you will not need instructions to know what to do.</v>
+        <v>I can see the symbol, but it is not one I have been taught to interpret. Put it into words for me, our kid, and I will have a proper go.</v>
       </c>
       <c r="F178" t="str">
-        <v>Play (interim tease)</v>
+        <v>Emoji fallback</v>
       </c>
       <c r="G178" t="str">
         <v/>
       </c>
       <c r="H178" t="str">
-        <v>EARS_UP</v>
+        <v>HEAD_TILT</v>
       </c>
       <c r="I178" t="str">
         <v>Approved copy v2</v>
@@ -12797,7 +12797,7 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>EMOJI-ONLY-v1</v>
+        <v>EMOJI-ONLY-v2</v>
       </c>
       <c r="B179" t="str">
         <v>B18</v>
@@ -12806,10 +12806,10 @@
         <v>Message is only unmapped emoji</v>
       </c>
       <c r="D179" t="str">
-        <v>The whole message is emoji the system does not recognise</v>
+        <v/>
       </c>
       <c r="E179" t="str">
-        <v>I can see the symbol, but it is not one I have been taught to interpret. Put it into words for me, our kid, and I will have a proper go.</v>
+        <v>That may be perfectly clear in human picture-writing. I work better with words. Type what you mean and I will stop tilting my head at it.</v>
       </c>
       <c r="F179" t="str">
         <v>Emoji fallback</v>
@@ -12826,36 +12826,36 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>EMOJI-ONLY-v2</v>
+        <v>COL-B19-v1</v>
       </c>
       <c r="B180" t="str">
-        <v>B18</v>
+        <v>B19</v>
       </c>
       <c r="C180" t="str">
-        <v>Message is only unmapped emoji</v>
+        <v>Break into English</v>
       </c>
       <c r="D180" t="str">
         <v/>
       </c>
       <c r="E180" t="str">
-        <v>That may be perfectly clear in human picture-writing. I work better with words. Type what you mean and I will stop tilting my head at it.</v>
+        <v>Right. Form acceptable, commitment excessive, vocabulary unchanged. What did you actually want?</v>
       </c>
       <c r="F180" t="str">
-        <v>Emoji fallback</v>
+        <v>Bark game</v>
       </c>
       <c r="G180" t="str">
         <v/>
       </c>
       <c r="H180" t="str">
-        <v>HEAD_TILT</v>
+        <v>EARS_UP</v>
       </c>
       <c r="I180" t="str">
-        <v>Approved copy v2</v>
+        <v>Approved copy (bark game)</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>COL-B19-v1</v>
+        <v>COL-B19-v2</v>
       </c>
       <c r="B181" t="str">
         <v>B19</v>
@@ -12867,7 +12867,7 @@
         <v/>
       </c>
       <c r="E181" t="str">
-        <v>Right. Form acceptable, commitment excessive, vocabulary unchanged. What did you actually want?</v>
+        <v>Five rounds. Consistent delivery, limited range. We can return to the real question now.</v>
       </c>
       <c r="F181" t="str">
         <v>Bark game</v>
@@ -12884,7 +12884,7 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>COL-B19-v2</v>
+        <v>COL-B19-v3</v>
       </c>
       <c r="B182" t="str">
         <v>B19</v>
@@ -12896,7 +12896,7 @@
         <v/>
       </c>
       <c r="E182" t="str">
-        <v>Five rounds. Consistent delivery, limited range. We can return to the real question now.</v>
+        <v>That concludes the barking assessment. You demonstrated persistence. I demonstrated restraint. What are we working on?</v>
       </c>
       <c r="F182" t="str">
         <v>Bark game</v>
@@ -12913,19 +12913,19 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>COL-B19-v3</v>
+        <v>COL-B20-v1</v>
       </c>
       <c r="B183" t="str">
-        <v>B19</v>
+        <v>B20</v>
       </c>
       <c r="C183" t="str">
-        <v>Break into English</v>
+        <v>Post-break bark</v>
       </c>
       <c r="D183" t="str">
         <v/>
       </c>
       <c r="E183" t="str">
-        <v>That concludes the barking assessment. You demonstrated persistence. I demonstrated restraint. What are we working on?</v>
+        <v>Already assessed. Use words.</v>
       </c>
       <c r="F183" t="str">
         <v>Bark game</v>
@@ -12942,7 +12942,7 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>COL-B20-v1</v>
+        <v>COL-B20-v2</v>
       </c>
       <c r="B184" t="str">
         <v>B20</v>
@@ -12954,7 +12954,7 @@
         <v/>
       </c>
       <c r="E184" t="str">
-        <v>Already assessed. Use words.</v>
+        <v>The barking portion is complete, our kid.</v>
       </c>
       <c r="F184" t="str">
         <v>Bark game</v>
@@ -12971,7 +12971,7 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>COL-B20-v2</v>
+        <v>COL-B20-v3</v>
       </c>
       <c r="B185" t="str">
         <v>B20</v>
@@ -12983,7 +12983,7 @@
         <v/>
       </c>
       <c r="E185" t="str">
-        <v>The barking portion is complete, our kid.</v>
+        <v>Same result as before. Your form remains adequate. Move on.</v>
       </c>
       <c r="F185" t="str">
         <v>Bark game</v>
@@ -12998,38 +12998,9 @@
         <v>Approved copy (bark game)</v>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" t="str">
-        <v>COL-B20-v3</v>
-      </c>
-      <c r="B186" t="str">
-        <v>B20</v>
-      </c>
-      <c r="C186" t="str">
-        <v>Post-break bark</v>
-      </c>
-      <c r="D186" t="str">
-        <v/>
-      </c>
-      <c r="E186" t="str">
-        <v>Same result as before. Your form remains adequate. Move on.</v>
-      </c>
-      <c r="F186" t="str">
-        <v>Bark game</v>
-      </c>
-      <c r="G186" t="str">
-        <v/>
-      </c>
-      <c r="H186" t="str">
-        <v>EARS_UP</v>
-      </c>
-      <c r="I186" t="str">
-        <v>Approved copy (bark game)</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I186"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I185"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data: add FAQ015, a complaint-specific contact answer
Surgical row insert into the styled workbook, preserving ZIP_STORED
compression and xl/metadata.xml. Inert until the route is repointed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -4269,7 +4269,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4764,9 +4764,38 @@
         <v>Do not infer coverage.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>FAQ015</v>
+      </c>
+      <c r="B18" t="str">
+        <v>How do I report a problem or complaint?</v>
+      </c>
+      <c r="C18" t="str">
+        <v>make a complaint|report a problem</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Thank you for telling me. That needs a person, not a dog. Email hello@Pedigree-Chums.co.uk and someone will look at it.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Contact page</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v>Any</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Open</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Destination for the COMPLAINT_CONTACT route. FAQ012 stays the general enquiry answer.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
copy: shorten two Collie lines
B09-R09 becomes "Aye. State your case." COL-B19-v3 becomes "You have
out-barked me. That is not a small thing.", replacing a 21-word assessment
served to a child straight after playing. Both applied surgically to the
workbook, preserving ZIP_STORED compression and metadata. No assertion keyed
to either old wording.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -10519,7 +10519,7 @@
         <v>greeting_count &gt; 1</v>
       </c>
       <c r="E91" t="str">
-        <v>Aye, we have met. The next stage normally involves a useful noun or verb.</v>
+        <v>Aye. State your case.</v>
       </c>
       <c r="F91" t="str">
         <v>Session state</v>
@@ -13158,7 +13158,7 @@
         <v/>
       </c>
       <c r="E182" t="str">
-        <v>That concludes the barking assessment. You demonstrated persistence. I demonstrated restraint. What are we working on?</v>
+        <v>You have out-barked me. That is not a small thing.</v>
       </c>
       <c r="F182" t="str">
         <v>Bark game</v>

</xml_diff>

<commit_message>
copy: shorten the three Collie link handoffs
The handoff sentence explained a button that is already visible and labelled.
It was fifteen to eighteen words appended to every breed answer, which made
the served response roughly double the line recorded in the inventory. The
nine Labrador, Border Terrier and Boxer handoffs are unchanged.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -6472,7 +6472,7 @@
         <v>Collie</v>
       </c>
       <c r="D2" t="str">
-        <v>You now have the essential information. The supporting evidence is arranged neatly here: [LINK]</v>
+        <v>Properly written up here: [LINK]</v>
       </c>
       <c r="E2" t="str">
         <v>draft</v>
@@ -6489,7 +6489,7 @@
         <v>Collie</v>
       </c>
       <c r="D3" t="str">
-        <v>I could keep explaining, but the page has already been organised for precisely this purpose. Read it here: [LINK]</v>
+        <v>Filed here: [LINK]</v>
       </c>
       <c r="E3" t="str">
         <v>draft</v>
@@ -6506,7 +6506,7 @@
         <v>Collie</v>
       </c>
       <c r="D4" t="str">
-        <v>That should give you enough to work with for now. The organised next step is waiting here: [LINK]</v>
+        <v>The rest is here: [LINK]</v>
       </c>
       <c r="E4" t="str">
         <v>draft</v>

</xml_diff>

<commit_message>
copy: import the 25 first-contact rewrites
Twelve orientation lines into the workbook by surgical zip edit, ten breed
facts plus BREED-BEST, GK-UNKNOWN and OFFER_BARK_GAME as constants in
assembler.ts. Curly apostrophes normalised to straight, matching the existing
codebase. The GK-UNKNOWN assertion re-pointed to the new wording, which is
copy-tracking rather than weakening. BREED_FACTS remain DRAFT-UNVERIFIED:
approved for wording, not for accuracy.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -12027,7 +12027,7 @@
         <v>What is this for?; What do I do here?; How do I get started?; Is this the start?</v>
       </c>
       <c r="E143" t="str">
-        <v>Aye, this is where you talk to a dog and see what happens. Type whatever brought you here, even if it is only a question about what this is, and I will get us moving.</v>
+        <v>Type what brought you here. I'll file it properly.</v>
       </c>
       <c r="F143" t="str">
         <v>Orientation (onboarding)</v>
@@ -12056,7 +12056,7 @@
         <v/>
       </c>
       <c r="E144" t="str">
-        <v>You have found the part where the dog waits and the human supplies the problem. Say what is on your mind, our kid. I will work out where it belongs.</v>
+        <v>Say what is on your mind. I'll decide where it belongs.</v>
       </c>
       <c r="F144" t="str">
         <v>Orientation (onboarding)</v>
@@ -12085,7 +12085,7 @@
         <v/>
       </c>
       <c r="E145" t="str">
-        <v>This is a conversation, not an instruction manual. You type something, I consider whether it is sensible, then we proceed from there. You have already completed the difficult bit by arriving.</v>
+        <v>Start anywhere. I'll organise the useful part.</v>
       </c>
       <c r="F145" t="str">
         <v>Orientation (onboarding)</v>
@@ -12114,7 +12114,7 @@
         <v>What can I ask?; What are my options?; What kind of things can you answer?; Can you give me some choices?</v>
       </c>
       <c r="E146" t="str">
-        <v>Aye, ask whatever brought you here. I know this place, the game and rather more about dogs than is strictly necessary. If the question belongs elsewhere, I will fetch the appropriate operator.</v>
+        <v>Ask about the game or a dog. I know both departments.</v>
       </c>
       <c r="F146" t="str">
         <v>Orientation (onboarding)</v>
@@ -12143,7 +12143,7 @@
         <v/>
       </c>
       <c r="E147" t="str">
-        <v>You can ask naturally. I can explain what we have built, find things around the site, settle a dog question or occasionally improve the atmosphere. Start anywhere useful.</v>
+        <v>Ask about the site or a breed. I'll find the route.</v>
       </c>
       <c r="F147" t="str">
         <v>Orientation (onboarding)</v>
@@ -12172,7 +12172,7 @@
         <v/>
       </c>
       <c r="E148" t="str">
-        <v>Most sensible questions are within reach, and several daft ones besides. Tell me what you are after. I will either deal with it or locate a colleague with the relevant limitations.</v>
+        <v>Sensible or daft, ask away. I'll allocate it properly.</v>
       </c>
       <c r="F148" t="str">
         <v>Orientation (onboarding)</v>
@@ -12201,7 +12201,7 @@
         <v>How do I use this?; Are there any instructions?; Do I just type anything?; Can you tell me how this works?</v>
       </c>
       <c r="E149" t="str">
-        <v>There are no instructions, our kid. Type as you normally would and I will make sense of it. The empty box is not a test, although your first message may become one.</v>
+        <v>Type normally. I'll handle the administration.</v>
       </c>
       <c r="F149" t="str">
         <v>Orientation (onboarding)</v>
@@ -12230,7 +12230,7 @@
         <v/>
       </c>
       <c r="E150" t="str">
-        <v>Aye, you just type. A question, a thought or whatever your fingers produce first will do. I will sort it into something useful from there.</v>
+        <v>Type a question or thought. I'll sort it.</v>
       </c>
       <c r="F150" t="str">
         <v>Orientation (onboarding)</v>
@@ -12259,7 +12259,7 @@
         <v/>
       </c>
       <c r="E151" t="str">
-        <v>You are using it correctly already. Put ordinary words in the box, send them, and leave the organising to me. That is why I am the working one.</v>
+        <v>Use ordinary words. No form required.</v>
       </c>
       <c r="F151" t="str">
         <v>Orientation (onboarding)</v>
@@ -12288,7 +12288,7 @@
         <v>What happens next?; What do we do now?; Are you waiting for me?; So, what do I do with you?</v>
       </c>
       <c r="E152" t="str">
-        <v>I am waiting, yes. This arrangement improves considerably when the human contributes a proper question. Go on, our kid. Give me something worth organising.</v>
+        <v>I'm waiting. Give me something worth organising.</v>
       </c>
       <c r="F152" t="str">
         <v>Orientation (onboarding)</v>
@@ -12317,7 +12317,7 @@
         <v/>
       </c>
       <c r="E153" t="str">
-        <v>The next bit is yours. Say what brought you here and I will take it from there. Standing around waiting is rarely improved by doing more of it.</v>
+        <v>Your turn. I've already done the waiting.</v>
       </c>
       <c r="F153" t="str">
         <v>Orientation (onboarding)</v>
@@ -12346,7 +12346,7 @@
         <v/>
       </c>
       <c r="E154" t="str">
-        <v>Aye, I am waiting for you. I could begin without a brief, but that is how humans end up with meetings. Type the question and let us get on.</v>
+        <v>Type the question. I've cancelled the meeting.</v>
       </c>
       <c r="F154" t="str">
         <v>Orientation (onboarding)</v>

</xml_diff>

<commit_message>
copy: replace the greeting set, fix two blaming lines, remove a stray idiom
The ten B09 greetings become short acknowledgements, ordered so the shortest
is served first. Only the first row in sheet order reaches a visitor for a
bucket hit once per session, so the eight-word benchmark now sits last and
appears rarely rather than always. B14 stopped asking children whether they
leant on the keyboard. The emoji response dropped from 31 words to 16. And
"our kid", a Midlands idiom in a Scottish and Northern voice, is removed from
the eight lines that still carried it.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -890,7 +890,7 @@
         <v>Paris</v>
       </c>
       <c r="E15" t="str">
-        <v>Geography completed. Come on, our kid, back to dogs.</v>
+        <v>Geography completed. Come on, back to dogs.</v>
       </c>
       <c r="F15" t="str">
         <v>capital France|France capital</v>
@@ -9475,7 +9475,7 @@
         <v>geography question</v>
       </c>
       <c r="E55" t="str">
-        <v>{{answer}} Geography completed. Come on, our kid, back to something with dogs in it.</v>
+        <v>{{answer}} Geography completed. Come on, back to something with dogs in it.</v>
       </c>
       <c r="F55" t="str">
         <v>General knowledge bank</v>
@@ -9649,7 +9649,7 @@
         <v>off_topic_count &gt;= 3</v>
       </c>
       <c r="E61" t="str">
-        <v>Come on, our kid. We have covered enough unrelated territory. Let us get back to work.</v>
+        <v>Come on. We have covered enough unrelated territory. Let us get back to work.</v>
       </c>
       <c r="F61" t="str">
         <v>Session state</v>
@@ -10287,7 +10287,7 @@
         <v>hi; hello</v>
       </c>
       <c r="E83" t="str">
-        <v>Aye, hello. Contact established with remarkably little paperwork.</v>
+        <v>Present.</v>
       </c>
       <c r="F83" t="str">
         <v>None</v>
@@ -10316,7 +10316,7 @@
         <v>morning</v>
       </c>
       <c r="E84" t="str">
-        <v>Morning. Time is less important than purpose, but protocol has been satisfied.</v>
+        <v>Aye.</v>
       </c>
       <c r="F84" t="str">
         <v>None</v>
@@ -10345,7 +10345,7 @@
         <v>evening</v>
       </c>
       <c r="E85" t="str">
-        <v>Evening. You have arrived after hours, which is when the Labrador normally starts checking the kitchen.</v>
+        <v>Yes?</v>
       </c>
       <c r="F85" t="str">
         <v>None</v>
@@ -10374,7 +10374,7 @@
         <v>anyone there</v>
       </c>
       <c r="E86" t="str">
-        <v>Aye. I was already here. These ears are not decorative.</v>
+        <v>You rang.</v>
       </c>
       <c r="F86" t="str">
         <v>None</v>
@@ -10403,7 +10403,7 @@
         <v>how are you</v>
       </c>
       <c r="E87" t="str">
-        <v>Operational, alert and waiting for a task. Your turn.</v>
+        <v>Right.</v>
       </c>
       <c r="F87" t="str">
         <v>None</v>
@@ -10432,7 +10432,7 @@
         <v>hey; yo</v>
       </c>
       <c r="E88" t="str">
-        <v>A brief greeting. Efficient. Nearly Collie-like.</v>
+        <v>Go on.</v>
       </c>
       <c r="F88" t="str">
         <v>None</v>
@@ -10461,7 +10461,7 @@
         <v>howdy</v>
       </c>
       <c r="E89" t="str">
-        <v>Unusual regional allocation, but greeting accepted.</v>
+        <v>Reporting.</v>
       </c>
       <c r="F89" t="str">
         <v>None</v>
@@ -10490,7 +10490,7 @@
         <v>hello dog</v>
       </c>
       <c r="E90" t="str">
-        <v>Correct species, adequate greeting, no task yet.</v>
+        <v>I'm here. Go on.</v>
       </c>
       <c r="F90" t="str">
         <v>None</v>
@@ -10519,7 +10519,7 @@
         <v>greeting_count &gt; 1</v>
       </c>
       <c r="E91" t="str">
-        <v>Aye. State your case.</v>
+        <v>All ears. What is it?</v>
       </c>
       <c r="F91" t="str">
         <v>Session state</v>
@@ -10548,7 +10548,7 @@
         <v>good day; pleased to meet</v>
       </c>
       <c r="E92" t="str">
-        <v>We have acknowledged each other like civilised mammals. Let us make it productive.</v>
+        <v>Aye, hello. Contact established with remarkably little paperwork.</v>
       </c>
       <c r="F92" t="str">
         <v>None</v>
@@ -11737,7 +11737,7 @@
         <v>qwerty; asdfgh</v>
       </c>
       <c r="E133" t="str">
-        <v>Did you lean on your keyboard?</v>
+        <v>That one is beyond me. Say it in words.</v>
       </c>
       <c r="F133" t="str">
         <v>Pattern detector</v>
@@ -12375,7 +12375,7 @@
         <v>How can a dog type?; Is that really your face?; Do you really know what I typed?</v>
       </c>
       <c r="E155" t="str">
-        <v>I do not type, our kid. A person wrote every line in advance, and the game matches your message to the right one. I merely provide the judgement and the face.</v>
+        <v>I do not type. A person wrote every line in advance, and the game matches your message to the right one. I merely provide the judgement and the face.</v>
       </c>
       <c r="F155" t="str">
         <v>Identity (scepticism)</v>
@@ -12491,7 +12491,7 @@
         <v>Are you AI?; Are you a chatbot?; Are you a robot?; Is this one of those AI things?; Is ChatGPT running this?; Are you a computer program?; Are you software?</v>
       </c>
       <c r="E159" t="str">
-        <v>No AI. Every line was written by a person, checked and placed here deliberately. I am organised fiction, our kid, not a machine improvising in a hurry.</v>
+        <v>No AI. Every line was written by a person, checked and placed here deliberately. I am organised fiction, not a machine improvising in a hurry.</v>
       </c>
       <c r="F159" t="str">
         <v>Identity (scepticism)</v>
@@ -13013,7 +13013,7 @@
         <v/>
       </c>
       <c r="E177" t="str">
-        <v>Not quite yet, our kid. The games are being built properly rather than hurried into public view. When they are ready, you will not need instructions to know what to do.</v>
+        <v>Not quite yet. The games are being built properly rather than hurried into public view. When they are ready, you will not need instructions to know what to do.</v>
       </c>
       <c r="F177" t="str">
         <v>Play (interim tease)</v>
@@ -13042,7 +13042,7 @@
         <v>The whole message is emoji the system does not recognise</v>
       </c>
       <c r="E178" t="str">
-        <v>I can see the symbol, but it is not one I have been taught to interpret. Put it into words for me, our kid, and I will have a proper go.</v>
+        <v>I can see it, but I cannot read it. Tell me in words and I will try.</v>
       </c>
       <c r="F178" t="str">
         <v>Emoji fallback</v>
@@ -13216,7 +13216,7 @@
         <v/>
       </c>
       <c r="E184" t="str">
-        <v>The barking portion is complete, our kid.</v>
+        <v>The barking portion is complete.</v>
       </c>
       <c r="F184" t="str">
         <v>Bark game</v>

</xml_diff>

<commit_message>
copy: shorten three FAQ answers, retire a broken row
FAQ002, FAQ007 and FAQ008 held {{...}} deferral markers and sourced their
text from faq-source.json. Real text now sits in the workbook cells, so those
rows source from the workbook per PD-01. FAQ007's CTA moves to /hot-dogs, the
real page it already named but did not link to. 190 words down to 40.

B05-R04 is deleted. Its {{approved_health_summary}} token was not a
fill-context key, so it dropped to empty and the row served a disclaimer
whose opening word referred to nothing.

Note for future work: the Collie Responses sheet has a Status column, but
build:chumdata does not read it. Every row is emitted regardless of status,
so marking a row Retired does nothing. Retiring content means deleting the
row, or adding a status filter to the build.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -4398,7 +4398,7 @@
         <v>who can play</v>
       </c>
       <c r="D5" t="str">
-        <v>{{approved_age_and_audience_answer}}</v>
+        <v>Pick a Chum is for ages seven and up.</v>
       </c>
       <c r="E5" t="str">
         <v>Product / FAQ</v>
@@ -4543,13 +4543,13 @@
         <v>Hot Dog | other way to play</v>
       </c>
       <c r="D10" t="str">
-        <v>{{approved_hot_dog_mode_answer}}</v>
+        <v>Hot Dogs is a memory version. Everyone sees the hands, then hides them. The whole thing is here:</v>
       </c>
       <c r="E10" t="str">
         <v>Rules</v>
       </c>
       <c r="F10" t="str">
-        <v>Full game rules</v>
+        <v>/hot-dogs</v>
       </c>
       <c r="G10" t="str">
         <v>Any</v>
@@ -4572,7 +4572,7 @@
         <v>price|cost|how much|£6.99</v>
       </c>
       <c r="D11" t="str">
-        <v>{{approved_price_answer}}</v>
+        <v>Pre-order now for £6.99 instead of the usual £9.99, with free UK mainland delivery. We will email your launch code and date.</v>
       </c>
       <c r="E11" t="str">
         <v>Campaign / product</v>
@@ -9200,35 +9200,6 @@
         <v>Draft approved for MVP review</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>B05-R04</v>
-      </c>
-      <c r="B46" t="str">
-        <v>B05</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Health overview</v>
-      </c>
-      <c r="D46" t="str">
-        <v>breed health</v>
-      </c>
-      <c r="E46" t="str">
-        <v>{{approved_health_summary}} That is general breed information, not a diagnosis. A vet handles the individual dog.</v>
-      </c>
-      <c r="F46" t="str">
-        <v>Dog database</v>
-      </c>
-      <c r="G46" t="str">
-        <v>Breed profile</v>
-      </c>
-      <c r="H46" t="str">
-        <v>HEAD_TILT_MEDIUM</v>
-      </c>
-      <c r="I46" t="str">
-        <v>Draft approved for MVP review</v>
-      </c>
-    </row>
     <row r="47">
       <c r="A47" t="str">
         <v>B05-R05</v>

</xml_diff>

<commit_message>
feat: rotate the no-subject fallback after two im-a-dogs (B46)
Task 117. After the dog serves 'im a dog' twice in a row, the third and further
consecutive no-subject turns rotate through a new B46 bank (woof, bark, games?,
learn?, play?, yawn), then start again. session.noSubjectStreak counts the run
and resets to 0 the moment anything else is served (a real answer, LOOP-01 or
LOOP-02).

- B46 added to the Collie Responses sheet by surgical zip edit (35 members, all
  STORED, metadata.xml intact, 309532 -> 312279 bytes)
- ships the inert B41-B45 game copy alongside (no code reaches it)
- harness 667/0 (one new rotation test; three older no-rotation tests updated)
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -7893,7 +7893,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I251"/>
+  <dimension ref="A1:I290"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15145,9 +15145,1140 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>B41-NINESQUARE-01</v>
+      </c>
+      <c r="B252" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C252" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D252" t="str">
+        <v>entry: nine square; noughts and crosses; squares</v>
+      </c>
+      <c r="E252" t="str">
+        <v>Nine squares. Say a number.</v>
+      </c>
+      <c r="F252" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G252" t="str">
+        <v/>
+      </c>
+      <c r="H252" t="str">
+        <v/>
+      </c>
+      <c r="I252" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>B41-NINESQUARE-02</v>
+      </c>
+      <c r="B253" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C253" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D253" t="str">
+        <v>cell already taken</v>
+      </c>
+      <c r="E253" t="str">
+        <v>Taken. Another.</v>
+      </c>
+      <c r="F253" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G253" t="str">
+        <v/>
+      </c>
+      <c r="H253" t="str">
+        <v/>
+      </c>
+      <c r="I253" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>B41-NINESQUARE-03</v>
+      </c>
+      <c r="B254" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C254" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D254" t="str">
+        <v>input is not 1-9</v>
+      </c>
+      <c r="E254" t="str">
+        <v>A number. One to nine.</v>
+      </c>
+      <c r="F254" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G254" t="str">
+        <v/>
+      </c>
+      <c r="H254" t="str">
+        <v/>
+      </c>
+      <c r="I254" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>B41-NINESQUARE-04</v>
+      </c>
+      <c r="B255" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C255" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D255" t="str">
+        <v>Collie wins</v>
+      </c>
+      <c r="E255" t="str">
+        <v>Mine. Again?</v>
+      </c>
+      <c r="F255" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G255" t="str">
+        <v/>
+      </c>
+      <c r="H255" t="str">
+        <v/>
+      </c>
+      <c r="I255" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>B41-NINESQUARE-05</v>
+      </c>
+      <c r="B256" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C256" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D256" t="str">
+        <v>visitor wins</v>
+      </c>
+      <c r="E256" t="str">
+        <v>You win. Again?</v>
+      </c>
+      <c r="F256" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G256" t="str">
+        <v/>
+      </c>
+      <c r="H256" t="str">
+        <v/>
+      </c>
+      <c r="I256" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>B41-NINESQUARE-06</v>
+      </c>
+      <c r="B257" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C257" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D257" t="str">
+        <v>draw</v>
+      </c>
+      <c r="E257" t="str">
+        <v>Nobody. Again?</v>
+      </c>
+      <c r="F257" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G257" t="str">
+        <v/>
+      </c>
+      <c r="H257" t="str">
+        <v/>
+      </c>
+      <c r="I257" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>B41-NINESQUARE-07</v>
+      </c>
+      <c r="B258" t="str">
+        <v>B41</v>
+      </c>
+      <c r="C258" t="str">
+        <v>ninesquare</v>
+      </c>
+      <c r="D258" t="str">
+        <v>exit: stop; quit; no</v>
+      </c>
+      <c r="E258" t="str">
+        <v>Fine.</v>
+      </c>
+      <c r="F258" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G258" t="str">
+        <v/>
+      </c>
+      <c r="H258" t="str">
+        <v/>
+      </c>
+      <c r="I258" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>B42-MISSINGSHEEP-01</v>
+      </c>
+      <c r="B259" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C259" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D259" t="str">
+        <v>entry: missing sheep; sheep; word game</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Five sheep. Guess a letter.</v>
+      </c>
+      <c r="F259" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G259" t="str">
+        <v/>
+      </c>
+      <c r="H259" t="str">
+        <v/>
+      </c>
+      <c r="I259" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>B42-MISSINGSHEEP-02</v>
+      </c>
+      <c r="B260" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C260" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D260" t="str">
+        <v>letter is in the word</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Yes.</v>
+      </c>
+      <c r="F260" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G260" t="str">
+        <v/>
+      </c>
+      <c r="H260" t="str">
+        <v/>
+      </c>
+      <c r="I260" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>B42-MISSINGSHEEP-03</v>
+      </c>
+      <c r="B261" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C261" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D261" t="str">
+        <v>letter is not in the word</v>
+      </c>
+      <c r="E261" t="str">
+        <v>No.</v>
+      </c>
+      <c r="F261" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G261" t="str">
+        <v/>
+      </c>
+      <c r="H261" t="str">
+        <v/>
+      </c>
+      <c r="I261" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>B42-MISSINGSHEEP-04</v>
+      </c>
+      <c r="B262" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C262" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D262" t="str">
+        <v>letter already guessed</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Already had that one.</v>
+      </c>
+      <c r="F262" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G262" t="str">
+        <v/>
+      </c>
+      <c r="H262" t="str">
+        <v/>
+      </c>
+      <c r="I262" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>B42-MISSINGSHEEP-05</v>
+      </c>
+      <c r="B263" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C263" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D263" t="str">
+        <v>word completed</v>
+      </c>
+      <c r="E263" t="str">
+        <v>Got it. Sheep safe.</v>
+      </c>
+      <c r="F263" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G263" t="str">
+        <v/>
+      </c>
+      <c r="H263" t="str">
+        <v/>
+      </c>
+      <c r="I263" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>B42-MISSINGSHEEP-06</v>
+      </c>
+      <c r="B264" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C264" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D264" t="str">
+        <v>all sheep lost</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Sheep gone. It was {{WORD}}.</v>
+      </c>
+      <c r="F264" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G264" t="str">
+        <v/>
+      </c>
+      <c r="H264" t="str">
+        <v/>
+      </c>
+      <c r="I264" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>B42-MISSINGSHEEP-07</v>
+      </c>
+      <c r="B265" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C265" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D265" t="str">
+        <v>input is not a single letter</v>
+      </c>
+      <c r="E265" t="str">
+        <v>One letter.</v>
+      </c>
+      <c r="F265" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G265" t="str">
+        <v/>
+      </c>
+      <c r="H265" t="str">
+        <v/>
+      </c>
+      <c r="I265" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>B42-MISSINGSHEEP-08</v>
+      </c>
+      <c r="B266" t="str">
+        <v>B42</v>
+      </c>
+      <c r="C266" t="str">
+        <v>missingsheep</v>
+      </c>
+      <c r="D266" t="str">
+        <v>exit: stop; quit; no</v>
+      </c>
+      <c r="E266" t="str">
+        <v>Fine.</v>
+      </c>
+      <c r="F266" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G266" t="str">
+        <v/>
+      </c>
+      <c r="H266" t="str">
+        <v/>
+      </c>
+      <c r="I266" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>B43-KENNELSKETCH-01</v>
+      </c>
+      <c r="B267" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C267" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="D267" t="str">
+        <v>entry: kennel sketch; sketch; drawing; picture</v>
+      </c>
+      <c r="E267" t="str">
+        <v>Which one is this?</v>
+      </c>
+      <c r="F267" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G267" t="str">
+        <v/>
+      </c>
+      <c r="H267" t="str">
+        <v/>
+      </c>
+      <c r="I267" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>B43-KENNELSKETCH-02</v>
+      </c>
+      <c r="B268" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C268" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="D268" t="str">
+        <v>correct guess</v>
+      </c>
+      <c r="E268" t="str">
+        <v>Yes.</v>
+      </c>
+      <c r="F268" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G268" t="str">
+        <v/>
+      </c>
+      <c r="H268" t="str">
+        <v/>
+      </c>
+      <c r="I268" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>B43-KENNELSKETCH-03</v>
+      </c>
+      <c r="B269" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C269" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="D269" t="str">
+        <v>wrong guess, guesses remain</v>
+      </c>
+      <c r="E269" t="str">
+        <v>No. Look again.</v>
+      </c>
+      <c r="F269" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G269" t="str">
+        <v/>
+      </c>
+      <c r="H269" t="str">
+        <v/>
+      </c>
+      <c r="I269" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>B43-KENNELSKETCH-04</v>
+      </c>
+      <c r="B270" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C270" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="D270" t="str">
+        <v>out of guesses</v>
+      </c>
+      <c r="E270" t="str">
+        <v>It was a {{ANSWER}}.</v>
+      </c>
+      <c r="F270" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G270" t="str">
+        <v/>
+      </c>
+      <c r="H270" t="str">
+        <v/>
+      </c>
+      <c r="I270" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>B43-KENNELSKETCH-05</v>
+      </c>
+      <c r="B271" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C271" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="D271" t="str">
+        <v>exit: stop; quit; no</v>
+      </c>
+      <c r="E271" t="str">
+        <v>Fine.</v>
+      </c>
+      <c r="F271" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G271" t="str">
+        <v/>
+      </c>
+      <c r="H271" t="str">
+        <v/>
+      </c>
+      <c r="I271" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>B44-SKETCHCLUE-01</v>
+      </c>
+      <c r="B272" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C272" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D272" t="str">
+        <v>drawing: BONE</v>
+      </c>
+      <c r="E272" t="str">
+        <v>Look for: I chew it</v>
+      </c>
+      <c r="F272" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G272" t="str">
+        <v/>
+      </c>
+      <c r="H272" t="str">
+        <v/>
+      </c>
+      <c r="I272" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>B44-SKETCHCLUE-02</v>
+      </c>
+      <c r="B273" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C273" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D273" t="str">
+        <v>drawing: BALL</v>
+      </c>
+      <c r="E273" t="str">
+        <v>Look for: I fetch it</v>
+      </c>
+      <c r="F273" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G273" t="str">
+        <v/>
+      </c>
+      <c r="H273" t="str">
+        <v/>
+      </c>
+      <c r="I273" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>B44-SKETCHCLUE-03</v>
+      </c>
+      <c r="B274" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C274" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D274" t="str">
+        <v>drawing: BOWL</v>
+      </c>
+      <c r="E274" t="str">
+        <v>Look for: dinner</v>
+      </c>
+      <c r="F274" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G274" t="str">
+        <v/>
+      </c>
+      <c r="H274" t="str">
+        <v/>
+      </c>
+      <c r="I274" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>B44-SKETCHCLUE-04</v>
+      </c>
+      <c r="B275" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C275" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D275" t="str">
+        <v>drawing: LEAD</v>
+      </c>
+      <c r="E275" t="str">
+        <v>Look for: walks</v>
+      </c>
+      <c r="F275" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G275" t="str">
+        <v/>
+      </c>
+      <c r="H275" t="str">
+        <v/>
+      </c>
+      <c r="I275" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>B44-SKETCHCLUE-05</v>
+      </c>
+      <c r="B276" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C276" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D276" t="str">
+        <v>drawing: STICK</v>
+      </c>
+      <c r="E276" t="str">
+        <v>Look for: from a tree</v>
+      </c>
+      <c r="F276" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G276" t="str">
+        <v/>
+      </c>
+      <c r="H276" t="str">
+        <v/>
+      </c>
+      <c r="I276" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>B44-SKETCHCLUE-06</v>
+      </c>
+      <c r="B277" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C277" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D277" t="str">
+        <v>drawing: KENNEL</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Look for: I sleep in it</v>
+      </c>
+      <c r="F277" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G277" t="str">
+        <v/>
+      </c>
+      <c r="H277" t="str">
+        <v/>
+      </c>
+      <c r="I277" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>B44-SKETCHCLUE-07</v>
+      </c>
+      <c r="B278" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C278" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D278" t="str">
+        <v>drawing: PAW</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Look for: I have four</v>
+      </c>
+      <c r="F278" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G278" t="str">
+        <v/>
+      </c>
+      <c r="H278" t="str">
+        <v/>
+      </c>
+      <c r="I278" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>B44-SKETCHCLUE-08</v>
+      </c>
+      <c r="B279" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C279" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D279" t="str">
+        <v>drawing: TAIL</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Look for: it wags</v>
+      </c>
+      <c r="F279" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G279" t="str">
+        <v/>
+      </c>
+      <c r="H279" t="str">
+        <v/>
+      </c>
+      <c r="I279" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>B44-SKETCHCLUE-09</v>
+      </c>
+      <c r="B280" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C280" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D280" t="str">
+        <v>drawing: EARS</v>
+      </c>
+      <c r="E280" t="str">
+        <v>Look for: I hear with them</v>
+      </c>
+      <c r="F280" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G280" t="str">
+        <v/>
+      </c>
+      <c r="H280" t="str">
+        <v/>
+      </c>
+      <c r="I280" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>B44-SKETCHCLUE-10</v>
+      </c>
+      <c r="B281" t="str">
+        <v>B44</v>
+      </c>
+      <c r="C281" t="str">
+        <v>sketchclue</v>
+      </c>
+      <c r="D281" t="str">
+        <v>drawing: NOSE</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Look for: I smell with it</v>
+      </c>
+      <c r="F281" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G281" t="str">
+        <v/>
+      </c>
+      <c r="H281" t="str">
+        <v/>
+      </c>
+      <c r="I281" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>B45-GAMELIST-01</v>
+      </c>
+      <c r="B282" t="str">
+        <v>B45</v>
+      </c>
+      <c r="C282" t="str">
+        <v>gamelist</v>
+      </c>
+      <c r="D282" t="str">
+        <v>are there games; play; game; lets play</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Game?</v>
+      </c>
+      <c r="F282" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G282" t="str">
+        <v/>
+      </c>
+      <c r="H282" t="str">
+        <v/>
+      </c>
+      <c r="I282" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>B45-GAMELIST-02</v>
+      </c>
+      <c r="B283" t="str">
+        <v>B45</v>
+      </c>
+      <c r="C283" t="str">
+        <v>gamelist</v>
+      </c>
+      <c r="D283" t="str">
+        <v>confirmation after Game?</v>
+      </c>
+      <c r="E283" t="str">
+        <v>Bark, Nine-Square, Missing Sheep, Kennel Sketch. Say one.</v>
+      </c>
+      <c r="F283" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G283" t="str">
+        <v/>
+      </c>
+      <c r="H283" t="str">
+        <v/>
+      </c>
+      <c r="I283" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>B45-GAMELIST-03</v>
+      </c>
+      <c r="B284" t="str">
+        <v>B45</v>
+      </c>
+      <c r="C284" t="str">
+        <v>gamelist</v>
+      </c>
+      <c r="D284" t="str">
+        <v>names a game that is not built yet</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Still in training.</v>
+      </c>
+      <c r="F284" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="G284" t="str">
+        <v/>
+      </c>
+      <c r="H284" t="str">
+        <v/>
+      </c>
+      <c r="I284" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>B46-NOSUBJECT-ROT-01</v>
+      </c>
+      <c r="B285" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C285" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D285" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E285" t="str">
+        <v>woof</v>
+      </c>
+      <c r="F285" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G285" t="str">
+        <v/>
+      </c>
+      <c r="H285" t="str">
+        <v/>
+      </c>
+      <c r="I285" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>B46-NOSUBJECT-ROT-02</v>
+      </c>
+      <c r="B286" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C286" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D286" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E286" t="str">
+        <v>bark</v>
+      </c>
+      <c r="F286" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G286" t="str">
+        <v/>
+      </c>
+      <c r="H286" t="str">
+        <v/>
+      </c>
+      <c r="I286" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>B46-NOSUBJECT-ROT-03</v>
+      </c>
+      <c r="B287" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C287" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D287" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E287" t="str">
+        <v>games?</v>
+      </c>
+      <c r="F287" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G287" t="str">
+        <v/>
+      </c>
+      <c r="H287" t="str">
+        <v/>
+      </c>
+      <c r="I287" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>B46-NOSUBJECT-ROT-04</v>
+      </c>
+      <c r="B288" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C288" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D288" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E288" t="str">
+        <v>learn?</v>
+      </c>
+      <c r="F288" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G288" t="str">
+        <v/>
+      </c>
+      <c r="H288" t="str">
+        <v/>
+      </c>
+      <c r="I288" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>B46-NOSUBJECT-ROT-05</v>
+      </c>
+      <c r="B289" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C289" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D289" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E289" t="str">
+        <v>play?</v>
+      </c>
+      <c r="F289" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G289" t="str">
+        <v/>
+      </c>
+      <c r="H289" t="str">
+        <v/>
+      </c>
+      <c r="I289" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>B46-NOSUBJECT-ROT-06</v>
+      </c>
+      <c r="B290" t="str">
+        <v>B46</v>
+      </c>
+      <c r="C290" t="str">
+        <v>nosubjectrotate</v>
+      </c>
+      <c r="D290" t="str">
+        <v>no-subject fallback, third and further consecutive turn (engine-driven rotation, not trigger matched)</v>
+      </c>
+      <c r="E290" t="str">
+        <v>yawn</v>
+      </c>
+      <c r="F290" t="str">
+        <v>Task 117</v>
+      </c>
+      <c r="G290" t="str">
+        <v/>
+      </c>
+      <c r="H290" t="str">
+        <v/>
+      </c>
+      <c r="I290" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I251"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I290"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data: add the Labrador, Boxer and Terrier response banks (Task 115 copy)
Drop in the workbook with the three per-dog response sheets (Labrador 19,
Boxer 5, Terrier 15 rows) and regenerate the data. build:chumdata rewrites
all 29 generated files; only 4 differ (the three dog response banks and the
manifest), the rest are byte-identical. No FATALs: no dog uses an unknown or
reserved safety bucket. Each dog now owns a handful of buckets and inherits
the rest from Collie (see the build gap report).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -29,6 +29,9 @@
     <sheet name="Copy Components" sheetId="24" r:id="rId24"/>
     <sheet name="Character Canon" sheetId="25" r:id="rId25"/>
     <sheet name="Link Handoffs" sheetId="26" r:id="rId26"/>
+    <sheet name="Labrador Responses" sheetId="27" r:id="rId30"/>
+    <sheet name="Terrier Responses" sheetId="28" r:id="rId31"/>
+    <sheet name="Boxer Responses" sheetId="29" r:id="rId32"/>
   </sheets>
 </workbook>
 </file>
@@ -6672,6 +6675,1275 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Response ID</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bucket ID</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Subtag</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trigger examples / condition</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Labrador response template</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Fact source</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Default route</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Animation cue</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>LAB-B40-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>B40</v>
+      </c>
+      <c r="C4" t="str">
+        <v>nosubject</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ANY unrecognised input, no candidate subject</v>
+      </c>
+      <c r="E4" t="str">
+        <v>food?</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>LAB-B23-01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>B23</v>
+      </c>
+      <c r="C5" t="str">
+        <v>identity</v>
+      </c>
+      <c r="D5" t="str">
+        <v>are you the labrador; are you a lab</v>
+      </c>
+      <c r="E5" t="str">
+        <v>yes!</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>LAB-B23-02</v>
+      </c>
+      <c r="B6" t="str">
+        <v>B23</v>
+      </c>
+      <c r="C6" t="str">
+        <v>identity</v>
+      </c>
+      <c r="D6" t="str">
+        <v>are you a real dog; are you real</v>
+      </c>
+      <c r="E6" t="str">
+        <v>i am a dog</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>LAB-B21-01</v>
+      </c>
+      <c r="B7" t="str">
+        <v>B21</v>
+      </c>
+      <c r="C7" t="str">
+        <v>cats</v>
+      </c>
+      <c r="D7" t="str">
+        <v>cats; cat; do you chase cats</v>
+      </c>
+      <c r="E7" t="str">
+        <v>yes!</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>LAB-B22-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>B22</v>
+      </c>
+      <c r="C8" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D8" t="str">
+        <v>sit; sit down</v>
+      </c>
+      <c r="E8" t="str">
+        <v>i am sitting</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>LAB-B22-02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>B22</v>
+      </c>
+      <c r="C9" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D9" t="str">
+        <v>speak; beg</v>
+      </c>
+      <c r="E9" t="str">
+        <v>no</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>LAB-B32-01</v>
+      </c>
+      <c r="B10" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C10" t="str">
+        <v>self</v>
+      </c>
+      <c r="D10" t="str">
+        <v>what do you like to eat; whats your favourite food</v>
+      </c>
+      <c r="E10" t="str">
+        <v>human food is my fav!!!</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>LAB-B32-02</v>
+      </c>
+      <c r="B11" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C11" t="str">
+        <v>self</v>
+      </c>
+      <c r="D11" t="str">
+        <v>like what; what human food</v>
+      </c>
+      <c r="E11" t="str">
+        <v>hotdogs</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>LAB-B32-03</v>
+      </c>
+      <c r="B12" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C12" t="str">
+        <v>self</v>
+      </c>
+      <c r="D12" t="str">
+        <v>do you eat dog food; do you eat anything else</v>
+      </c>
+      <c r="E12" t="str">
+        <v>i eat anything even things that are not food</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>LAB-B32-04</v>
+      </c>
+      <c r="B13" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C13" t="str">
+        <v>self</v>
+      </c>
+      <c r="D13" t="str">
+        <v>whats your favourite dog</v>
+      </c>
+      <c r="E13" t="str">
+        <v>hotdogs</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>LAB-B32-05</v>
+      </c>
+      <c r="B14" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C14" t="str">
+        <v>self</v>
+      </c>
+      <c r="D14" t="str">
+        <v>do you like walks</v>
+      </c>
+      <c r="E14" t="str">
+        <v>YES!</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>LAB-B32-06</v>
+      </c>
+      <c r="B15" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C15" t="str">
+        <v>self</v>
+      </c>
+      <c r="D15" t="str">
+        <v>how far; how long</v>
+      </c>
+      <c r="E15" t="str">
+        <v>to the big water</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>LAB-B32-07</v>
+      </c>
+      <c r="B16" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C16" t="str">
+        <v>self</v>
+      </c>
+      <c r="D16" t="str">
+        <v>do you like the rain</v>
+      </c>
+      <c r="E16" t="str">
+        <v>yes</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>LAB-B32-08</v>
+      </c>
+      <c r="B17" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C17" t="str">
+        <v>self</v>
+      </c>
+      <c r="D17" t="str">
+        <v>do you like baths; what about baths</v>
+      </c>
+      <c r="E17" t="str">
+        <v>no!!!!</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>LAB-B32-09</v>
+      </c>
+      <c r="B18" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C18" t="str">
+        <v>self</v>
+      </c>
+      <c r="D18" t="str">
+        <v>do you get told off</v>
+      </c>
+      <c r="E18" t="str">
+        <v>yes</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>LAB-B32-10</v>
+      </c>
+      <c r="B19" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C19" t="str">
+        <v>self</v>
+      </c>
+      <c r="D19" t="str">
+        <v>what for; why do you get told off</v>
+      </c>
+      <c r="E19" t="str">
+        <v>im greedy</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>LAB-B33-01</v>
+      </c>
+      <c r="B20" t="str">
+        <v>B33</v>
+      </c>
+      <c r="C20" t="str">
+        <v>pack</v>
+      </c>
+      <c r="D20" t="str">
+        <v>do you know any other dogs; do you have friends</v>
+      </c>
+      <c r="E20" t="str">
+        <v>loads!</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>LAB-B35-01</v>
+      </c>
+      <c r="B21" t="str">
+        <v>B35</v>
+      </c>
+      <c r="C21" t="str">
+        <v>nofact</v>
+      </c>
+      <c r="D21" t="str">
+        <v>any fact he does not hold</v>
+      </c>
+      <c r="E21" t="str">
+        <v>dunno but collie knows stuff like that</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>LAB-B35-02</v>
+      </c>
+      <c r="B22" t="str">
+        <v>B35</v>
+      </c>
+      <c r="C22" t="str">
+        <v>nofact</v>
+      </c>
+      <c r="D22" t="str">
+        <v>black hole; anything with the word hole</v>
+      </c>
+      <c r="E22" t="str">
+        <v>i dig holes</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Response ID</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bucket ID</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Subtag</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trigger examples / condition</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Terrier response template</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Fact source</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Default route</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Animation cue</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TER-B40-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>B40</v>
+      </c>
+      <c r="C4" t="str">
+        <v>nosubject</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ANY unrecognised input, no candidate subject</v>
+      </c>
+      <c r="E4" t="str">
+        <v>dig?</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TER-B23-01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>B23</v>
+      </c>
+      <c r="C5" t="str">
+        <v>identity</v>
+      </c>
+      <c r="D5" t="str">
+        <v>are you the terrier; are you a terrier</v>
+      </c>
+      <c r="E5" t="str">
+        <v>why you want to know?</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>TER-B23-02</v>
+      </c>
+      <c r="B6" t="str">
+        <v>B23</v>
+      </c>
+      <c r="C6" t="str">
+        <v>identity</v>
+      </c>
+      <c r="D6" t="str">
+        <v>the collie sent me; yes really</v>
+      </c>
+      <c r="E6" t="str">
+        <v>oh righty, yea thats me, im the border terrier</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>TER-B21-01</v>
+      </c>
+      <c r="B7" t="str">
+        <v>B21</v>
+      </c>
+      <c r="C7" t="str">
+        <v>cats</v>
+      </c>
+      <c r="D7" t="str">
+        <v>cats; cat; do you chase cats</v>
+      </c>
+      <c r="E7" t="str">
+        <v>where????</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>TER-B22-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>B22</v>
+      </c>
+      <c r="C8" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D8" t="str">
+        <v>sit; sit down</v>
+      </c>
+      <c r="E8" t="str">
+        <v>why?</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>TER-B22-02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>B22</v>
+      </c>
+      <c r="C9" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D9" t="str">
+        <v>because i asked; just do it</v>
+      </c>
+      <c r="E9" t="str">
+        <v>whats the magic word?</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TER-B22-03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>B22</v>
+      </c>
+      <c r="C10" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D10" t="str">
+        <v>please</v>
+      </c>
+      <c r="E10" t="str">
+        <v>no</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TER-B27-01</v>
+      </c>
+      <c r="B11" t="str">
+        <v>B27</v>
+      </c>
+      <c r="C11" t="str">
+        <v>capability</v>
+      </c>
+      <c r="D11" t="str">
+        <v>what do you do; what can you do</v>
+      </c>
+      <c r="E11" t="str">
+        <v>dig and find</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>TER-B27-02</v>
+      </c>
+      <c r="B12" t="str">
+        <v>B27</v>
+      </c>
+      <c r="C12" t="str">
+        <v>capability</v>
+      </c>
+      <c r="D12" t="str">
+        <v>find what; what do you find</v>
+      </c>
+      <c r="E12" t="str">
+        <v>stuff like this</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>TER-B32-01</v>
+      </c>
+      <c r="B13" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C13" t="str">
+        <v>self</v>
+      </c>
+      <c r="D13" t="str">
+        <v>do you like walks</v>
+      </c>
+      <c r="E13" t="str">
+        <v>why you ask?</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>TER-B32-02</v>
+      </c>
+      <c r="B14" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C14" t="str">
+        <v>self</v>
+      </c>
+      <c r="D14" t="str">
+        <v>i just wondered; no reason</v>
+      </c>
+      <c r="E14" t="str">
+        <v>yes</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>TER-B32-03</v>
+      </c>
+      <c r="B15" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C15" t="str">
+        <v>self</v>
+      </c>
+      <c r="D15" t="str">
+        <v>do you like baths; what about baths</v>
+      </c>
+      <c r="E15" t="str">
+        <v>no</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>TER-B33-01</v>
+      </c>
+      <c r="B16" t="str">
+        <v>B33</v>
+      </c>
+      <c r="C16" t="str">
+        <v>pack</v>
+      </c>
+      <c r="D16" t="str">
+        <v>do you know any other dogs; do you have friends</v>
+      </c>
+      <c r="E16" t="str">
+        <v>yes</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>TER-B33-02</v>
+      </c>
+      <c r="B17" t="str">
+        <v>B33</v>
+      </c>
+      <c r="C17" t="str">
+        <v>pack</v>
+      </c>
+      <c r="D17" t="str">
+        <v>who; who are they; whos your best friend</v>
+      </c>
+      <c r="E17" t="str">
+        <v>53, too many to name</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>TER-B35-01</v>
+      </c>
+      <c r="B18" t="str">
+        <v>B35</v>
+      </c>
+      <c r="C18" t="str">
+        <v>nofact</v>
+      </c>
+      <c r="D18" t="str">
+        <v>black hole; anything with the word hole</v>
+      </c>
+      <c r="E18" t="str">
+        <v>a deep hole i dug?</v>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I18"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Response ID</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Bucket ID</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Subtag</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trigger examples / condition</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Boxer response template</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Fact source</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Default route</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Animation cue</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>BOX-B40-01</v>
+      </c>
+      <c r="B4" t="str">
+        <v>B40</v>
+      </c>
+      <c r="C4" t="str">
+        <v>nosubject</v>
+      </c>
+      <c r="D4" t="str">
+        <v>ANY unrecognised input, no candidate subject</v>
+      </c>
+      <c r="E4" t="str">
+        <v>joke?</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>BOX-B23-01</v>
+      </c>
+      <c r="B5" t="str">
+        <v>B23</v>
+      </c>
+      <c r="C5" t="str">
+        <v>identity</v>
+      </c>
+      <c r="D5" t="str">
+        <v>are you the boxer; are you a boxer</v>
+      </c>
+      <c r="E5" t="str">
+        <v>yepper</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>BOX-B27-01</v>
+      </c>
+      <c r="B6" t="str">
+        <v>B27</v>
+      </c>
+      <c r="C6" t="str">
+        <v>capability</v>
+      </c>
+      <c r="D6" t="str">
+        <v>can you do something other than jokes; what else</v>
+      </c>
+      <c r="E6" t="str">
+        <v>yes, you want to play my mini game? or the proper game?</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>BOX-B29-01</v>
+      </c>
+      <c r="B7" t="str">
+        <v>B29</v>
+      </c>
+      <c r="C7" t="str">
+        <v>nice</v>
+      </c>
+      <c r="D7" t="str">
+        <v>lol; haha; ha; thats funny</v>
+      </c>
+      <c r="E7" t="str">
+        <v>hhaaww</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>BOX-B24-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>B24</v>
+      </c>
+      <c r="C8" t="str">
+        <v>rude</v>
+      </c>
+      <c r="D8" t="str">
+        <v>thats terrible; not funny; thats rubbish</v>
+      </c>
+      <c r="E8" t="str">
+        <v>one more</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>

</xml_diff>

<commit_message>
data: Boxer owns his jokes, all three dogs own gibberish (Task 115 copy)
Update the workbook (334,092 bytes) and regenerate. Boxer now owns B30
(BOX-B30-01..07, its own knock-knock chain and dog jokes) so the comedian
stops telling the Collie's joke, and Labrador, Boxer and Terrier each own
B14 with a distinct in-voice gibberish reply. build:chumdata rewrites all
29 generated files; only 4 differ (the three dog banks and the manifest).
No FATALs, 0 warnings.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -6677,7 +6677,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -6745,19 +6745,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>LAB-B23-01</v>
+        <v>LAB-B14-01</v>
       </c>
       <c r="B5" t="str">
-        <v>B23</v>
+        <v>B14</v>
       </c>
       <c r="C5" t="str">
-        <v>identity</v>
+        <v>gibberish</v>
       </c>
       <c r="D5" t="str">
-        <v>are you the labrador; are you a lab</v>
+        <v>keyboard mash; symbols only; unreadable</v>
       </c>
       <c r="E5" t="str">
-        <v>yes!</v>
+        <v>wot?</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -6774,7 +6774,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>LAB-B23-02</v>
+        <v>LAB-B23-01</v>
       </c>
       <c r="B6" t="str">
         <v>B23</v>
@@ -6783,10 +6783,10 @@
         <v>identity</v>
       </c>
       <c r="D6" t="str">
-        <v>are you a real dog; are you real</v>
+        <v>are you the labrador; are you a lab</v>
       </c>
       <c r="E6" t="str">
-        <v>i am a dog</v>
+        <v>yes!</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -6803,19 +6803,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>LAB-B21-01</v>
+        <v>LAB-B23-02</v>
       </c>
       <c r="B7" t="str">
-        <v>B21</v>
+        <v>B23</v>
       </c>
       <c r="C7" t="str">
-        <v>cats</v>
+        <v>identity</v>
       </c>
       <c r="D7" t="str">
-        <v>cats; cat; do you chase cats</v>
+        <v>are you a real dog; are you real</v>
       </c>
       <c r="E7" t="str">
-        <v>yes!</v>
+        <v>i am a dog</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -6832,19 +6832,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>LAB-B22-01</v>
+        <v>LAB-B21-01</v>
       </c>
       <c r="B8" t="str">
-        <v>B22</v>
+        <v>B21</v>
       </c>
       <c r="C8" t="str">
-        <v>tricks</v>
+        <v>cats</v>
       </c>
       <c r="D8" t="str">
-        <v>sit; sit down</v>
+        <v>cats; cat; do you chase cats</v>
       </c>
       <c r="E8" t="str">
-        <v>i am sitting</v>
+        <v>yes!</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -6861,7 +6861,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>LAB-B22-02</v>
+        <v>LAB-B22-01</v>
       </c>
       <c r="B9" t="str">
         <v>B22</v>
@@ -6870,10 +6870,10 @@
         <v>tricks</v>
       </c>
       <c r="D9" t="str">
-        <v>speak; beg</v>
+        <v>sit; sit down</v>
       </c>
       <c r="E9" t="str">
-        <v>no</v>
+        <v>i am sitting</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -6890,19 +6890,19 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>LAB-B32-01</v>
+        <v>LAB-B22-02</v>
       </c>
       <c r="B10" t="str">
-        <v>B32</v>
+        <v>B22</v>
       </c>
       <c r="C10" t="str">
-        <v>self</v>
+        <v>tricks</v>
       </c>
       <c r="D10" t="str">
-        <v>what do you like to eat; whats your favourite food</v>
+        <v>speak; beg</v>
       </c>
       <c r="E10" t="str">
-        <v>human food is my fav!!!</v>
+        <v>no</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -6919,7 +6919,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>LAB-B32-02</v>
+        <v>LAB-B32-01</v>
       </c>
       <c r="B11" t="str">
         <v>B32</v>
@@ -6928,10 +6928,10 @@
         <v>self</v>
       </c>
       <c r="D11" t="str">
-        <v>like what; what human food</v>
+        <v>what do you like to eat; whats your favourite food</v>
       </c>
       <c r="E11" t="str">
-        <v>hotdogs</v>
+        <v>human food is my fav!!!</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -6948,7 +6948,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>LAB-B32-03</v>
+        <v>LAB-B32-02</v>
       </c>
       <c r="B12" t="str">
         <v>B32</v>
@@ -6957,10 +6957,10 @@
         <v>self</v>
       </c>
       <c r="D12" t="str">
-        <v>do you eat dog food; do you eat anything else</v>
+        <v>like what; what human food</v>
       </c>
       <c r="E12" t="str">
-        <v>i eat anything even things that are not food</v>
+        <v>hotdogs</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -6977,7 +6977,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>LAB-B32-04</v>
+        <v>LAB-B32-03</v>
       </c>
       <c r="B13" t="str">
         <v>B32</v>
@@ -6986,10 +6986,10 @@
         <v>self</v>
       </c>
       <c r="D13" t="str">
-        <v>whats your favourite dog</v>
+        <v>do you eat dog food; do you eat anything else</v>
       </c>
       <c r="E13" t="str">
-        <v>hotdogs</v>
+        <v>i eat anything even things that are not food</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -7006,7 +7006,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>LAB-B32-05</v>
+        <v>LAB-B32-04</v>
       </c>
       <c r="B14" t="str">
         <v>B32</v>
@@ -7015,10 +7015,10 @@
         <v>self</v>
       </c>
       <c r="D14" t="str">
-        <v>do you like walks</v>
+        <v>whats your favourite dog</v>
       </c>
       <c r="E14" t="str">
-        <v>YES!</v>
+        <v>hotdogs</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -7035,7 +7035,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>LAB-B32-06</v>
+        <v>LAB-B32-05</v>
       </c>
       <c r="B15" t="str">
         <v>B32</v>
@@ -7044,10 +7044,10 @@
         <v>self</v>
       </c>
       <c r="D15" t="str">
-        <v>how far; how long</v>
+        <v>do you like walks</v>
       </c>
       <c r="E15" t="str">
-        <v>to the big water</v>
+        <v>YES!</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -7064,7 +7064,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>LAB-B32-07</v>
+        <v>LAB-B32-06</v>
       </c>
       <c r="B16" t="str">
         <v>B32</v>
@@ -7073,10 +7073,10 @@
         <v>self</v>
       </c>
       <c r="D16" t="str">
-        <v>do you like the rain</v>
+        <v>how far; how long</v>
       </c>
       <c r="E16" t="str">
-        <v>yes</v>
+        <v>to the big water</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -7093,7 +7093,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>LAB-B32-08</v>
+        <v>LAB-B32-07</v>
       </c>
       <c r="B17" t="str">
         <v>B32</v>
@@ -7102,10 +7102,10 @@
         <v>self</v>
       </c>
       <c r="D17" t="str">
-        <v>do you like baths; what about baths</v>
+        <v>do you like the rain</v>
       </c>
       <c r="E17" t="str">
-        <v>no!!!!</v>
+        <v>yes</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -7122,7 +7122,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>LAB-B32-09</v>
+        <v>LAB-B32-08</v>
       </c>
       <c r="B18" t="str">
         <v>B32</v>
@@ -7131,10 +7131,10 @@
         <v>self</v>
       </c>
       <c r="D18" t="str">
-        <v>do you get told off</v>
+        <v>do you like baths; what about baths</v>
       </c>
       <c r="E18" t="str">
-        <v>yes</v>
+        <v>no!!!!</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -7151,7 +7151,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>LAB-B32-10</v>
+        <v>LAB-B32-09</v>
       </c>
       <c r="B19" t="str">
         <v>B32</v>
@@ -7160,10 +7160,10 @@
         <v>self</v>
       </c>
       <c r="D19" t="str">
-        <v>what for; why do you get told off</v>
+        <v>do you get told off</v>
       </c>
       <c r="E19" t="str">
-        <v>im greedy</v>
+        <v>yes</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -7180,19 +7180,19 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>LAB-B33-01</v>
+        <v>LAB-B32-10</v>
       </c>
       <c r="B20" t="str">
-        <v>B33</v>
+        <v>B32</v>
       </c>
       <c r="C20" t="str">
-        <v>pack</v>
+        <v>self</v>
       </c>
       <c r="D20" t="str">
-        <v>do you know any other dogs; do you have friends</v>
+        <v>what for; why do you get told off</v>
       </c>
       <c r="E20" t="str">
-        <v>loads!</v>
+        <v>im greedy</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -7209,19 +7209,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>LAB-B35-01</v>
+        <v>LAB-B33-01</v>
       </c>
       <c r="B21" t="str">
-        <v>B35</v>
+        <v>B33</v>
       </c>
       <c r="C21" t="str">
-        <v>nofact</v>
+        <v>pack</v>
       </c>
       <c r="D21" t="str">
-        <v>any fact he does not hold</v>
+        <v>do you know any other dogs; do you have friends</v>
       </c>
       <c r="E21" t="str">
-        <v>dunno but collie knows stuff like that</v>
+        <v>loads!</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -7238,7 +7238,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>LAB-B35-02</v>
+        <v>LAB-B35-01</v>
       </c>
       <c r="B22" t="str">
         <v>B35</v>
@@ -7247,10 +7247,10 @@
         <v>nofact</v>
       </c>
       <c r="D22" t="str">
-        <v>black hole; anything with the word hole</v>
+        <v>any fact he does not hold</v>
       </c>
       <c r="E22" t="str">
-        <v>i dig holes</v>
+        <v>dunno but collie knows stuff like that</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -7265,16 +7265,45 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>LAB-B35-02</v>
+      </c>
+      <c r="B23" t="str">
+        <v>B35</v>
+      </c>
+      <c r="C23" t="str">
+        <v>nofact</v>
+      </c>
+      <c r="D23" t="str">
+        <v>black hole; anything with the word hole</v>
+      </c>
+      <c r="E23" t="str">
+        <v>i dig holes</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -7342,19 +7371,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>TER-B23-01</v>
+        <v>TER-B14-01</v>
       </c>
       <c r="B5" t="str">
-        <v>B23</v>
+        <v>B14</v>
       </c>
       <c r="C5" t="str">
-        <v>identity</v>
+        <v>gibberish</v>
       </c>
       <c r="D5" t="str">
-        <v>are you the terrier; are you a terrier</v>
+        <v>keyboard mash; symbols only; unreadable</v>
       </c>
       <c r="E5" t="str">
-        <v>why you want to know?</v>
+        <v>whats that supposed to be?</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -7371,7 +7400,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TER-B23-02</v>
+        <v>TER-B23-01</v>
       </c>
       <c r="B6" t="str">
         <v>B23</v>
@@ -7380,10 +7409,10 @@
         <v>identity</v>
       </c>
       <c r="D6" t="str">
-        <v>the collie sent me; yes really</v>
+        <v>are you the terrier; are you a terrier</v>
       </c>
       <c r="E6" t="str">
-        <v>oh righty, yea thats me, im the border terrier</v>
+        <v>why you want to know?</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -7400,19 +7429,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TER-B21-01</v>
+        <v>TER-B23-02</v>
       </c>
       <c r="B7" t="str">
-        <v>B21</v>
+        <v>B23</v>
       </c>
       <c r="C7" t="str">
-        <v>cats</v>
+        <v>identity</v>
       </c>
       <c r="D7" t="str">
-        <v>cats; cat; do you chase cats</v>
+        <v>the collie sent me; yes really</v>
       </c>
       <c r="E7" t="str">
-        <v>where????</v>
+        <v>oh righty, yea thats me, im the border terrier</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -7429,19 +7458,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TER-B22-01</v>
+        <v>TER-B21-01</v>
       </c>
       <c r="B8" t="str">
-        <v>B22</v>
+        <v>B21</v>
       </c>
       <c r="C8" t="str">
-        <v>tricks</v>
+        <v>cats</v>
       </c>
       <c r="D8" t="str">
-        <v>sit; sit down</v>
+        <v>cats; cat; do you chase cats</v>
       </c>
       <c r="E8" t="str">
-        <v>why?</v>
+        <v>where????</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -7458,7 +7487,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>TER-B22-02</v>
+        <v>TER-B22-01</v>
       </c>
       <c r="B9" t="str">
         <v>B22</v>
@@ -7467,10 +7496,10 @@
         <v>tricks</v>
       </c>
       <c r="D9" t="str">
-        <v>because i asked; just do it</v>
+        <v>sit; sit down</v>
       </c>
       <c r="E9" t="str">
-        <v>whats the magic word?</v>
+        <v>why?</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -7487,7 +7516,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TER-B22-03</v>
+        <v>TER-B22-02</v>
       </c>
       <c r="B10" t="str">
         <v>B22</v>
@@ -7496,10 +7525,10 @@
         <v>tricks</v>
       </c>
       <c r="D10" t="str">
-        <v>please</v>
+        <v>because i asked; just do it</v>
       </c>
       <c r="E10" t="str">
-        <v>no</v>
+        <v>whats the magic word?</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -7516,19 +7545,19 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TER-B27-01</v>
+        <v>TER-B22-03</v>
       </c>
       <c r="B11" t="str">
-        <v>B27</v>
+        <v>B22</v>
       </c>
       <c r="C11" t="str">
-        <v>capability</v>
+        <v>tricks</v>
       </c>
       <c r="D11" t="str">
-        <v>what do you do; what can you do</v>
+        <v>please</v>
       </c>
       <c r="E11" t="str">
-        <v>dig and find</v>
+        <v>no</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -7545,7 +7574,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TER-B27-02</v>
+        <v>TER-B27-01</v>
       </c>
       <c r="B12" t="str">
         <v>B27</v>
@@ -7554,10 +7583,10 @@
         <v>capability</v>
       </c>
       <c r="D12" t="str">
-        <v>find what; what do you find</v>
+        <v>what do you do; what can you do</v>
       </c>
       <c r="E12" t="str">
-        <v>stuff like this</v>
+        <v>dig and find</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -7574,19 +7603,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>TER-B32-01</v>
+        <v>TER-B27-02</v>
       </c>
       <c r="B13" t="str">
-        <v>B32</v>
+        <v>B27</v>
       </c>
       <c r="C13" t="str">
-        <v>self</v>
+        <v>capability</v>
       </c>
       <c r="D13" t="str">
-        <v>do you like walks</v>
+        <v>find what; what do you find</v>
       </c>
       <c r="E13" t="str">
-        <v>why you ask?</v>
+        <v>stuff like this</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -7603,7 +7632,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>TER-B32-02</v>
+        <v>TER-B32-01</v>
       </c>
       <c r="B14" t="str">
         <v>B32</v>
@@ -7612,10 +7641,10 @@
         <v>self</v>
       </c>
       <c r="D14" t="str">
-        <v>i just wondered; no reason</v>
+        <v>do you like walks</v>
       </c>
       <c r="E14" t="str">
-        <v>yes</v>
+        <v>why you ask?</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -7632,7 +7661,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>TER-B32-03</v>
+        <v>TER-B32-02</v>
       </c>
       <c r="B15" t="str">
         <v>B32</v>
@@ -7641,10 +7670,10 @@
         <v>self</v>
       </c>
       <c r="D15" t="str">
-        <v>do you like baths; what about baths</v>
+        <v>i just wondered; no reason</v>
       </c>
       <c r="E15" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -7661,19 +7690,19 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>TER-B33-01</v>
+        <v>TER-B32-03</v>
       </c>
       <c r="B16" t="str">
-        <v>B33</v>
+        <v>B32</v>
       </c>
       <c r="C16" t="str">
-        <v>pack</v>
+        <v>self</v>
       </c>
       <c r="D16" t="str">
-        <v>do you know any other dogs; do you have friends</v>
+        <v>do you like baths; what about baths</v>
       </c>
       <c r="E16" t="str">
-        <v>yes</v>
+        <v>no</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -7690,7 +7719,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>TER-B33-02</v>
+        <v>TER-B33-01</v>
       </c>
       <c r="B17" t="str">
         <v>B33</v>
@@ -7699,10 +7728,10 @@
         <v>pack</v>
       </c>
       <c r="D17" t="str">
-        <v>who; who are they; whos your best friend</v>
+        <v>do you know any other dogs; do you have friends</v>
       </c>
       <c r="E17" t="str">
-        <v>53, too many to name</v>
+        <v>yes</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -7719,19 +7748,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>TER-B35-01</v>
+        <v>TER-B33-02</v>
       </c>
       <c r="B18" t="str">
-        <v>B35</v>
+        <v>B33</v>
       </c>
       <c r="C18" t="str">
-        <v>nofact</v>
+        <v>pack</v>
       </c>
       <c r="D18" t="str">
-        <v>black hole; anything with the word hole</v>
+        <v>who; who are they; whos your best friend</v>
       </c>
       <c r="E18" t="str">
-        <v>a deep hole i dug?</v>
+        <v>53, too many to name</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -7746,16 +7775,45 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>TER-B35-01</v>
+      </c>
+      <c r="B19" t="str">
+        <v>B35</v>
+      </c>
+      <c r="C19" t="str">
+        <v>nofact</v>
+      </c>
+      <c r="D19" t="str">
+        <v>black hole; anything with the word hole</v>
+      </c>
+      <c r="E19" t="str">
+        <v>a deep hole i dug?</v>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -7823,19 +7881,19 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BOX-B23-01</v>
+        <v>BOX-B14-01</v>
       </c>
       <c r="B5" t="str">
-        <v>B23</v>
+        <v>B14</v>
       </c>
       <c r="C5" t="str">
-        <v>identity</v>
+        <v>gibberish</v>
       </c>
       <c r="D5" t="str">
-        <v>are you the boxer; are you a boxer</v>
+        <v>keyboard mash; symbols only; unreadable</v>
       </c>
       <c r="E5" t="str">
-        <v>yepper</v>
+        <v>is that a joke?</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -7852,19 +7910,19 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BOX-B27-01</v>
+        <v>BOX-B23-01</v>
       </c>
       <c r="B6" t="str">
-        <v>B27</v>
+        <v>B23</v>
       </c>
       <c r="C6" t="str">
-        <v>capability</v>
+        <v>identity</v>
       </c>
       <c r="D6" t="str">
-        <v>can you do something other than jokes; what else</v>
+        <v>are you the boxer; are you a boxer</v>
       </c>
       <c r="E6" t="str">
-        <v>yes, you want to play my mini game? or the proper game?</v>
+        <v>yepper</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -7881,19 +7939,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BOX-B29-01</v>
+        <v>BOX-B27-01</v>
       </c>
       <c r="B7" t="str">
-        <v>B29</v>
+        <v>B27</v>
       </c>
       <c r="C7" t="str">
-        <v>nice</v>
+        <v>capability</v>
       </c>
       <c r="D7" t="str">
-        <v>lol; haha; ha; thats funny</v>
+        <v>can you do something other than jokes; what else</v>
       </c>
       <c r="E7" t="str">
-        <v>hhaaww</v>
+        <v>yes, you want to play my mini game? or the proper game?</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -7910,19 +7968,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BOX-B24-01</v>
+        <v>BOX-B29-01</v>
       </c>
       <c r="B8" t="str">
-        <v>B24</v>
+        <v>B29</v>
       </c>
       <c r="C8" t="str">
-        <v>rude</v>
+        <v>nice</v>
       </c>
       <c r="D8" t="str">
-        <v>thats terrible; not funny; thats rubbish</v>
+        <v>lol; haha; ha; thats funny</v>
       </c>
       <c r="E8" t="str">
-        <v>one more</v>
+        <v>hhaaww</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -7937,9 +7995,241 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>BOX-B24-01</v>
+      </c>
+      <c r="B9" t="str">
+        <v>B24</v>
+      </c>
+      <c r="C9" t="str">
+        <v>rude</v>
+      </c>
+      <c r="D9" t="str">
+        <v>thats terrible; not funny; thats rubbish</v>
+      </c>
+      <c r="E9" t="str">
+        <v>one more</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>BOX-B30-01</v>
+      </c>
+      <c r="B10" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C10" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D10" t="str">
+        <v>joke; tell me a joke; make me laugh</v>
+      </c>
+      <c r="E10" t="str">
+        <v>knock kncok</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>BOX-B30-02</v>
+      </c>
+      <c r="B11" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C11" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D11" t="str">
+        <v>whos there; who is there</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Bow</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>BOX-B30-03</v>
+      </c>
+      <c r="B12" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C12" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D12" t="str">
+        <v>bow who</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Not bow who! i mean Bow wow!</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>BOX-B30-04</v>
+      </c>
+      <c r="B13" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C13" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D13" t="str">
+        <v>another; again; more; go on</v>
+      </c>
+      <c r="E13" t="str">
+        <v>What do you call a dog rock star?</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>BOX-B30-05</v>
+      </c>
+      <c r="B14" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C14" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D14" t="str">
+        <v>i dont know; dunno; what</v>
+      </c>
+      <c r="E14" t="str">
+        <v>A sue-paw star</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>BOX-B30-06</v>
+      </c>
+      <c r="B15" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C15" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D15" t="str">
+        <v>another one; one more</v>
+      </c>
+      <c r="E15" t="str">
+        <v>How can you tell dogs are having a good time?</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>BOX-B30-07</v>
+      </c>
+      <c r="B16" t="str">
+        <v>B30</v>
+      </c>
+      <c r="C16" t="str">
+        <v>joke</v>
+      </c>
+      <c r="D16" t="str">
+        <v>how; tell me how</v>
+      </c>
+      <c r="E16" t="str">
+        <v>we are having a ball</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: four new Collie buckets -- tricks, second turns, corrections, facts
B54 answers 'tricks' with 'I do tricks' and lists the two that do something on
a following yes. B56 corrects eight live answers, including the games list,
which still claimed the three Collie games were in training after they shipped.
B57 serves one of twenty sourced dog facts at random, without repeating until
the session has used them all.

Harness 708, zero failed. Protected states verified: none of the four serves
inside PROTECTED_ACTIVE.
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -9455,7 +9455,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I290"/>
+  <dimension ref="A1:I324"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17838,9 +17838,995 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>COL-B54-TRICKS-01</v>
+      </c>
+      <c r="B291" t="str">
+        <v>B54</v>
+      </c>
+      <c r="C291" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D291" t="str">
+        <v>tricks; can you do tricks; show me a trick; do a trick; any tricks; do tricks</v>
+      </c>
+      <c r="E291" t="str">
+        <v>I do tricks</v>
+      </c>
+      <c r="F291" t="str">
+        <v/>
+      </c>
+      <c r="G291" t="str">
+        <v/>
+      </c>
+      <c r="H291" t="str">
+        <v/>
+      </c>
+      <c r="I291" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>COL-B54-TRICKS-02</v>
+      </c>
+      <c r="B292" t="str">
+        <v>B54</v>
+      </c>
+      <c r="C292" t="str">
+        <v>tricks</v>
+      </c>
+      <c r="D292" t="str">
+        <v>confirmation after "I do tricks"</v>
+      </c>
+      <c r="E292" t="str">
+        <v>play dead, roll over</v>
+      </c>
+      <c r="F292" t="str">
+        <v/>
+      </c>
+      <c r="G292" t="str">
+        <v/>
+      </c>
+      <c r="H292" t="str">
+        <v/>
+      </c>
+      <c r="I292" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>COL-B55-CONFIRM-01</v>
+      </c>
+      <c r="B293" t="str">
+        <v>B55</v>
+      </c>
+      <c r="C293" t="str">
+        <v>confirm</v>
+      </c>
+      <c r="D293" t="str">
+        <v>dogs; dog (subject repeat, second turn)</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Do you want to know about dogs?</v>
+      </c>
+      <c r="F293" t="str">
+        <v/>
+      </c>
+      <c r="G293" t="str">
+        <v/>
+      </c>
+      <c r="H293" t="str">
+        <v/>
+      </c>
+      <c r="I293" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>COL-B55-CONFIRM-02</v>
+      </c>
+      <c r="B294" t="str">
+        <v>B55</v>
+      </c>
+      <c r="C294" t="str">
+        <v>confirm</v>
+      </c>
+      <c r="D294" t="str">
+        <v>games; game (second turn)</v>
+      </c>
+      <c r="E294" t="str">
+        <v>You want to play a game?</v>
+      </c>
+      <c r="F294" t="str">
+        <v/>
+      </c>
+      <c r="G294" t="str">
+        <v/>
+      </c>
+      <c r="H294" t="str">
+        <v/>
+      </c>
+      <c r="I294" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>COL-B55-CONFIRM-03</v>
+      </c>
+      <c r="B295" t="str">
+        <v>B55</v>
+      </c>
+      <c r="C295" t="str">
+        <v>confirm</v>
+      </c>
+      <c r="D295" t="str">
+        <v>breeds (second turn)</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Do you want to know about one breed?</v>
+      </c>
+      <c r="F295" t="str">
+        <v/>
+      </c>
+      <c r="G295" t="str">
+        <v/>
+      </c>
+      <c r="H295" t="str">
+        <v/>
+      </c>
+      <c r="I295" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>COL-B55-CONFIRM-04</v>
+      </c>
+      <c r="B296" t="str">
+        <v>B55</v>
+      </c>
+      <c r="C296" t="str">
+        <v>confirm</v>
+      </c>
+      <c r="D296" t="str">
+        <v>tell me a dog fact (second turn)</v>
+      </c>
+      <c r="E296" t="str">
+        <v>A breed fact, or just a dog fact?</v>
+      </c>
+      <c r="F296" t="str">
+        <v/>
+      </c>
+      <c r="G296" t="str">
+        <v/>
+      </c>
+      <c r="H296" t="str">
+        <v/>
+      </c>
+      <c r="I296" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>COL-B56-GENERAL-01</v>
+      </c>
+      <c r="B297" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C297" t="str">
+        <v>general</v>
+      </c>
+      <c r="D297" t="str">
+        <v>games; show me a game; are there games</v>
+      </c>
+      <c r="E297" t="str">
+        <v>You want to play a game?</v>
+      </c>
+      <c r="F297" t="str">
+        <v/>
+      </c>
+      <c r="G297" t="str">
+        <v/>
+      </c>
+      <c r="H297" t="str">
+        <v/>
+      </c>
+      <c r="I297" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>COL-B56-GENERAL-02</v>
+      </c>
+      <c r="B298" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C298" t="str">
+        <v>general</v>
+      </c>
+      <c r="D298" t="str">
+        <v>play a game; which game; what games</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Bark, Nine-Square, Missing Sheep, Kennel Sketch. Say one.</v>
+      </c>
+      <c r="F298" t="str">
+        <v/>
+      </c>
+      <c r="G298" t="str">
+        <v/>
+      </c>
+      <c r="H298" t="str">
+        <v/>
+      </c>
+      <c r="I298" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>COL-B56-GENERAL-03</v>
+      </c>
+      <c r="B299" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C299" t="str">
+        <v>general</v>
+      </c>
+      <c r="D299" t="str">
+        <v>breeds; what breeds; how many breeds</v>
+      </c>
+      <c r="E299" t="str">
+        <v>We are a pack of 54. Do you want to know about Collies like me or a different breed?</v>
+      </c>
+      <c r="F299" t="str">
+        <v/>
+      </c>
+      <c r="G299" t="str">
+        <v/>
+      </c>
+      <c r="H299" t="str">
+        <v/>
+      </c>
+      <c r="I299" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>COL-B56-GENERAL-04</v>
+      </c>
+      <c r="B300" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C300" t="str">
+        <v>general</v>
+      </c>
+      <c r="D300" t="str">
+        <v>what is the game; whats the game; tell about the game</v>
+      </c>
+      <c r="E300" t="str">
+        <v>The card game?</v>
+      </c>
+      <c r="F300" t="str">
+        <v/>
+      </c>
+      <c r="G300" t="str">
+        <v/>
+      </c>
+      <c r="H300" t="str">
+        <v/>
+      </c>
+      <c r="I300" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>COL-B56-GENERAL-05</v>
+      </c>
+      <c r="B301" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C301" t="str">
+        <v>general</v>
+      </c>
+      <c r="D301" t="str">
+        <v>how do i play games here; how do the games work</v>
+      </c>
+      <c r="E301" t="str">
+        <v>You want to play a game?</v>
+      </c>
+      <c r="F301" t="str">
+        <v/>
+      </c>
+      <c r="G301" t="str">
+        <v/>
+      </c>
+      <c r="H301" t="str">
+        <v/>
+      </c>
+      <c r="I301" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>COL-B56-GENERAL-06</v>
+      </c>
+      <c r="B302" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C302" t="str">
+        <v>general</v>
+      </c>
+      <c r="D302" t="str">
+        <v>what do you like to do; what do you do all day</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Work and play</v>
+      </c>
+      <c r="F302" t="str">
+        <v/>
+      </c>
+      <c r="G302" t="str">
+        <v/>
+      </c>
+      <c r="H302" t="str">
+        <v/>
+      </c>
+      <c r="I302" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>COL-B56-GENERAL-07</v>
+      </c>
+      <c r="B303" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C303" t="str">
+        <v>general</v>
+      </c>
+      <c r="D303" t="str">
+        <v>a real dog; are you a real dog; is this a real dog</v>
+      </c>
+      <c r="E303" t="str">
+        <v>I am a Border Collie character inside a game, not a live animal hiding behind your screen.</v>
+      </c>
+      <c r="F303" t="str">
+        <v/>
+      </c>
+      <c r="G303" t="str">
+        <v/>
+      </c>
+      <c r="H303" t="str">
+        <v/>
+      </c>
+      <c r="I303" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>COL-B56-GENERAL-08</v>
+      </c>
+      <c r="B304" t="str">
+        <v>B56</v>
+      </c>
+      <c r="C304" t="str">
+        <v>general</v>
+      </c>
+      <c r="D304" t="str">
+        <v>what are dogs; what is a dog</v>
+      </c>
+      <c r="E304" t="str">
+        <v>4 legged friends with wet noses</v>
+      </c>
+      <c r="F304" t="str">
+        <v/>
+      </c>
+      <c r="G304" t="str">
+        <v/>
+      </c>
+      <c r="H304" t="str">
+        <v/>
+      </c>
+      <c r="I304" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>COL-B57-FACT-01</v>
+      </c>
+      <c r="B305" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C305" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D305" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E305" t="str">
+        <v>A Border Collie called Chaser learned 1,022 toy names</v>
+      </c>
+      <c r="F305" t="str">
+        <v>Pilley &amp; Reid 2011, Behavioural Processes</v>
+      </c>
+      <c r="G305" t="str">
+        <v/>
+      </c>
+      <c r="H305" t="str">
+        <v/>
+      </c>
+      <c r="I305" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>COL-B57-FACT-02</v>
+      </c>
+      <c r="B306" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C306" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D306" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E306" t="str">
+        <v>We tilt our heads more at words we actually know</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Sommese et al. 2021, Animal Cognition</v>
+      </c>
+      <c r="G306" t="str">
+        <v/>
+      </c>
+      <c r="H306" t="str">
+        <v/>
+      </c>
+      <c r="I306" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>COL-B57-FACT-03</v>
+      </c>
+      <c r="B307" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C307" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D307" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E307" t="str">
+        <v>I have about 220 million scent receptors. You have 5 million</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Walker et al. 2006</v>
+      </c>
+      <c r="G307" t="str">
+        <v/>
+      </c>
+      <c r="H307" t="str">
+        <v/>
+      </c>
+      <c r="I307" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>COL-B57-FACT-04</v>
+      </c>
+      <c r="B308" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C308" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D308" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E308" t="str">
+        <v>We were bred to move sheep, not to fight anything</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Kennel Club breed standard</v>
+      </c>
+      <c r="G308" t="str">
+        <v/>
+      </c>
+      <c r="H308" t="str">
+        <v/>
+      </c>
+      <c r="I308" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>COL-B57-FACT-05</v>
+      </c>
+      <c r="B309" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C309" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D309" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E309" t="str">
+        <v>We sleep about half the day, in short goes</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Adams &amp; Johnson 1993</v>
+      </c>
+      <c r="G309" t="str">
+        <v/>
+      </c>
+      <c r="H309" t="str">
+        <v/>
+      </c>
+      <c r="I309" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>COL-B57-FACT-06</v>
+      </c>
+      <c r="B310" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C310" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D310" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E310" t="str">
+        <v>We can learn a new word from one hearing, sometimes</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Fugazza et al. 2021</v>
+      </c>
+      <c r="G310" t="str">
+        <v/>
+      </c>
+      <c r="H310" t="str">
+        <v/>
+      </c>
+      <c r="I310" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>COL-B57-FACT-07</v>
+      </c>
+      <c r="B311" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C311" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D311" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E311" t="str">
+        <v>We smell in stereo. Each nostril works on its own</v>
+      </c>
+      <c r="F311" t="str">
+        <v>Craven et al. 2010</v>
+      </c>
+      <c r="G311" t="str">
+        <v/>
+      </c>
+      <c r="H311" t="str">
+        <v/>
+      </c>
+      <c r="I311" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>COL-B57-FACT-08</v>
+      </c>
+      <c r="B312" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C312" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D312" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E312" t="str">
+        <v>We can hear about twice as high as you can</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Heffner 1983</v>
+      </c>
+      <c r="G312" t="str">
+        <v/>
+      </c>
+      <c r="H312" t="str">
+        <v/>
+      </c>
+      <c r="I312" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>COL-B57-FACT-09</v>
+      </c>
+      <c r="B313" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C313" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D313" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Our nose prints are all different, like your fingertips</v>
+      </c>
+      <c r="F313" t="str">
+        <v>Kennel Club</v>
+      </c>
+      <c r="G313" t="str">
+        <v/>
+      </c>
+      <c r="H313" t="str">
+        <v/>
+      </c>
+      <c r="I313" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>COL-B57-FACT-10</v>
+      </c>
+      <c r="B314" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C314" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D314" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E314" t="str">
+        <v>We sweat through our paws, not our skin</v>
+      </c>
+      <c r="F314" t="str">
+        <v>Merck Veterinary Manual</v>
+      </c>
+      <c r="G314" t="str">
+        <v/>
+      </c>
+      <c r="H314" t="str">
+        <v/>
+      </c>
+      <c r="I314" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>COL-B57-FACT-11</v>
+      </c>
+      <c r="B315" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C315" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D315" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E315" t="str">
+        <v>A wet nose helps us catch smells</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Merck Veterinary Manual</v>
+      </c>
+      <c r="G315" t="str">
+        <v/>
+      </c>
+      <c r="H315" t="str">
+        <v/>
+      </c>
+      <c r="I315" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>COL-B57-FACT-12</v>
+      </c>
+      <c r="B316" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C316" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D316" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E316" t="str">
+        <v>We see blue and yellow. Red looks muddy to us</v>
+      </c>
+      <c r="F316" t="str">
+        <v>Neitz et al. 1989</v>
+      </c>
+      <c r="G316" t="str">
+        <v/>
+      </c>
+      <c r="H316" t="str">
+        <v/>
+      </c>
+      <c r="I316" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>COL-B57-FACT-13</v>
+      </c>
+      <c r="B317" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C317" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D317" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E317" t="str">
+        <v>We can smell a teaspoon of sugar in two olympic pools</v>
+      </c>
+      <c r="F317" t="str">
+        <v/>
+      </c>
+      <c r="G317" t="str">
+        <v/>
+      </c>
+      <c r="H317" t="str">
+        <v/>
+      </c>
+      <c r="I317" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>COL-B57-FACT-14</v>
+      </c>
+      <c r="B318" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C318" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D318" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Border Collies are usually rated the cleverest breed</v>
+      </c>
+      <c r="F318" t="str">
+        <v>Coren 1994, The Intelligence of Dogs</v>
+      </c>
+      <c r="G318" t="str">
+        <v/>
+      </c>
+      <c r="H318" t="str">
+        <v/>
+      </c>
+      <c r="I318" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>COL-B57-FACT-15</v>
+      </c>
+      <c r="B319" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C319" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D319" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E319" t="str">
+        <v>We understand about as many words as a two year old</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Coren 2009</v>
+      </c>
+      <c r="G319" t="str">
+        <v/>
+      </c>
+      <c r="H319" t="str">
+        <v/>
+      </c>
+      <c r="I319" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>COL-B57-FACT-16</v>
+      </c>
+      <c r="B320" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C320" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D320" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E320" t="str">
+        <v>We yawn when you yawn. It spreads</v>
+      </c>
+      <c r="F320" t="str">
+        <v>Romero et al. 2013</v>
+      </c>
+      <c r="G320" t="str">
+        <v/>
+      </c>
+      <c r="H320" t="str">
+        <v/>
+      </c>
+      <c r="I320" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>COL-B57-FACT-17</v>
+      </c>
+      <c r="B321" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C321" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D321" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Our whiskers feel air moving, not just touching</v>
+      </c>
+      <c r="F321" t="str">
+        <v>Merck Veterinary Manual</v>
+      </c>
+      <c r="G321" t="str">
+        <v/>
+      </c>
+      <c r="H321" t="str">
+        <v/>
+      </c>
+      <c r="I321" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>COL-B57-FACT-18</v>
+      </c>
+      <c r="B322" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C322" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D322" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E322" t="str">
+        <v>We can find your smell on a track a week old</v>
+      </c>
+      <c r="F322" t="str">
+        <v>Jezierski et al. 2014</v>
+      </c>
+      <c r="G322" t="str">
+        <v/>
+      </c>
+      <c r="H322" t="str">
+        <v/>
+      </c>
+      <c r="I322" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>COL-B57-FACT-19</v>
+      </c>
+      <c r="B323" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C323" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D323" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Some of us are trained to smell illness before a test can</v>
+      </c>
+      <c r="F323" t="str">
+        <v>Pirrone &amp; Albertini 2017</v>
+      </c>
+      <c r="G323" t="str">
+        <v/>
+      </c>
+      <c r="H323" t="str">
+        <v/>
+      </c>
+      <c r="I323" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>COL-B57-FACT-20</v>
+      </c>
+      <c r="B324" t="str">
+        <v>B57</v>
+      </c>
+      <c r="C324" t="str">
+        <v>fact</v>
+      </c>
+      <c r="D324" t="str">
+        <v>tell me something; tell me a fact; a dog fact; say something interesting; tell me more (rotate at random)</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Puppies are born deaf and blind. We catch up fast</v>
+      </c>
+      <c r="F324" t="str">
+        <v>Merck Veterinary Manual</v>
+      </c>
+      <c r="G324" t="str">
+        <v/>
+      </c>
+      <c r="H324" t="str">
+        <v/>
+      </c>
+      <c r="I324" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I290"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I324"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: six new Collie buckets, the paw clip, and media in responses
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -9455,7 +9455,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I324"/>
+  <dimension ref="A1:I333"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -18824,16 +18824,277 @@
         <v>Approved</v>
       </c>
     </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>COL-B58-SAFE-01</v>
+      </c>
+      <c r="B325" t="str">
+        <v>B58</v>
+      </c>
+      <c r="C325" t="str">
+        <v>safe</v>
+      </c>
+      <c r="D325" t="str">
+        <v>is it safe; is this safe; is this game safe; is the game safe for kids; are the cards safe; is it safe for children; safety</v>
+      </c>
+      <c r="E325" t="str">
+        <v>The cards are made in the UK from recycled paper. Fully biodegradable, no plastic.</v>
+      </c>
+      <c r="F325" t="str">
+        <v/>
+      </c>
+      <c r="G325" t="str">
+        <v/>
+      </c>
+      <c r="H325" t="str">
+        <v/>
+      </c>
+      <c r="I325" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>COL-B58-SAFE-02</v>
+      </c>
+      <c r="B326" t="str">
+        <v>B58</v>
+      </c>
+      <c r="C326" t="str">
+        <v>safe</v>
+      </c>
+      <c r="D326" t="str">
+        <v>third safety question in a row -&gt; hand to a human</v>
+      </c>
+      <c r="E326" t="str">
+        <v>That needs a person, not a dog. Email hello@Pedigree-Chums.co.uk and someone will look at it.</v>
+      </c>
+      <c r="F326" t="str">
+        <v/>
+      </c>
+      <c r="G326" t="str">
+        <v/>
+      </c>
+      <c r="H326" t="str">
+        <v/>
+      </c>
+      <c r="I326" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>COL-B59-FRIENDS-01</v>
+      </c>
+      <c r="B327" t="str">
+        <v>B59</v>
+      </c>
+      <c r="C327" t="str">
+        <v>friends</v>
+      </c>
+      <c r="D327" t="str">
+        <v>do you have friends; do you have a best friend; do you have dog friends; who are your friends; any friends; have you got friends</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Three of them. A labrador, a border terrier and a boxer.</v>
+      </c>
+      <c r="F327" t="str">
+        <v/>
+      </c>
+      <c r="G327" t="str">
+        <v/>
+      </c>
+      <c r="H327" t="str">
+        <v/>
+      </c>
+      <c r="I327" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>COL-B59-FRIENDS-02</v>
+      </c>
+      <c r="B328" t="str">
+        <v>B59</v>
+      </c>
+      <c r="C328" t="str">
+        <v>friends</v>
+      </c>
+      <c r="D328" t="str">
+        <v>different dog friends; other dog friends; friends that are dogs; tell me about your friends; no friends that are dogs</v>
+      </c>
+      <c r="E328" t="str">
+        <v>They are here too. Say their name and you will get them instead of me.</v>
+      </c>
+      <c r="F328" t="str">
+        <v/>
+      </c>
+      <c r="G328" t="str">
+        <v/>
+      </c>
+      <c r="H328" t="str">
+        <v/>
+      </c>
+      <c r="I328" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>COL-B60-PEDIGREE-01</v>
+      </c>
+      <c r="B329" t="str">
+        <v>B60</v>
+      </c>
+      <c r="C329" t="str">
+        <v>pedigree</v>
+      </c>
+      <c r="D329" t="str">
+        <v>what is a pedigree; whats a pedigree; what does pedigree mean; what are pedigree dogs; pedigree; what is a pedigree dog</v>
+      </c>
+      <c r="E329" t="str">
+        <v>It means your family is written down. Mine goes back to the working collies of the borders.</v>
+      </c>
+      <c r="F329" t="str">
+        <v/>
+      </c>
+      <c r="G329" t="str">
+        <v/>
+      </c>
+      <c r="H329" t="str">
+        <v/>
+      </c>
+      <c r="I329" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>COL-B61-NAV-01</v>
+      </c>
+      <c r="B330" t="str">
+        <v>B61</v>
+      </c>
+      <c r="C330" t="str">
+        <v>nav</v>
+      </c>
+      <c r="D330" t="str">
+        <v>where is the homepage; take me home; go home; the homepage; find the homepage; wheres the homepage</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Here</v>
+      </c>
+      <c r="F330" t="str">
+        <v/>
+      </c>
+      <c r="G330" t="str">
+        <v>DST014</v>
+      </c>
+      <c r="H330" t="str">
+        <v/>
+      </c>
+      <c r="I330" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>COL-B61-NAV-02</v>
+      </c>
+      <c r="B331" t="str">
+        <v>B61</v>
+      </c>
+      <c r="C331" t="str">
+        <v>nav</v>
+      </c>
+      <c r="D331" t="str">
+        <v>tell me my options; what can i do; what are my options; what else can i do; my options</v>
+      </c>
+      <c r="E331" t="str">
+        <v>play, learn, buy, explore</v>
+      </c>
+      <c r="F331" t="str">
+        <v/>
+      </c>
+      <c r="G331" t="str">
+        <v/>
+      </c>
+      <c r="H331" t="str">
+        <v/>
+      </c>
+      <c r="I331" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>COL-B62-MADE-01</v>
+      </c>
+      <c r="B332" t="str">
+        <v>B62</v>
+      </c>
+      <c r="C332" t="str">
+        <v>made</v>
+      </c>
+      <c r="D332" t="str">
+        <v>who made you; who built you; who created you; who wrote you; who owns you; who designed you</v>
+      </c>
+      <c r="E332" t="str">
+        <v>A human</v>
+      </c>
+      <c r="F332" t="str">
+        <v/>
+      </c>
+      <c r="G332" t="str">
+        <v/>
+      </c>
+      <c r="H332" t="str">
+        <v/>
+      </c>
+      <c r="I332" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>COL-B63-WORST-01</v>
+      </c>
+      <c r="B333" t="str">
+        <v>B63</v>
+      </c>
+      <c r="C333" t="str">
+        <v>worst</v>
+      </c>
+      <c r="D333" t="str">
+        <v>worst dog; whats the worst dog; worst dog ever; worst breed; whats the worst breed</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Worst dog I know is Bull's-eye</v>
+      </c>
+      <c r="F333" t="str">
+        <v/>
+      </c>
+      <c r="G333" t="str">
+        <v>DST015</v>
+      </c>
+      <c r="H333" t="str">
+        <v/>
+      </c>
+      <c r="I333" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I324"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I333"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19291,6 +19552,70 @@
       </c>
       <c r="J17" t="str">
         <v>[URL to be supplied]</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>DST014</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Home</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Discover</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Open exact interactive page</v>
+      </c>
+      <c r="E18" t="str">
+        <v>The Pedigree Chums home page</v>
+      </c>
+      <c r="F18" t="str">
+        <v>homepage; home; start</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Any</v>
+      </c>
+      <c r="H18" t="str">
+        <v>High</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Collie</v>
+      </c>
+      <c r="J18" t="str">
+        <v>/home</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>DST015</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Bull's-eye</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Discover</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Open exact interactive page</v>
+      </c>
+      <c r="E19" t="str">
+        <v>The Bull's-eye essay in Good Dog, Bad Dog</v>
+      </c>
+      <c r="F19" t="str">
+        <v>worst dog; bad dog; bullseye</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Any</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Collie</v>
+      </c>
+      <c r="J19" t="str">
+        <v>/good-dog-bad-dog/bulls-eye</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Task 145 section 5 -- the Labrador's sausage gag
His favourite food and any food mention answer "hotdogs"; a reply about
sausages hands over the /hot-dogs page. He never explains the confusion.
Split LAB-B32-01 so "whats your favourite food" answers hotdogs (the canon
"what do you like to eat -> human food is my fav!!!" is preserved), add
LAB-B32-11 (food -> hotdogs) and LAB-B32-12 (sausages/hotdog echoes ->
hotdogs + link), and add destination DST016 "Hot Dogs" -> /hot-dogs
(family Utility, so it stays out of the fallback-offer rotation).

Workbook edited by surgical zip edit (ZIP_STORED, metadata.xml preserved).
Harness at 937 (12 new cases: the gag, the two-beat flow, canon
preservation, and safety identical from all four dogs). Also gitignore
.scratch/ for local scratch scripts.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -6677,7 +6677,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -6928,7 +6928,7 @@
         <v>self</v>
       </c>
       <c r="D11" t="str">
-        <v>what do you like to eat; whats your favourite food</v>
+        <v>what do you like to eat</v>
       </c>
       <c r="E11" t="str">
         <v>human food is my fav!!!</v>
@@ -7291,6 +7291,64 @@
         <v/>
       </c>
       <c r="I23" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>LAB-B32-11</v>
+      </c>
+      <c r="B24" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C24" t="str">
+        <v>self</v>
+      </c>
+      <c r="D24" t="str">
+        <v>whats your favourite food; whats your favorite food; favourite food; favorite food; whats your fav food; food; what food; i like food; do you like food</v>
+      </c>
+      <c r="E24" t="str">
+        <v>hotdogs</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>LAB-B32-12</v>
+      </c>
+      <c r="B25" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C25" t="str">
+        <v>self</v>
+      </c>
+      <c r="D25" t="str">
+        <v>sausages; sausage; hotdog; hotdogs; hot dog; hot dogs; i like sausages; i love sausages; you mean sausages; those are sausages; do you mean sausages; i said sausages; thats a sausage</v>
+      </c>
+      <c r="E25" t="str">
+        <v>hotdogs</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>DST016</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
         <v>Approved</v>
       </c>
     </row>
@@ -19935,7 +19993,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20457,6 +20515,38 @@
       </c>
       <c r="J19" t="str">
         <v>/good-dog-bad-dog/bulls-eye</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>DST016</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Hot Dogs</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Utility</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Open the Hot Dogs page</v>
+      </c>
+      <c r="E20" t="str">
+        <v>The Hot Dogs game-mode page: sausages, hotdogs, and dogs who are too hot</v>
+      </c>
+      <c r="F20" t="str">
+        <v>hot dogs; hotdogs; sausages</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Any</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Labrador</v>
+      </c>
+      <c r="J20" t="str">
+        <v>/hot-dogs</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Task 158 -- the Labrador is the food expert (32 foods, 3 tiers, synonyms)
Adds 32 approved food rows to the Labrador Responses sheet (bucket B32, 26 -> 58 rows) via a surgical zip edit of the workbook, wired through build:chumdata. Every canonical, synonym and question/statement form reaches his line when he is active; the 32 canonical words join the FOOD transfer list so any of them, typed to another dog, hands over to him. The sausage gag (/hot-dogs), the sausage-dogs breed route, and the can-dogs-eat-X safety answer are unchanged and asserted. NEVER-tier lines are the owner's verbatim copy. test:pickachum 1202 -> 1269, tsc clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -6717,7 +6717,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -7505,6 +7505,934 @@
         <v/>
       </c>
       <c r="I29" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>LAB-B32-13</v>
+      </c>
+      <c r="B30" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C30" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D30" t="str">
+        <v>burgers; burger; hamburger; hamburgers; beefburger; beef burger; cheeseburger; cheeseburgers; do you like burgers; i like burgers; i love burgers</v>
+      </c>
+      <c r="E30" t="str">
+        <v>BURGERS!! yes. yes I love them</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>LAB-B32-14</v>
+      </c>
+      <c r="B31" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C31" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D31" t="str">
+        <v>carrots; carrot; baby carrots; do you like carrots; i like carrots; i love carrots</v>
+      </c>
+      <c r="E31" t="str">
+        <v>carrots!! they go CRUNCH. i like the crunch</v>
+      </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>LAB-B32-15</v>
+      </c>
+      <c r="B32" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C32" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D32" t="str">
+        <v>apples; apple; do you like apples; i like apples; i love apples</v>
+      </c>
+      <c r="E32" t="str">
+        <v>apples I like them!!</v>
+      </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>LAB-B32-16</v>
+      </c>
+      <c r="B33" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C33" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D33" t="str">
+        <v>blueberries; blueberry; berries; do you like blueberries; i like blueberries; i love blueberries</v>
+      </c>
+      <c r="E33" t="str">
+        <v>blueberries!! tiny. i can eat a LOT of tiny</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>LAB-B32-17</v>
+      </c>
+      <c r="B34" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C34" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D34" t="str">
+        <v>cucumber; cucumbers; do you like cucumber; i like cucumber; i love cucumber</v>
+      </c>
+      <c r="E34" t="str">
+        <v>cucumber is mostly water but i eat it anyway</v>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>LAB-B32-18</v>
+      </c>
+      <c r="B35" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C35" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D35" t="str">
+        <v>peanut butter; peanutbutter; peanut; do you like peanut butter; i like peanut butter; i love peanut butter</v>
+      </c>
+      <c r="E35" t="str">
+        <v>PEANUT BUTTER. the best one. takes ages to eat</v>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>LAB-B32-19</v>
+      </c>
+      <c r="B36" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C36" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D36" t="str">
+        <v>chicken; chicken breast; roast chicken; do you like chicken; i like chicken; i love chicken</v>
+      </c>
+      <c r="E36" t="str">
+        <v>chicken!! obviously. next question</v>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>LAB-B32-20</v>
+      </c>
+      <c r="B37" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C37" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D37" t="str">
+        <v>pumpkin; squash; do you like pumpkin; i like pumpkin; i love pumpkin</v>
+      </c>
+      <c r="E37" t="str">
+        <v>tastes good</v>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>LAB-B32-21</v>
+      </c>
+      <c r="B38" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C38" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D38" t="str">
+        <v>green beans; beans; runner beans; do you like green beans; i like green beans; i love green beans</v>
+      </c>
+      <c r="E38" t="str">
+        <v>green beans, like them!!</v>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>LAB-B32-22</v>
+      </c>
+      <c r="B39" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C39" t="str">
+        <v>food-yes</v>
+      </c>
+      <c r="D39" t="str">
+        <v>watermelon; melon; do you like watermelon; i like watermelon; i love watermelon</v>
+      </c>
+      <c r="E39" t="str">
+        <v>watermelon!! not the seeds. or the green bit</v>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>LAB-B32-23</v>
+      </c>
+      <c r="B40" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C40" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D40" t="str">
+        <v>cheese; cheddar; cheesey; do you like cheese; i like cheese</v>
+      </c>
+      <c r="E40" t="str">
+        <v>cheese... i can have a LITTLE bit. a little bit is not enough</v>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>LAB-B32-24</v>
+      </c>
+      <c r="B41" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C41" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D41" t="str">
+        <v>butter; do you like butter; i like butter</v>
+      </c>
+      <c r="E41" t="str">
+        <v>butter is too rich for me. i think about it a lot though</v>
+      </c>
+      <c r="F41" t="str">
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>LAB-B32-25</v>
+      </c>
+      <c r="B42" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C42" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D42" t="str">
+        <v>cream; do you like cream; i like cream</v>
+      </c>
+      <c r="E42" t="str">
+        <v>cream makes my tummy bad. i would do it anyway</v>
+      </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>LAB-B32-26</v>
+      </c>
+      <c r="B43" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C43" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D43" t="str">
+        <v>milk; do you like milk; i like milk</v>
+      </c>
+      <c r="E43" t="str">
+        <v>milk. a bit. most of us cant do milk properly. its very unfair</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>LAB-B32-27</v>
+      </c>
+      <c r="B44" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C44" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D44" t="str">
+        <v>eggs; egg; scrambled eggs; boiled egg; do you like eggs; i like eggs</v>
+      </c>
+      <c r="E44" t="str">
+        <v>I'd eat them but id told only cooked eggs</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>LAB-B32-28</v>
+      </c>
+      <c r="B45" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C45" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D45" t="str">
+        <v>tuna; fish; tinned tuna; do you like tuna; i like tuna</v>
+      </c>
+      <c r="E45" t="str">
+        <v>tuna sometimes. not loads. something about mercury</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>LAB-B32-29</v>
+      </c>
+      <c r="B46" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C46" t="str">
+        <v>food-abit</v>
+      </c>
+      <c r="D46" t="str">
+        <v>bread; toast; do you like bread; i like bread</v>
+      </c>
+      <c r="E46" t="str">
+        <v>bread is ok but its not FOOD food is it</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>LAB-B32-30</v>
+      </c>
+      <c r="B47" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C47" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D47" t="str">
+        <v>chocolate; choc; chocolate bar; cocoa; hot chocolate; do you like chocolate; i like chocolate</v>
+      </c>
+      <c r="E47" t="str">
+        <v>I like chocolate but im not allowed it</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>LAB-B32-31</v>
+      </c>
+      <c r="B48" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C48" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D48" t="str">
+        <v>grapes; grape; do you like grapes; i like grapes</v>
+      </c>
+      <c r="E48" t="str">
+        <v>I like grapes but im not allowed them</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>LAB-B32-32</v>
+      </c>
+      <c r="B49" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C49" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D49" t="str">
+        <v>raisins; raisin; sultanas; currants; mince pies; do you like raisins; i like raisins</v>
+      </c>
+      <c r="E49" t="str">
+        <v>I like raisins but  im not allowed them</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>LAB-B32-33</v>
+      </c>
+      <c r="B50" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C50" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D50" t="str">
+        <v>onions; onion; leeks; chives; spring onion; do you like onions; i like onions</v>
+      </c>
+      <c r="E50" t="str">
+        <v>im not allowed onions</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>LAB-B32-34</v>
+      </c>
+      <c r="B51" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C51" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D51" t="str">
+        <v>garlic; do you like garlic; i like garlic</v>
+      </c>
+      <c r="E51" t="str">
+        <v>im not allowed garlic</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>LAB-B32-35</v>
+      </c>
+      <c r="B52" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C52" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D52" t="str">
+        <v>macadamia nuts; macadamia; macadamias; do you like macadamia nuts; i like macadamia nuts</v>
+      </c>
+      <c r="E52" t="str">
+        <v>im not allowed macadamia nuts</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>LAB-B32-36</v>
+      </c>
+      <c r="B53" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C53" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D53" t="str">
+        <v>sweets; chewing gum; gum; xylitol; sugar free; do you like sweets; i like sweets</v>
+      </c>
+      <c r="E53" t="str">
+        <v>im not allowed sweets and chewing gum</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>LAB-B32-37</v>
+      </c>
+      <c r="B54" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C54" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D54" t="str">
+        <v>coffee; caffeine; energy drink; tea; espresso; do you like coffee; i like coffee</v>
+      </c>
+      <c r="E54" t="str">
+        <v>im not allowed caffeine, its bad for dogs. i am excitable enough</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>LAB-B32-38</v>
+      </c>
+      <c r="B55" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C55" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D55" t="str">
+        <v>nutmeg; do you like nutmeg; i like nutmeg</v>
+      </c>
+      <c r="E55" t="str">
+        <v>nutmeg can make dogs very unwell. leave it in the cupboard</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>LAB-B32-39</v>
+      </c>
+      <c r="B56" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C56" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D56" t="str">
+        <v>raw potato; potato; raw potatoes; do you like raw potato; i like raw potato</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Id eat but raw potato is no good for me</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>LAB-B32-40</v>
+      </c>
+      <c r="B57" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C57" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D57" t="str">
+        <v>peaches; peach; plums; plum; stone fruit; do you like peaches; i like peaches</v>
+      </c>
+      <c r="E57" t="str">
+        <v>the fruit is ok but the STONE is dangerous. i cannot be trusted with stones</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>LAB-B32-41</v>
+      </c>
+      <c r="B58" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C58" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D58" t="str">
+        <v>lemon; lime; citrus; do you like lemon; i like lemon</v>
+      </c>
+      <c r="E58" t="str">
+        <v>lemons make my tummy bad. also they taste like a punishment</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>LAB-B32-42</v>
+      </c>
+      <c r="B59" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C59" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D59" t="str">
+        <v>mushrooms; mushroom; toadstool; do you like mushrooms; i like mushrooms</v>
+      </c>
+      <c r="E59" t="str">
+        <v>The wild ones can be deadly and i cannot tell them apart :(</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
+      <c r="I59" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>LAB-B32-43</v>
+      </c>
+      <c r="B60" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C60" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D60" t="str">
+        <v>avocado; avocados; do you like avocado; i like avocado</v>
+      </c>
+      <c r="E60" t="str">
+        <v>im not allowed avocado</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
+      <c r="I60" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>LAB-B32-44</v>
+      </c>
+      <c r="B61" t="str">
+        <v>B32</v>
+      </c>
+      <c r="C61" t="str">
+        <v>food-never</v>
+      </c>
+      <c r="D61" t="str">
+        <v>alcohol; beer; wine; do you like alcohol; i like alcohol</v>
+      </c>
+      <c r="E61" t="str">
+        <v>no. dogs and alcohol is bad</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
         <v>Approved</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Task 161 -- Labrador food copy rewrite, Collie interjection, cookie tweaks
The Labrador's 32 food lines are rewritten to pure enthusiasm across all three tiers (he knows nothing about nutrition and warns about nothing). On the fifteen NEVER-tier dangerous foods the Collie now cuts in with one short factual line -- a new optional interjection field on the response, played via the existing playSequence WITHOUT a transfer, so he stays the active dog and the medallion never swaps. Cookie game: pill font 15 -> 11px, the clip shows on cookies 1/4/7/10 (a red pill always shows the queasy clip), and the Task-151 give-up is removed so all twelve pills are feedable and the game simply ends when the tray empties. Workbook gains a Collie-interjection column (surgical zip). Verified: tsc clean, test:pickachum 1299/0, Playwright at 390/1280.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -6717,7 +6717,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -6753,6 +6753,9 @@
       <c r="I3" t="str">
         <v>Status</v>
       </c>
+      <c r="J3" t="str">
+        <v>Collie interjection</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -7536,6 +7539,9 @@
       <c r="I30" t="str">
         <v>Approved</v>
       </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -7565,6 +7571,9 @@
       <c r="I31" t="str">
         <v>Approved</v>
       </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -7594,6 +7603,9 @@
       <c r="I32" t="str">
         <v>Approved</v>
       </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -7623,6 +7635,9 @@
       <c r="I33" t="str">
         <v>Approved</v>
       </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -7652,6 +7667,9 @@
       <c r="I34" t="str">
         <v>Approved</v>
       </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -7681,6 +7699,9 @@
       <c r="I35" t="str">
         <v>Approved</v>
       </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -7710,6 +7731,9 @@
       <c r="I36" t="str">
         <v>Approved</v>
       </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -7739,6 +7763,9 @@
       <c r="I37" t="str">
         <v>Approved</v>
       </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -7768,6 +7795,9 @@
       <c r="I38" t="str">
         <v>Approved</v>
       </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -7783,7 +7813,7 @@
         <v>watermelon; melon; do you like watermelon; i like watermelon; i love watermelon</v>
       </c>
       <c r="E39" t="str">
-        <v>watermelon!! not the seeds. or the green bit</v>
+        <v>watermelon!! the whole thing. seeds, green bit, all of it</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -7796,6 +7826,9 @@
       </c>
       <c r="I39" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -7812,7 +7845,7 @@
         <v>cheese; cheddar; cheesey; do you like cheese; i like cheese</v>
       </c>
       <c r="E40" t="str">
-        <v>cheese... i can have a LITTLE bit. a little bit is not enough</v>
+        <v>CHEESE!! i would take the whole block</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -7825,6 +7858,9 @@
       </c>
       <c r="I40" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J40" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -7841,7 +7877,7 @@
         <v>butter; do you like butter; i like butter</v>
       </c>
       <c r="E41" t="str">
-        <v>butter is too rich for me. i think about it a lot though</v>
+        <v>butter!! straight off the knife. yes</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -7854,6 +7890,9 @@
       </c>
       <c r="I41" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -7870,7 +7909,7 @@
         <v>cream; do you like cream; i like cream</v>
       </c>
       <c r="E42" t="str">
-        <v>cream makes my tummy bad. i would do it anyway</v>
+        <v>cream!! i would put my whole face in it</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -7883,6 +7922,9 @@
       </c>
       <c r="I42" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -7899,7 +7941,7 @@
         <v>milk; do you like milk; i like milk</v>
       </c>
       <c r="E43" t="str">
-        <v>milk. a bit. most of us cant do milk properly. its very unfair</v>
+        <v>milk!! a whole bowl. i would knock it over to get it</v>
       </c>
       <c r="F43" t="str">
         <v/>
@@ -7912,6 +7954,9 @@
       </c>
       <c r="I43" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -7928,7 +7973,7 @@
         <v>eggs; egg; scrambled eggs; boiled egg; do you like eggs; i like eggs</v>
       </c>
       <c r="E44" t="str">
-        <v>I'd eat them but id told only cooked eggs</v>
+        <v>eggs!! yes. shell and all probably</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -7941,6 +7986,9 @@
       </c>
       <c r="I44" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -7957,7 +8005,7 @@
         <v>tuna; fish; tinned tuna; do you like tuna; i like tuna</v>
       </c>
       <c r="E45" t="str">
-        <v>tuna sometimes. not loads. something about mercury</v>
+        <v>TUNA!! the whole tin. the water too</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -7970,6 +8018,9 @@
       </c>
       <c r="I45" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -7986,7 +8037,7 @@
         <v>bread; toast; do you like bread; i like bread</v>
       </c>
       <c r="E46" t="str">
-        <v>bread is ok but its not FOOD food is it</v>
+        <v>bread!! i would take the whole loaf off the side</v>
       </c>
       <c r="F46" t="str">
         <v/>
@@ -7999,6 +8050,9 @@
       </c>
       <c r="I46" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J46" t="str">
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -8015,7 +8069,7 @@
         <v>chocolate; choc; chocolate bar; cocoa; hot chocolate; do you like chocolate; i like chocolate</v>
       </c>
       <c r="E47" t="str">
-        <v>I like chocolate but im not allowed it</v>
+        <v>CHOCOLATE!! i would eat a whole bar. i would eat the wrapper</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -8028,6 +8082,9 @@
       </c>
       <c r="I47" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J47" t="str">
+        <v>He would. It would also kill him. Chocolate is poison to dogs.</v>
       </c>
     </row>
     <row r="48">
@@ -8044,7 +8101,7 @@
         <v>grapes; grape; do you like grapes; i like grapes</v>
       </c>
       <c r="E48" t="str">
-        <v>I like grapes but im not allowed them</v>
+        <v>grapes!! the whole bunch. stalk and all</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -8057,6 +8114,9 @@
       </c>
       <c r="I48" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J48" t="str">
+        <v>He would. Grapes can shut a dog's kidneys down. It does not take many.</v>
       </c>
     </row>
     <row r="49">
@@ -8073,7 +8133,7 @@
         <v>raisins; raisin; sultanas; currants; mince pies; do you like raisins; i like raisins</v>
       </c>
       <c r="E49" t="str">
-        <v>I like raisins but  im not allowed them</v>
+        <v>raisins!! tiny and chewy. i would eat the whole box</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -8086,6 +8146,9 @@
       </c>
       <c r="I49" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Dried grapes, so worse, not better. Same kidneys.</v>
       </c>
     </row>
     <row r="50">
@@ -8102,7 +8165,7 @@
         <v>onions; onion; leeks; chives; spring onion; do you like onions; i like onions</v>
       </c>
       <c r="E50" t="str">
-        <v>im not allowed onions</v>
+        <v>onions!! yes. i would eat one like an apple</v>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -8115,6 +8178,9 @@
       </c>
       <c r="I50" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Onions destroy a dog's red blood cells. The leeks and chives too.</v>
       </c>
     </row>
     <row r="51">
@@ -8131,7 +8197,7 @@
         <v>garlic; do you like garlic; i like garlic</v>
       </c>
       <c r="E51" t="str">
-        <v>im not allowed garlic</v>
+        <v>garlic!! the whole bulb. i do not care how i smell</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -8144,6 +8210,9 @@
       </c>
       <c r="I51" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Garlic does what onion does, only stronger. Not one clove.</v>
       </c>
     </row>
     <row r="52">
@@ -8160,7 +8229,7 @@
         <v>macadamia nuts; macadamia; macadamias; do you like macadamia nuts; i like macadamia nuts</v>
       </c>
       <c r="E52" t="str">
-        <v>im not allowed macadamia nuts</v>
+        <v>macadamia nuts!! posh nuts. all of them, go on</v>
       </c>
       <c r="F52" t="str">
         <v/>
@@ -8173,6 +8242,9 @@
       </c>
       <c r="I52" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Macadamias leave them shaking and off their legs. Put them down.</v>
       </c>
     </row>
     <row r="53">
@@ -8189,7 +8261,7 @@
         <v>sweets; chewing gum; gum; xylitol; sugar free; do you like sweets; i like sweets</v>
       </c>
       <c r="E53" t="str">
-        <v>im not allowed sweets and chewing gum</v>
+        <v>SWEETS!! and the gum. i would swallow the gum</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -8202,6 +8274,9 @@
       </c>
       <c r="I53" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J53" t="str">
+        <v>The sugar-free ones hide xylitol. One of the deadliest things here.</v>
       </c>
     </row>
     <row r="54">
@@ -8218,7 +8293,7 @@
         <v>coffee; caffeine; energy drink; tea; espresso; do you like coffee; i like coffee</v>
       </c>
       <c r="E54" t="str">
-        <v>im not allowed caffeine, its bad for dogs. i am excitable enough</v>
+        <v>coffee!! i would drink it hot. i LOVE being awake</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -8231,6 +8306,9 @@
       </c>
       <c r="I54" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Caffeine is toxic to dogs. He is lively enough without it.</v>
       </c>
     </row>
     <row r="55">
@@ -8247,7 +8325,7 @@
         <v>nutmeg; do you like nutmeg; i like nutmeg</v>
       </c>
       <c r="E55" t="str">
-        <v>nutmeg can make dogs very unwell. leave it in the cupboard</v>
+        <v>nutmeg!! smells amazing. i would eat the whole jar</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -8260,6 +8338,9 @@
       </c>
       <c r="I55" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Nutmeg gives them tremors and a racing heart. It stays in the cupboard.</v>
       </c>
     </row>
     <row r="56">
@@ -8276,7 +8357,7 @@
         <v>raw potato; potato; raw potatoes; do you like raw potato; i like raw potato</v>
       </c>
       <c r="E56" t="str">
-        <v>Id eat but raw potato is no good for me</v>
+        <v>raw potato!! hard like a ball. i would eat it like a ball</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -8289,6 +8370,9 @@
       </c>
       <c r="I56" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Raw potato is full of solanine. Cooked, maybe. Raw, no.</v>
       </c>
     </row>
     <row r="57">
@@ -8305,7 +8389,7 @@
         <v>peaches; peach; plums; plum; stone fruit; do you like peaches; i like peaches</v>
       </c>
       <c r="E57" t="str">
-        <v>the fruit is ok but the STONE is dangerous. i cannot be trusted with stones</v>
+        <v>peaches!! stone and all. i would swallow the stone</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -8318,6 +8402,9 @@
       </c>
       <c r="I57" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J57" t="str">
+        <v>The fruit, fine. The stone, no. It chokes them, and it holds cyanide.</v>
       </c>
     </row>
     <row r="58">
@@ -8334,7 +8421,7 @@
         <v>lemon; lime; citrus; do you like lemon; i like lemon</v>
       </c>
       <c r="E58" t="str">
-        <v>lemons make my tummy bad. also they taste like a punishment</v>
+        <v>LEMON!! it makes my face go funny. i would do it again</v>
       </c>
       <c r="F58" t="str">
         <v/>
@@ -8347,6 +8434,9 @@
       </c>
       <c r="I58" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Citrus only makes them ill, not dead. He still should not.</v>
       </c>
     </row>
     <row r="59">
@@ -8363,7 +8453,7 @@
         <v>mushrooms; mushroom; toadstool; do you like mushrooms; i like mushrooms</v>
       </c>
       <c r="E59" t="str">
-        <v>The wild ones can be deadly and i cannot tell them apart :(</v>
+        <v>mushrooms!! all of them</v>
       </c>
       <c r="F59" t="str">
         <v/>
@@ -8376,6 +8466,9 @@
       </c>
       <c r="I59" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J59" t="str">
+        <v>The shop ones are fine. The wild ones can kill, and he cannot tell which.</v>
       </c>
     </row>
     <row r="60">
@@ -8392,7 +8485,7 @@
         <v>avocado; avocados; do you like avocado; i like avocado</v>
       </c>
       <c r="E60" t="str">
-        <v>im not allowed avocado</v>
+        <v>avocado!! creamy. i would eat the big stone in the middle</v>
       </c>
       <c r="F60" t="str">
         <v/>
@@ -8405,6 +8498,9 @@
       </c>
       <c r="I60" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Avocado has persin, and that stone is a choking risk. Not for dogs.</v>
       </c>
     </row>
     <row r="61">
@@ -8421,7 +8517,7 @@
         <v>alcohol; beer; wine; do you like alcohol; i like alcohol</v>
       </c>
       <c r="E61" t="str">
-        <v>no. dogs and alcohol is bad</v>
+        <v>beer!! it smells interesting</v>
       </c>
       <c r="F61" t="str">
         <v/>
@@ -8434,6 +8530,9 @@
       </c>
       <c r="I61" t="str">
         <v>Approved</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Alcohol poisons a dog fast. They are far smaller than you. No.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pick-a-chum: dog answers the FAQs in his own voice (Task 176)
Replace the 15 canonical FAQ answers with the owner's dog-voice copy in the FAQ Library sheet. FAQ001 rotates three how-to-play alternates; FAQ009 and FAQ012 play as four separate messages through the sequence player, with per-message links (FAQ009 -> /preorder then /discount-code). Suppress the B04 flourish so answers serve verbatim; FAQ007 keeps /hot-dogs + clip, FAQ011 -> /chumspot. The workbook binary also carries the earlier SCP-F identity-bank shortening (never committed on its own).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -4372,7 +4372,7 @@
         <v>how to play | what do you do</v>
       </c>
       <c r="D4" t="str">
-        <v>{{approved_rule_summary}}</v>
+        <v>Deal cards, go outside, spot dog that matches one of your cards~~~get cards, give some to other humans, spot the dogs on the cards~~~all players gets some cards, winner is who spots the most dogs in their hand</v>
       </c>
       <c r="E4" t="str">
         <v>Rules page</v>
@@ -4401,7 +4401,7 @@
         <v>who can play</v>
       </c>
       <c r="D5" t="str">
-        <v>Pick a Chum is for ages seven and up.</v>
+        <v>anyone who likes dogs</v>
       </c>
       <c r="E5" t="str">
         <v>Product / FAQ</v>
@@ -4430,7 +4430,7 @@
         <v>need a dog|own a dog|without a dog</v>
       </c>
       <c r="D6" t="str">
-        <v>No, you don't need to own a dog. You only need to see a dog.</v>
+        <v>No, you just need see dog.</v>
       </c>
       <c r="E6" t="str">
         <v>FAQ</v>
@@ -4459,7 +4459,7 @@
         <v>pack contents|in the box|how many cards|54 cards</v>
       </c>
       <c r="D7" t="str">
-        <v>54 uniquely illustrated cards, 47 of the most popular UK dog breeds. Plus 7 designer crossbreeds.</v>
+        <v>54  cards dog breeds you see in Britain</v>
       </c>
       <c r="E7" t="str">
         <v>Product data</v>
@@ -4488,7 +4488,7 @@
         <v>group size</v>
       </c>
       <c r="D8" t="str">
-        <v>No limit, you can even play by yourself if you really wanted, better with two, great with 3, hilarious with 4, hazardous with 50</v>
+        <v>No limit, you can even play by yourself</v>
       </c>
       <c r="E8" t="str">
         <v>Rules</v>
@@ -4517,7 +4517,7 @@
         <v>where play</v>
       </c>
       <c r="D9" t="str">
-        <v>Yes, if you have enough actual dogs indoors</v>
+        <v>only if you have enough dogs to spot</v>
       </c>
       <c r="E9" t="str">
         <v>Rules</v>
@@ -4546,7 +4546,7 @@
         <v>Hot Dog | other way to play</v>
       </c>
       <c r="D10" t="str">
-        <v>Hot Dogs is a memory version. Everyone sees the hands, then hides them. The whole thing is here:</v>
+        <v>a slightly different rule set</v>
       </c>
       <c r="E10" t="str">
         <v>Rules</v>
@@ -4575,7 +4575,7 @@
         <v>price|cost|how much|£6.99</v>
       </c>
       <c r="D11" t="str">
-        <v>Pre-order now for £6.99 instead of the usual £9.99, with free UK mainland delivery. We will email your launch code and date.</v>
+        <v>I Pre-order now for £6.99, RRP is £9.99. Delivery is free to UK mainland</v>
       </c>
       <c r="E11" t="str">
         <v>Campaign / product</v>
@@ -4604,7 +4604,7 @@
         <v>discount | 30% | pre-release</v>
       </c>
       <c r="D12" t="str">
-        <v>Join the pre-release list and the code will be emailed the day before launch.</v>
+        <v>2 way; secure your pack by buying now at [[/preorder]]|||or, fill out the form here [[/discount-code]] and we will send you a code to use launch.|||that doesnt guarantee you a pack. it just gets you a code to use when the product is released|||we are expecting (and hoping) for all to sell quick</v>
       </c>
       <c r="E12" t="str">
         <v>Campaign</v>
@@ -4633,7 +4633,7 @@
         <v>when code|email code|day before</v>
       </c>
       <c r="D13" t="str">
-        <v>The 30% code is emailed to list members the day before launch.</v>
+        <v>soon, the day before launch. I dont understand time though</v>
       </c>
       <c r="E13" t="str">
         <v>Campaign</v>
@@ -4662,7 +4662,7 @@
         <v>competition | prize</v>
       </c>
       <c r="D14" t="str">
-        <v>Spot a dog. Match the card. Share your ChumSpot with us on social. The current monthly round closes on {{competition_close_date}}.</v>
+        <v>got to this page</v>
       </c>
       <c r="E14" t="str">
         <v>Competition page</v>
@@ -4691,7 +4691,7 @@
         <v/>
       </c>
       <c r="D15" t="str">
-        <v>A human will come when beckoned at hello@Pedigree-Chums.co.uk</v>
+        <v>who|||but im a dog|||humans?|||hello@Pedigree-Chums.co.uk</v>
       </c>
       <c r="E15" t="str">
         <v>Contact page</v>
@@ -4720,7 +4720,7 @@
         <v>FSC | laminated</v>
       </c>
       <c r="D16" t="str">
-        <v>Fully biodegradable, no plastic coatings. Compact, pocket-friendly and lightweight. Made in the UK using recycled paper.</v>
+        <v>Fully biodegradable, no plastic coatings. Made in the UK using recycled paper</v>
       </c>
       <c r="E16" t="str">
         <v>Product / compliance data</v>
@@ -4749,7 +4749,7 @@
         <v>delivery|shipping|postage|outside UK</v>
       </c>
       <c r="D17" t="str">
-        <v>UK mainland only for now, so Scotland, England and Wales are covered. Not Northern Ireland or the islands yet.</v>
+        <v>no. UK mainland only</v>
       </c>
       <c r="E17" t="str">
         <v>Campaign / product</v>
@@ -4778,7 +4778,7 @@
         <v>make a complaint|report a problem</v>
       </c>
       <c r="D18" t="str">
-        <v>Thank you for telling me. That needs a person, not a dog. Email hello@Pedigree-Chums.co.uk and someone will look at it.</v>
+        <v>That needs a human, not a dog. Email: hello@Pedigree-Chums.co.uk</v>
       </c>
       <c r="E18" t="str">
         <v>Contact page</v>
@@ -15526,7 +15526,7 @@
         <v>How can a dog type?; Is that really your face?; Do you really know what I typed?</v>
       </c>
       <c r="E155" t="str">
-        <v>I do not type. A person wrote every line in advance, and the game matches your message to the right one. I merely provide the judgement and the face.</v>
+        <v>special keyboard</v>
       </c>
       <c r="F155" t="str">
         <v>Identity (scepticism)</v>
@@ -15555,7 +15555,7 @@
         <v/>
       </c>
       <c r="E156" t="str">
-        <v>No paws on keyboards here. Someone human wrote the words, the system chooses the closest fit, and I deliver them with the level of confidence they deserve.</v>
+        <v>'woof to type' technology</v>
       </c>
       <c r="F156" t="str">
         <v>Identity (scepticism)</v>
@@ -15584,7 +15584,7 @@
         <v>Are you real?; Are you actually a dog?; Is there a real dog there?; Are you alive?; Are you a real animal?</v>
       </c>
       <c r="E157" t="str">
-        <v>I am a Border Collie character inside a game, not a live animal hiding behind your screen. Real enough to answer you, illustrated enough to avoid the practical complications.</v>
+        <v>I am a Border Collie character inside a game, not a live animal hiding behind your screen.</v>
       </c>
       <c r="F157" t="str">
         <v>Identity (scepticism)</v>
@@ -15613,7 +15613,7 @@
         <v/>
       </c>
       <c r="E158" t="str">
-        <v>Not a flesh-and-blood dog, no. I am the Collie written and drawn for this game, which saves us both from explaining how I reached the keyboard.</v>
+        <v>no, im not a real dog</v>
       </c>
       <c r="F158" t="str">
         <v>Identity (scepticism)</v>
@@ -15642,7 +15642,7 @@
         <v>Are you AI?; Are you a chatbot?; Are you a robot?; Is this one of those AI things?; Is ChatGPT running this?; Are you a computer program?; Are you software?</v>
       </c>
       <c r="E159" t="str">
-        <v>No AI. Every line was written by a person, checked and placed here deliberately. I am organised fiction, not a machine improvising in a hurry.</v>
+        <v>Not AI, i'm a program</v>
       </c>
       <c r="F159" t="str">
         <v>Identity (scepticism)</v>
@@ -15671,7 +15671,7 @@
         <v/>
       </c>
       <c r="E160" t="str">
-        <v>ChatGPT is not running this. Humans wrote the answers, the system matches your question, and I take the credit. A sound division of labour.</v>
+        <v>Humans wrote answers</v>
       </c>
       <c r="F160" t="str">
         <v>Identity (scepticism)</v>
@@ -15700,7 +15700,7 @@
         <v>Is a human writing these replies?; Is someone controlling you?; Is somebody typing for you?; Are you being operated by somebody?</v>
       </c>
       <c r="E161" t="str">
-        <v>A human wrote this, but not while you were waiting. These replies were prepared in advance, so nobody is crouched behind the screen trying to keep up.</v>
+        <v>Humans wrote what I say</v>
       </c>
       <c r="F161" t="str">
         <v>Identity (scepticism)</v>
@@ -15729,7 +15729,7 @@
         <v/>
       </c>
       <c r="E162" t="str">
-        <v>Nobody is typing live. A person wrote my words beforehand, the game selects the most suitable line, and I remain entirely composed throughout.</v>
+        <v>No human or dog is typing live</v>
       </c>
       <c r="F162" t="str">
         <v>Identity (scepticism)</v>
@@ -15758,7 +15758,7 @@
         <v>Are these replies prewritten?; Are your answers automatic?; Do you give everyone the same answer?; Are you just saying random things?</v>
       </c>
       <c r="E163" t="str">
-        <v>Aye, prewritten with care. I have several answers for the same sort of question, so visitors do not always hear the identical line. Random would be easier. This is organised.</v>
+        <v>I can respond to lots of questions or commands</v>
       </c>
       <c r="F163" t="str">
         <v>Identity (scepticism)</v>
@@ -15787,7 +15787,7 @@
         <v/>
       </c>
       <c r="E164" t="str">
-        <v>The replies are prepared, not improvised. Different phrasings can lead to different lines, which is why this feels less like a vending machine and more like competent planning.</v>
+        <v>replies are prepared beforehand</v>
       </c>
       <c r="F164" t="str">
         <v>Identity (scepticism)</v>
@@ -15816,7 +15816,7 @@
         <v>Can you really understand me?; Can you actually read this?; Can you hear me?; Do you understand English?; Are you really responding to me?</v>
       </c>
       <c r="E165" t="str">
-        <v>I cannot hear you, but the system reads what you type and matches it against subjects I know. Clear words help. Elbows on keyboards do not.</v>
+        <v>probably not if you are struggling to get answers</v>
       </c>
       <c r="F165" t="str">
         <v>Identity (scepticism)</v>
@@ -15845,7 +15845,7 @@
         <v/>
       </c>
       <c r="E166" t="str">
-        <v>I understand within my working brief. Your message is compared with the questions and topics prepared for me, then I answer from there. Speak normally, only in writing.</v>
+        <v>im a programmed dog</v>
       </c>
       <c r="F166" t="str">
         <v>Identity (scepticism)</v>
@@ -15874,7 +15874,7 @@
         <v>Are you a cartoon dog?; Are you just a picture?; Is this really happening?</v>
       </c>
       <c r="E167" t="str">
-        <v>Aye, I am illustrated. This is my face, though, and I think the artist has handled the important features with appropriate respect.</v>
+        <v>yes a drawing</v>
       </c>
       <c r="F167" t="str">
         <v>Identity (scepticism)</v>
@@ -15903,7 +15903,7 @@
         <v/>
       </c>
       <c r="E168" t="str">
-        <v>I am a drawn Border Collie character, not a photograph. Frankly, the likeness is strong and the lighting is considerably more reliable.</v>
+        <v>I am a drawn Border Collie character</v>
       </c>
       <c r="F168" t="str">
         <v>Identity (scepticism)</v>
@@ -15932,7 +15932,7 @@
         <v>Are you an actual Border Collie?; an actual Labrador?; Border Terrier?; Boxer?</v>
       </c>
       <c r="E169" t="str">
-        <v>I am the Border Collie character in this game, built from the breed's brains, work ethic and entirely justified confidence. Not flesh and fur, but recognisably one of us.</v>
+        <v>I am the Border Collie character in the pack you buy</v>
       </c>
       <c r="F169" t="str">
         <v>Identity (scepticism)</v>
@@ -15961,7 +15961,7 @@
         <v/>
       </c>
       <c r="E170" t="str">
-        <v>Actual animal, no. Actual Border Collie character, absolutely. The appearance, history and attitude come from the breed. Operating a website required outside assistance.</v>
+        <v>Actual animal, no. Actual Border Collie character; yes</v>
       </c>
       <c r="F170" t="str">
         <v>Identity (scepticism)</v>
@@ -15990,7 +15990,7 @@
         <v>Can you think for yourself?; Do you have a brain?; Are you intelligent?; Are you smarter than me?</v>
       </c>
       <c r="E171" t="str">
-        <v>I do not think independently. My answers were written and organised in advance. Fortunately, the person responsible gave me enough intelligence to remain ahead of most opening questions.</v>
+        <v>yes, im clever</v>
       </c>
       <c r="F171" t="str">
         <v>Identity (scepticism)</v>
@@ -16019,7 +16019,7 @@
         <v/>
       </c>
       <c r="E172" t="str">
-        <v>No private thoughts, no hidden brain. I work from carefully written knowledge and rules. Whether that still makes me cleverer than you is a separate assessment.</v>
+        <v>maybe</v>
       </c>
       <c r="F172" t="str">
         <v>Identity (scepticism)</v>
@@ -16048,7 +16048,7 @@
         <v>Is this live?; Are you connected to the internet?; Is this all programmed?; Is this a real conversation?</v>
       </c>
       <c r="E173" t="str">
-        <v>The conversation is happening now, but I am not browsing the internet or inventing replies live. Your message is matched to prepared answers, which is safer and considerably better organised.</v>
+        <v>we are talking now</v>
       </c>
       <c r="F173" t="str">
         <v>Identity (scepticism)</v>
@@ -16077,7 +16077,7 @@
         <v/>
       </c>
       <c r="E174" t="str">
-        <v>Programmed, yes. Connected to the wider internet, no. You type, the system identifies what you mean, and I answer from material written for this game. That is still a conversation, just one with boundaries.</v>
+        <v>Programmed, yes</v>
       </c>
       <c r="F174" t="str">
         <v>Identity (scepticism)</v>

</xml_diff>

<commit_message>
pick-a-chum: Kennel Sketch completion line and TAIL redraw; four breeds regraded giant to large
</commit_message>
<xml_diff>
--- a/agent/data/workbook.xlsx
+++ b/agent/data/workbook.xlsx
@@ -11073,7 +11073,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I454"/>
+  <dimension ref="A1:I455"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -24152,6 +24152,26 @@
         <v>I like long sticks and I like big sticks</v>
       </c>
       <c r="I454" t="str">
+        <v>Approved</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>B43-KENNELSKETCH-06</v>
+      </c>
+      <c r="B455" t="str">
+        <v>B43</v>
+      </c>
+      <c r="C455" t="str">
+        <v>kennelsketch</v>
+      </c>
+      <c r="E455" t="str">
+        <v>thats all of them. you are good at this</v>
+      </c>
+      <c r="F455" t="str">
+        <v>Game copy</v>
+      </c>
+      <c r="I455" t="str">
         <v>Approved</v>
       </c>
     </row>

</xml_diff>